<commit_message>
Add image, JSON, QR and text tools, tool page content, browser tests (T3.3-T3.7)
Image compressor, resizer and converter; JSON formatter; QR generator; word
counter. Help, examples, FAQ and related tools per tool from tool_settings
(schema 1.0.1 with migration). Performance, privacy and cross-browser tests.
All 10 tools published.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="320">
   <si>
     <t>setting_key</t>
   </si>
@@ -43,7 +43,7 @@
     <t>schema_version</t>
   </si>
   <si>
-    <t>1.0.0</t>
+    <t>1.0.1</t>
   </si>
   <si>
     <t>string</t>
@@ -437,7 +437,7 @@
     <t>max_file_size_mb</t>
   </si>
   <si>
-    <t>20</t>
+    <t>25</t>
   </si>
   <si>
     <t>int</t>
@@ -468,6 +468,303 @@
   </si>
   <si>
     <t>18</t>
+  </si>
+  <si>
+    <t>TSET0005</t>
+  </si>
+  <si>
+    <t>help</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Follow these steps:
+- Choose a JPG, PNG or WebP image.
+- Pick the output format. JPG and WebP make the smallest files.
+- Move the quality slider. Lower quality means a smaller file.
+- Check the preview and the size saved, then download the result.</t>
+  </si>
+  <si>
+    <t>TSET0006</t>
+  </si>
+  <si>
+    <t>examples</t>
+  </si>
+  <si>
+    <t>[{"title":"Photo for a website","text":"A 4 MB phone photo saved as WebP at 75% quality is often under 500 KB and looks the same on screen."},{"title":"Email attachment","text":"Choose JPG at 60% quality to bring a scanned page well under typical email size limits."}]</t>
+  </si>
+  <si>
+    <t>json</t>
+  </si>
+  <si>
+    <t>TSET0007</t>
+  </si>
+  <si>
+    <t>faq</t>
+  </si>
+  <si>
+    <t>[{"q":"Is my image uploaded anywhere?","a":"No. The image is processed in your browser on your own device and is never sent to a server."},{"q":"Why is my PNG not getting smaller?","a":"PNG is lossless, so the quality slider has no effect on it. Choose JPG or WebP as the output format for a much smaller file."},{"q":"What is the largest image I can use?","a":"Files up to 25 MB and about 50 megapixels. Very large photos can be slow on older phones."}]</t>
+  </si>
+  <si>
+    <t>TSET0008</t>
+  </si>
+  <si>
+    <t>related</t>
+  </si>
+  <si>
+    <t>["TOOL0002","TOOL0003"]</t>
+  </si>
+  <si>
+    <t>TSET0009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Follow these steps:
+- Choose a JPG, PNG or WebP image. Its current size is filled in for you.
+- Either type a new width or height in pixels, or switch to a percentage of the original.
+- Leave **Keep the original proportions** ticked so the picture is not stretched.
+- Download the resized image.</t>
+  </si>
+  <si>
+    <t>TSET0010</t>
+  </si>
+  <si>
+    <t>[{"title":"Profile picture","text":"Set the width to 400 with proportions kept. A 2000 × 1500 photo becomes 400 × 300."},{"title":"Half size","text":"Switch to percentage and enter 50 to halve both width and height."}]</t>
+  </si>
+  <si>
+    <t>TSET0011</t>
+  </si>
+  <si>
+    <t>[{"q":"Does resizing reduce quality?","a":"Making an image smaller keeps it sharp. Making it larger cannot add detail, so enlarged images look soft."},{"q":"Which format is the result?","a":"The same format as the image you chose. Use the image converter to change format."},{"q":"Is my image uploaded anywhere?","a":"No. Everything happens in your browser on your own device."}]</t>
+  </si>
+  <si>
+    <t>TSET0012</t>
+  </si>
+  <si>
+    <t>["TOOL0001","TOOL0003"]</t>
+  </si>
+  <si>
+    <t>TSET0013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Follow these steps:
+- Choose a JPG, PNG or WebP image.
+- Pick the format to convert to.
+- For JPG and WebP, set the quality. Higher quality means a larger file.
+- Download the converted image.</t>
+  </si>
+  <si>
+    <t>TSET0014</t>
+  </si>
+  <si>
+    <t>[{"title":"PNG to JPG","text":"Convert a PNG screenshot to JPG for a smaller file. Transparent areas turn white."},{"title":"JPG to WebP","text":"Convert a JPG to WebP at 90% quality for a smaller file with similar looks."}]</t>
+  </si>
+  <si>
+    <t>TSET0015</t>
+  </si>
+  <si>
+    <t>[{"q":"What happens to transparency?","a":"PNG and WebP keep transparent areas. JPG cannot, so transparent areas become white."},{"q":"Can it convert GIF, HEIC or other types?","a":"Not yet. Only JPG, PNG and WebP are supported."},{"q":"Is my image uploaded anywhere?","a":"No. Everything happens in your browser on your own device."}]</t>
+  </si>
+  <si>
+    <t>TSET0016</t>
+  </si>
+  <si>
+    <t>["TOOL0001","TOOL0002"]</t>
+  </si>
+  <si>
+    <t>TSET0017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Follow these steps:
+- Enter the loan amount, the yearly interest rate and the tenure.
+- Choose whether the tenure is in years or months.
+- The monthly EMI, total interest and total payment update as you type.
+## How it is calculated
+EMI = P × r × (1 + r)^n ÷ ((1 + r)^n − 1), where P is the loan amount, r is the monthly rate (yearly rate ÷ 12 ÷ 100) and n is the number of months.</t>
+  </si>
+  <si>
+    <t>TSET0018</t>
+  </si>
+  <si>
+    <t>[{"title":"Home loan","text":"₹50,00,000 at 8.5% for 20 years gives a monthly EMI of about ₹43,391."},{"title":"Car loan","text":"₹8,00,000 at 9% for 5 years gives a monthly EMI of about ₹16,607."}]</t>
+  </si>
+  <si>
+    <t>TSET0019</t>
+  </si>
+  <si>
+    <t>[{"q":"Does this match my bank's figure?","a":"It uses the standard reducing-balance formula. Banks may differ slightly because of rounding, processing fees or the day the first instalment falls."},{"q":"Does it include processing fees or insurance?","a":"No. It only calculates principal and interest."},{"q":"Is the information I type saved?","a":"No. The calculation runs in your browser and nothing is sent or stored."}]</t>
+  </si>
+  <si>
+    <t>TSET0020</t>
+  </si>
+  <si>
+    <t>["TOOL0005","TOOL0007"]</t>
+  </si>
+  <si>
+    <t>TSET0021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Follow these steps:
+- Enter the deposit amount, the yearly interest rate and the tenure.
+- Choose how often the interest is compounded. Most banks compound fixed deposits quarterly.
+- See the maturity amount and the interest earned.
+## How it is calculated
+Maturity = P × (1 + r ÷ n)^(n × t), where P is the deposit, r the yearly rate, n the compounding periods per year and t the years. With simple interest, maturity = P × (1 + r × t).</t>
+  </si>
+  <si>
+    <t>TSET0022</t>
+  </si>
+  <si>
+    <t>[{"title":"Three-year deposit","text":"₹1,00,000 at 7% compounded quarterly for 3 years matures to about ₹1,23,144."},{"title":"Simple interest","text":"₹1,00,000 at 7% simple interest for 2 years earns ₹14,000."}]</t>
+  </si>
+  <si>
+    <t>TSET0023</t>
+  </si>
+  <si>
+    <t>[{"q":"Is the interest taxable?","a":"Interest on fixed deposits is usually taxable. This calculator does not include tax or TDS."},{"q":"Why is my bank's maturity amount a little different?","a":"Banks round each period and may count days exactly. Use this as a close estimate."},{"q":"Is the information I type saved?","a":"No. The calculation runs in your browser and nothing is sent or stored."}]</t>
+  </si>
+  <si>
+    <t>TSET0024</t>
+  </si>
+  <si>
+    <t>["TOOL0004","TOOL0007"]</t>
+  </si>
+  <si>
+    <t>TSET0025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Follow these steps:
+- Choose whether to add GST to an amount or remove it from an amount that already includes GST.
+- Enter the amount and the GST rate. Common rates are 0, 5, 12, 18 and 28.
+- See the amount without GST, the GST, and the CGST and SGST halves.</t>
+  </si>
+  <si>
+    <t>TSET0026</t>
+  </si>
+  <si>
+    <t>[{"title":"Add GST","text":"₹1,000 plus 18% GST gives ₹180 of GST and a total of ₹1,180."},{"title":"Remove GST","text":"A bill of ₹1,180 that includes 18% GST is ₹1,000 before tax, with ₹180 of GST."}]</t>
+  </si>
+  <si>
+    <t>TSET0027</t>
+  </si>
+  <si>
+    <t>[{"q":"What are CGST and SGST?","a":"For a sale within one state, GST is split equally between the central (CGST) and state (SGST) governments. For a sale between states, the whole amount is IGST."},{"q":"Does it check the correct rate for my goods?","a":"No. Enter the rate that applies to your goods or services. Check the official GST rate schedule if you are unsure."},{"q":"Is the information I type saved?","a":"No. The calculation runs in your browser and nothing is sent or stored."}]</t>
+  </si>
+  <si>
+    <t>TSET0028</t>
+  </si>
+  <si>
+    <t>["TOOL0007","TOOL0004"]</t>
+  </si>
+  <si>
+    <t>TSET0029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pick the kind of calculation, then enter two numbers:
+- **X% of Y**: for example, 20% of 150.
+- **X is what % of Y**: for example, 25 out of 200.
+- **% change from X to Y**: how much a value went up or down.
+- **Increase or decrease X by Y%**: for example, a price rise of 10%.</t>
+  </si>
+  <si>
+    <t>TSET0030</t>
+  </si>
+  <si>
+    <t>[{"title":"Discount","text":"Decrease 2,000 by 25% to get 1,500."},{"title":"Marks","text":"42 out of 60 is 70%."},{"title":"Price change","text":"From 80 to 100 is a 25% increase."}]</t>
+  </si>
+  <si>
+    <t>TSET0031</t>
+  </si>
+  <si>
+    <t>[{"q":"Why can't the old value be 0 for a % change?","a":"A change from zero cannot be shown as a percentage because dividing by zero is undefined."},{"q":"Can I use decimals and negative numbers?","a":"Yes for most modes. Commas in numbers such as 1,00,000 are fine."},{"q":"Is the information I type saved?","a":"No. The calculation runs in your browser and nothing is sent or stored."}]</t>
+  </si>
+  <si>
+    <t>TSET0032</t>
+  </si>
+  <si>
+    <t>["TOOL0006","TOOL0004"]</t>
+  </si>
+  <si>
+    <t>TSET0033</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Follow these steps:
+- Paste your JSON on the left. It is checked as you type.
+- Choose **Format** to make it easy to read, or **Minify** to make it as small as possible.
+- Pick the indentation and, if you like, sort the keys A to Z.
+- Copy the result.
+If the JSON is invalid, the message says what is wrong and, where your browser gives it, the line and column.</t>
+  </si>
+  <si>
+    <t>TSET0034</t>
+  </si>
+  <si>
+    <t>[{"title":"Tidy a response","text":"Paste {\"name\":\"OEWER\",\"tools\":[1,2]} and choose Format to see it spread over several indented lines."},{"title":"Find a mistake","text":"A trailing comma such as {\"a\": 1,} is not valid JSON. The error message points to where it goes wrong."}]</t>
+  </si>
+  <si>
+    <t>TSET0035</t>
+  </si>
+  <si>
+    <t>[{"q":"Is my JSON sent to a server?","a":"No. It is checked and formatted in your browser and never leaves your device."},{"q":"Why is my JSON invalid when it works in my code?","a":"JSON is stricter than JavaScript: keys need double quotes, single quotes are not allowed, and trailing commas and comments are not allowed."},{"q":"How large can the input be?","a":"Up to 5 million characters."}]</t>
+  </si>
+  <si>
+    <t>TSET0036</t>
+  </si>
+  <si>
+    <t>["TOOL0010","TOOL0009"]</t>
+  </si>
+  <si>
+    <t>TSET0037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Follow these steps:
+- Type or paste a link or any text.
+- Choose the error correction. Medium suits most uses; High lets the code still scan if part of it is damaged.
+- Pick the image size and colour.
+- Download the code as a PNG or SVG.
+Always test the code with a phone before you print it.</t>
+  </si>
+  <si>
+    <t>TSET0038</t>
+  </si>
+  <si>
+    <t>[{"title":"Website link","text":"Enter https://example.com to make a code that opens the site when scanned."},{"title":"Wi-Fi details","text":"Enter WIFI:T:WPA;S:MyNetwork;P:mypassword;; and phones can join the network by scanning."}]</t>
+  </si>
+  <si>
+    <t>TSET0039</t>
+  </si>
+  <si>
+    <t>[{"q":"Do the codes expire?","a":"No. The text is stored in the code itself, so it works as long as it is readable."},{"q":"Is my text sent to a server?","a":"No. The code is generated in your browser and your text never leaves your device."},{"q":"PNG or SVG?","a":"Use PNG for screens and documents. Use SVG when you need it to stay sharp at any size, for example for print."}]</t>
+  </si>
+  <si>
+    <t>TSET0040</t>
+  </si>
+  <si>
+    <t>["TOOL0010","TOOL0008"]</t>
+  </si>
+  <si>
+    <t>TSET0041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Follow these steps:
+- Type or paste your text.
+- The counts update as you type: words, characters, sentences, paragraphs and lines.
+- Reading and speaking time are estimates based on average speeds.</t>
+  </si>
+  <si>
+    <t>TSET0042</t>
+  </si>
+  <si>
+    <t>[{"title":"Essay limit","text":"Paste your essay to check it is within a 500-word limit."},{"title":"Social post","text":"Check a post stays under a character limit, counting spaces."}]</t>
+  </si>
+  <si>
+    <t>TSET0043</t>
+  </si>
+  <si>
+    <t>[{"q":"How are words counted?","a":"A word is a run of letters or numbers separated by spaces or punctuation. Hyphenated words and numbers each count as words."},{"q":"How are reading and speaking time worked out?","a":"Reading time assumes 200 words a minute and speaking time 130 words a minute."},{"q":"Is my text sent to a server?","a":"No. The count happens in your browser and your text never leaves your device."}]</t>
+  </si>
+  <si>
+    <t>TSET0044</t>
+  </si>
+  <si>
+    <t>["TOOL0008","TOOL0009"]</t>
   </si>
   <si>
     <t>BCAT0001</t>
@@ -734,9 +1031,6 @@
   </si>
   <si>
     <t>rows_per_page</t>
-  </si>
-  <si>
-    <t>25</t>
   </si>
 </sst>
 </file>
@@ -1276,122 +1570,122 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>170</v>
+        <v>255</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>163</v>
+        <v>248</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>171</v>
+        <v>256</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>26</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>172</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>173</v>
+        <v>258</v>
       </c>
       <c r="B2" t="s">
-        <v>166</v>
+        <v>251</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>174</v>
+        <v>259</v>
       </c>
       <c r="E2" t="s">
-        <v>175</v>
+        <v>260</v>
       </c>
       <c r="F2" t="s">
-        <v>162</v>
+        <v>247</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>176</v>
+        <v>261</v>
       </c>
       <c r="B3" t="s">
-        <v>166</v>
+        <v>251</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>177</v>
+        <v>262</v>
       </c>
       <c r="E3" t="s">
-        <v>178</v>
+        <v>263</v>
       </c>
       <c r="F3" t="s">
-        <v>162</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>179</v>
+        <v>264</v>
       </c>
       <c r="B4" t="s">
-        <v>166</v>
+        <v>251</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>174</v>
+        <v>259</v>
       </c>
       <c r="E4" t="s">
-        <v>180</v>
+        <v>265</v>
       </c>
       <c r="F4" t="s">
-        <v>162</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>181</v>
+        <v>266</v>
       </c>
       <c r="B5" t="s">
-        <v>166</v>
+        <v>251</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>177</v>
+        <v>262</v>
       </c>
       <c r="E5" t="s">
-        <v>182</v>
+        <v>267</v>
       </c>
       <c r="F5" t="s">
-        <v>162</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>183</v>
+        <v>268</v>
       </c>
       <c r="B6" t="s">
-        <v>166</v>
+        <v>251</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>184</v>
+        <v>269</v>
       </c>
       <c r="E6" t="s">
-        <v>185</v>
+        <v>270</v>
       </c>
       <c r="F6" t="s">
-        <v>162</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -1411,7 +1705,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>186</v>
+        <v>271</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>72</v>
@@ -1422,24 +1716,24 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>187</v>
+        <v>272</v>
       </c>
       <c r="B2" t="s">
-        <v>188</v>
+        <v>273</v>
       </c>
       <c r="C2" t="s">
-        <v>189</v>
+        <v>274</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>190</v>
+        <v>275</v>
       </c>
       <c r="B3" t="s">
-        <v>191</v>
+        <v>276</v>
       </c>
       <c r="C3" t="s">
-        <v>192</v>
+        <v>277</v>
       </c>
     </row>
   </sheetData>
@@ -1459,35 +1753,35 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>193</v>
+        <v>278</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>163</v>
+        <v>248</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>186</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>194</v>
+        <v>279</v>
       </c>
       <c r="B2" t="s">
-        <v>166</v>
+        <v>251</v>
       </c>
       <c r="C2" t="s">
-        <v>187</v>
+        <v>272</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>195</v>
+        <v>280</v>
       </c>
       <c r="B3" t="s">
-        <v>166</v>
+        <v>251</v>
       </c>
       <c r="C3" t="s">
-        <v>190</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -1512,45 +1806,45 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>196</v>
+        <v>281</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>197</v>
+        <v>282</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>198</v>
+        <v>283</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>199</v>
+        <v>284</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>200</v>
+        <v>285</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>201</v>
+        <v>286</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>202</v>
+        <v>287</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>203</v>
+        <v>288</v>
       </c>
       <c r="B2" t="s">
-        <v>204</v>
+        <v>289</v>
       </c>
       <c r="C2" t="s">
         <v>105</v>
       </c>
       <c r="D2" t="s">
-        <v>205</v>
+        <v>290</v>
       </c>
       <c r="E2" t="s">
-        <v>206</v>
+        <v>291</v>
       </c>
       <c r="F2" t="s">
-        <v>162</v>
+        <v>247</v>
       </c>
       <c r="G2" t="b">
         <v>0</v>
@@ -1558,22 +1852,22 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>207</v>
+        <v>292</v>
       </c>
       <c r="B3" t="s">
-        <v>208</v>
+        <v>293</v>
       </c>
       <c r="C3" t="s">
-        <v>166</v>
+        <v>251</v>
       </c>
       <c r="D3" t="s">
-        <v>209</v>
+        <v>294</v>
       </c>
       <c r="E3" t="s">
-        <v>210</v>
+        <v>295</v>
       </c>
       <c r="F3" t="s">
-        <v>162</v>
+        <v>247</v>
       </c>
       <c r="G3" t="b">
         <v>0</v>
@@ -1581,10 +1875,10 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>211</v>
+        <v>296</v>
       </c>
       <c r="B4" t="s">
-        <v>212</v>
+        <v>297</v>
       </c>
       <c r="C4" t="s">
         <v>28</v>
@@ -1593,10 +1887,10 @@
         <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>213</v>
+        <v>298</v>
       </c>
       <c r="F4" t="s">
-        <v>162</v>
+        <v>247</v>
       </c>
       <c r="G4" t="b">
         <v>0</v>
@@ -1620,70 +1914,70 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>214</v>
+        <v>299</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>215</v>
+        <v>300</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>216</v>
+        <v>301</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>217</v>
+        <v>302</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>218</v>
+        <v>303</v>
       </c>
       <c r="B2" t="s">
-        <v>219</v>
+        <v>304</v>
       </c>
       <c r="C2" t="s">
-        <v>220</v>
+        <v>305</v>
       </c>
       <c r="D2" t="b">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>162</v>
+        <v>247</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>221</v>
+        <v>306</v>
       </c>
       <c r="B3" t="s">
-        <v>222</v>
+        <v>307</v>
       </c>
       <c r="C3" t="s">
-        <v>204</v>
+        <v>289</v>
       </c>
       <c r="D3" t="b">
         <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>162</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>223</v>
+        <v>308</v>
       </c>
       <c r="B4" t="s">
-        <v>224</v>
+        <v>309</v>
       </c>
       <c r="C4" t="s">
-        <v>225</v>
+        <v>310</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>162</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -1706,16 +2000,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>226</v>
+        <v>311</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>227</v>
+        <v>312</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>228</v>
+        <v>313</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>229</v>
+        <v>314</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>51</v>
@@ -1723,16 +2017,16 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>230</v>
+        <v>315</v>
       </c>
       <c r="B2" t="s">
-        <v>231</v>
+        <v>316</v>
       </c>
       <c r="C2" t="s">
-        <v>232</v>
+        <v>317</v>
       </c>
       <c r="D2" t="s">
-        <v>233</v>
+        <v>318</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -1766,10 +2060,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>234</v>
+        <v>319</v>
       </c>
       <c r="B2" t="s">
-        <v>235</v>
+        <v>136</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -2238,7 +2532,7 @@
         <v>95</v>
       </c>
       <c r="G2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -2267,7 +2561,7 @@
         <v>99</v>
       </c>
       <c r="G3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H3" t="b">
         <v>0</v>
@@ -2296,7 +2590,7 @@
         <v>103</v>
       </c>
       <c r="G4" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
@@ -2325,7 +2619,7 @@
         <v>107</v>
       </c>
       <c r="G5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -2354,7 +2648,7 @@
         <v>111</v>
       </c>
       <c r="G6" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -2383,7 +2677,7 @@
         <v>115</v>
       </c>
       <c r="G7" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
@@ -2412,7 +2706,7 @@
         <v>119</v>
       </c>
       <c r="G8" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
@@ -2441,7 +2735,7 @@
         <v>123</v>
       </c>
       <c r="G9" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H9" t="b">
         <v>1</v>
@@ -2470,7 +2764,7 @@
         <v>127</v>
       </c>
       <c r="G10" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -2499,7 +2793,7 @@
         <v>131</v>
       </c>
       <c r="G11" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H11" t="b">
         <v>0</v>
@@ -2516,12 +2810,12 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="4" max="4" width="60" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2608,6 +2902,686 @@
       </c>
       <c r="E5" t="s">
         <v>137</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>147</v>
+      </c>
+      <c r="B6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D6" t="s">
+        <v>149</v>
+      </c>
+      <c r="E6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>150</v>
+      </c>
+      <c r="B7" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7" t="s">
+        <v>151</v>
+      </c>
+      <c r="D7" t="s">
+        <v>152</v>
+      </c>
+      <c r="E7" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>154</v>
+      </c>
+      <c r="B8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C8" t="s">
+        <v>155</v>
+      </c>
+      <c r="D8" t="s">
+        <v>156</v>
+      </c>
+      <c r="E8" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>157</v>
+      </c>
+      <c r="B9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C9" t="s">
+        <v>158</v>
+      </c>
+      <c r="D9" t="s">
+        <v>159</v>
+      </c>
+      <c r="E9" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>160</v>
+      </c>
+      <c r="B10" t="s">
+        <v>97</v>
+      </c>
+      <c r="C10" t="s">
+        <v>148</v>
+      </c>
+      <c r="D10" t="s">
+        <v>161</v>
+      </c>
+      <c r="E10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>162</v>
+      </c>
+      <c r="B11" t="s">
+        <v>97</v>
+      </c>
+      <c r="C11" t="s">
+        <v>151</v>
+      </c>
+      <c r="D11" t="s">
+        <v>163</v>
+      </c>
+      <c r="E11" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>164</v>
+      </c>
+      <c r="B12" t="s">
+        <v>97</v>
+      </c>
+      <c r="C12" t="s">
+        <v>155</v>
+      </c>
+      <c r="D12" t="s">
+        <v>165</v>
+      </c>
+      <c r="E12" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>166</v>
+      </c>
+      <c r="B13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C13" t="s">
+        <v>158</v>
+      </c>
+      <c r="D13" t="s">
+        <v>167</v>
+      </c>
+      <c r="E13" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>168</v>
+      </c>
+      <c r="B14" t="s">
+        <v>101</v>
+      </c>
+      <c r="C14" t="s">
+        <v>148</v>
+      </c>
+      <c r="D14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>170</v>
+      </c>
+      <c r="B15" t="s">
+        <v>101</v>
+      </c>
+      <c r="C15" t="s">
+        <v>151</v>
+      </c>
+      <c r="D15" t="s">
+        <v>171</v>
+      </c>
+      <c r="E15" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>172</v>
+      </c>
+      <c r="B16" t="s">
+        <v>101</v>
+      </c>
+      <c r="C16" t="s">
+        <v>155</v>
+      </c>
+      <c r="D16" t="s">
+        <v>173</v>
+      </c>
+      <c r="E16" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>174</v>
+      </c>
+      <c r="B17" t="s">
+        <v>101</v>
+      </c>
+      <c r="C17" t="s">
+        <v>158</v>
+      </c>
+      <c r="D17" t="s">
+        <v>175</v>
+      </c>
+      <c r="E17" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>176</v>
+      </c>
+      <c r="B18" t="s">
+        <v>105</v>
+      </c>
+      <c r="C18" t="s">
+        <v>148</v>
+      </c>
+      <c r="D18" t="s">
+        <v>177</v>
+      </c>
+      <c r="E18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>178</v>
+      </c>
+      <c r="B19" t="s">
+        <v>105</v>
+      </c>
+      <c r="C19" t="s">
+        <v>151</v>
+      </c>
+      <c r="D19" t="s">
+        <v>179</v>
+      </c>
+      <c r="E19" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>180</v>
+      </c>
+      <c r="B20" t="s">
+        <v>105</v>
+      </c>
+      <c r="C20" t="s">
+        <v>155</v>
+      </c>
+      <c r="D20" t="s">
+        <v>181</v>
+      </c>
+      <c r="E20" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>182</v>
+      </c>
+      <c r="B21" t="s">
+        <v>105</v>
+      </c>
+      <c r="C21" t="s">
+        <v>158</v>
+      </c>
+      <c r="D21" t="s">
+        <v>183</v>
+      </c>
+      <c r="E21" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>184</v>
+      </c>
+      <c r="B22" t="s">
+        <v>109</v>
+      </c>
+      <c r="C22" t="s">
+        <v>148</v>
+      </c>
+      <c r="D22" t="s">
+        <v>185</v>
+      </c>
+      <c r="E22" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>186</v>
+      </c>
+      <c r="B23" t="s">
+        <v>109</v>
+      </c>
+      <c r="C23" t="s">
+        <v>151</v>
+      </c>
+      <c r="D23" t="s">
+        <v>187</v>
+      </c>
+      <c r="E23" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>188</v>
+      </c>
+      <c r="B24" t="s">
+        <v>109</v>
+      </c>
+      <c r="C24" t="s">
+        <v>155</v>
+      </c>
+      <c r="D24" t="s">
+        <v>189</v>
+      </c>
+      <c r="E24" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>190</v>
+      </c>
+      <c r="B25" t="s">
+        <v>109</v>
+      </c>
+      <c r="C25" t="s">
+        <v>158</v>
+      </c>
+      <c r="D25" t="s">
+        <v>191</v>
+      </c>
+      <c r="E25" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>192</v>
+      </c>
+      <c r="B26" t="s">
+        <v>113</v>
+      </c>
+      <c r="C26" t="s">
+        <v>148</v>
+      </c>
+      <c r="D26" t="s">
+        <v>193</v>
+      </c>
+      <c r="E26" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>194</v>
+      </c>
+      <c r="B27" t="s">
+        <v>113</v>
+      </c>
+      <c r="C27" t="s">
+        <v>151</v>
+      </c>
+      <c r="D27" t="s">
+        <v>195</v>
+      </c>
+      <c r="E27" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>196</v>
+      </c>
+      <c r="B28" t="s">
+        <v>113</v>
+      </c>
+      <c r="C28" t="s">
+        <v>155</v>
+      </c>
+      <c r="D28" t="s">
+        <v>197</v>
+      </c>
+      <c r="E28" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>198</v>
+      </c>
+      <c r="B29" t="s">
+        <v>113</v>
+      </c>
+      <c r="C29" t="s">
+        <v>158</v>
+      </c>
+      <c r="D29" t="s">
+        <v>199</v>
+      </c>
+      <c r="E29" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>200</v>
+      </c>
+      <c r="B30" t="s">
+        <v>117</v>
+      </c>
+      <c r="C30" t="s">
+        <v>148</v>
+      </c>
+      <c r="D30" t="s">
+        <v>201</v>
+      </c>
+      <c r="E30" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>202</v>
+      </c>
+      <c r="B31" t="s">
+        <v>117</v>
+      </c>
+      <c r="C31" t="s">
+        <v>151</v>
+      </c>
+      <c r="D31" t="s">
+        <v>203</v>
+      </c>
+      <c r="E31" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>204</v>
+      </c>
+      <c r="B32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C32" t="s">
+        <v>155</v>
+      </c>
+      <c r="D32" t="s">
+        <v>205</v>
+      </c>
+      <c r="E32" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>206</v>
+      </c>
+      <c r="B33" t="s">
+        <v>117</v>
+      </c>
+      <c r="C33" t="s">
+        <v>158</v>
+      </c>
+      <c r="D33" t="s">
+        <v>207</v>
+      </c>
+      <c r="E33" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>208</v>
+      </c>
+      <c r="B34" t="s">
+        <v>121</v>
+      </c>
+      <c r="C34" t="s">
+        <v>148</v>
+      </c>
+      <c r="D34" t="s">
+        <v>209</v>
+      </c>
+      <c r="E34" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>210</v>
+      </c>
+      <c r="B35" t="s">
+        <v>121</v>
+      </c>
+      <c r="C35" t="s">
+        <v>151</v>
+      </c>
+      <c r="D35" t="s">
+        <v>211</v>
+      </c>
+      <c r="E35" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>212</v>
+      </c>
+      <c r="B36" t="s">
+        <v>121</v>
+      </c>
+      <c r="C36" t="s">
+        <v>155</v>
+      </c>
+      <c r="D36" t="s">
+        <v>213</v>
+      </c>
+      <c r="E36" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>214</v>
+      </c>
+      <c r="B37" t="s">
+        <v>121</v>
+      </c>
+      <c r="C37" t="s">
+        <v>158</v>
+      </c>
+      <c r="D37" t="s">
+        <v>215</v>
+      </c>
+      <c r="E37" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>216</v>
+      </c>
+      <c r="B38" t="s">
+        <v>125</v>
+      </c>
+      <c r="C38" t="s">
+        <v>148</v>
+      </c>
+      <c r="D38" t="s">
+        <v>217</v>
+      </c>
+      <c r="E38" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>218</v>
+      </c>
+      <c r="B39" t="s">
+        <v>125</v>
+      </c>
+      <c r="C39" t="s">
+        <v>151</v>
+      </c>
+      <c r="D39" t="s">
+        <v>219</v>
+      </c>
+      <c r="E39" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>220</v>
+      </c>
+      <c r="B40" t="s">
+        <v>125</v>
+      </c>
+      <c r="C40" t="s">
+        <v>155</v>
+      </c>
+      <c r="D40" t="s">
+        <v>221</v>
+      </c>
+      <c r="E40" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>222</v>
+      </c>
+      <c r="B41" t="s">
+        <v>125</v>
+      </c>
+      <c r="C41" t="s">
+        <v>158</v>
+      </c>
+      <c r="D41" t="s">
+        <v>223</v>
+      </c>
+      <c r="E41" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>224</v>
+      </c>
+      <c r="B42" t="s">
+        <v>129</v>
+      </c>
+      <c r="C42" t="s">
+        <v>148</v>
+      </c>
+      <c r="D42" t="s">
+        <v>225</v>
+      </c>
+      <c r="E42" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>226</v>
+      </c>
+      <c r="B43" t="s">
+        <v>129</v>
+      </c>
+      <c r="C43" t="s">
+        <v>151</v>
+      </c>
+      <c r="D43" t="s">
+        <v>227</v>
+      </c>
+      <c r="E43" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>228</v>
+      </c>
+      <c r="B44" t="s">
+        <v>129</v>
+      </c>
+      <c r="C44" t="s">
+        <v>155</v>
+      </c>
+      <c r="D44" t="s">
+        <v>229</v>
+      </c>
+      <c r="E44" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>230</v>
+      </c>
+      <c r="B45" t="s">
+        <v>129</v>
+      </c>
+      <c r="C45" t="s">
+        <v>158</v>
+      </c>
+      <c r="D45" t="s">
+        <v>231</v>
+      </c>
+      <c r="E45" t="s">
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -2642,30 +3616,30 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>147</v>
+        <v>232</v>
       </c>
       <c r="B2" t="s">
-        <v>148</v>
+        <v>233</v>
       </c>
       <c r="C2" t="s">
-        <v>149</v>
+        <v>234</v>
       </c>
       <c r="D2" t="s">
-        <v>150</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>151</v>
+        <v>236</v>
       </c>
       <c r="B3" t="s">
-        <v>152</v>
+        <v>237</v>
       </c>
       <c r="C3" t="s">
-        <v>153</v>
+        <v>238</v>
       </c>
       <c r="D3" t="s">
-        <v>154</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -2687,30 +3661,30 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>155</v>
+        <v>240</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>156</v>
+        <v>241</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>157</v>
+        <v>242</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>158</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>159</v>
+        <v>244</v>
       </c>
       <c r="B2" t="s">
-        <v>160</v>
+        <v>245</v>
       </c>
       <c r="C2" t="s">
-        <v>161</v>
+        <v>246</v>
       </c>
       <c r="D2" t="s">
-        <v>162</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -2734,7 +3708,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>163</v>
+        <v>248</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>25</v>
@@ -2743,19 +3717,19 @@
         <v>24</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>164</v>
+        <v>249</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>155</v>
+        <v>240</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>27</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>165</v>
+        <v>250</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>3</v>
@@ -2763,22 +3737,22 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>166</v>
+        <v>251</v>
       </c>
       <c r="B2" t="s">
-        <v>167</v>
+        <v>252</v>
       </c>
       <c r="C2" t="s">
-        <v>168</v>
+        <v>253</v>
       </c>
       <c r="D2" t="s">
-        <v>169</v>
+        <v>254</v>
       </c>
       <c r="E2" t="s">
-        <v>147</v>
+        <v>232</v>
       </c>
       <c r="F2" t="s">
-        <v>159</v>
+        <v>244</v>
       </c>
       <c r="G2" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
Premium redesign, new home page and more content (T2.7)
New design system (Inter + Fraunces, icons, gold accent), redesigned home,
tool, blog and static pages, five new articles, richer About and Contact.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="957" uniqueCount="489">
   <si>
     <t>setting_key</t>
   </si>
@@ -121,8 +121,17 @@
     <t>About OEWER Tools</t>
   </si>
   <si>
-    <t xml:space="preserve">OEWER Tools is a collection of free, fast online tools. Most tools run entirely in your browser, so your files and numbers stay on your device.
-We publish practical guides alongside each tool so you understand how the results are calculated.</t>
+    <t xml:space="preserve">OEWER Tools is a collection of free, fast online tools for everyday jobs: shrinking an image, working out a loan EMI, tidying JSON or making a QR code.
+We built it because too many online tools ask you to upload your files, sign up for an account or sit through pop-ups just to do something simple. Ours do not.
+# What makes us different
+- **Private by design.** Our tools run in your browser. Your images, text and numbers stay on your device and are never uploaded to our servers.
+- **No sign-up.** Open a tool and use it.
+- **Explained, not just answered.** Each tool comes with how-to steps, worked examples and answers to common questions, and our guides explain the formulas behind the results.
+- **Made for every device.** The site works on phones, tablets and computers, and with a keyboard or a screen reader.
+# How we keep our word
+We test the privacy promise. Our automated tests watch the network while each tool is used and fail if anything is sent anywhere. The calculators use standard published formulas, and we check their results against worked examples.
+# What is next
+We are adding more tools and more guides. If there is a tool you wish existed, tell us on the contact page.</t>
   </si>
   <si>
     <t>published</t>
@@ -164,7 +173,15 @@
     <t>Contact Us</t>
   </si>
   <si>
-    <t>Questions or feedback? Email us at hello@example.com.</t>
+    <t xml:space="preserve">Questions, bug reports or ideas for a new tool? We would like to hear from you.
+Email us at hello@example.com.
+# Helpful details to include
+- The name of the tool and what you were trying to do.
+- What you expected to happen, and what happened instead.
+- Your browser and device, for example Chrome on Android.
+Please do not send passwords, bank details or files containing personal information. We do not need them to help.
+# Suggest a tool
+Tell us what you would use it for and how often. Tools that save people the most time go to the top of our list.</t>
   </si>
   <si>
     <t>nav_id</t>
@@ -836,6 +853,81 @@
     <t>Understand the formula behind your loan EMI and how interest and tenure change what you pay.</t>
   </si>
   <si>
+    <t>POST0002</t>
+  </si>
+  <si>
+    <t>How to Compress Images Without Losing Quality</t>
+  </si>
+  <si>
+    <t>compress-images-without-losing-quality</t>
+  </si>
+  <si>
+    <t>Big photos slow down websites and fill up inboxes. Learn which format and quality setting to choose so images get smaller without looking worse.</t>
+  </si>
+  <si>
+    <t>2026-10-12T09:00:00Z</t>
+  </si>
+  <si>
+    <t>POST0003</t>
+  </si>
+  <si>
+    <t>GST Explained: How to Add and Remove GST</t>
+  </si>
+  <si>
+    <t>gst-explained-add-and-remove-gst</t>
+  </si>
+  <si>
+    <t>Adding GST to a price is easy. Taking it back out of a total is where people slip. Here are both calculations with worked examples.</t>
+  </si>
+  <si>
+    <t>2026-10-16T09:00:00Z</t>
+  </si>
+  <si>
+    <t>POST0004</t>
+  </si>
+  <si>
+    <t>Fixed Deposit Interest: Simple vs Compound</t>
+  </si>
+  <si>
+    <t>fixed-deposit-interest-simple-vs-compound</t>
+  </si>
+  <si>
+    <t>Two fixed deposits at the same rate can pay different amounts. The difference is how often the interest is added back and earns interest itself.</t>
+  </si>
+  <si>
+    <t>2026-10-20T09:00:00Z</t>
+  </si>
+  <si>
+    <t>POST0005</t>
+  </si>
+  <si>
+    <t>How to Make a QR Code That Scans Every Time</t>
+  </si>
+  <si>
+    <t>make-a-qr-code-that-scans-every-time</t>
+  </si>
+  <si>
+    <t>A QR code that will not scan is worse than none at all. Follow these simple rules for size, colour and error correction.</t>
+  </si>
+  <si>
+    <t>2026-10-24T09:00:00Z</t>
+  </si>
+  <si>
+    <t>POST0006</t>
+  </si>
+  <si>
+    <t>Why Browser-Based Tools Keep Your Files Private</t>
+  </si>
+  <si>
+    <t>why-browser-based-tools-keep-your-files-private</t>
+  </si>
+  <si>
+    <t>Some online tools upload your files to a server to process them. Others do the work on your own device. Here is how to tell the difference and why it matters.</t>
+  </si>
+  <si>
+    <t>2026-10-28T09:00:00Z</t>
+  </si>
+  <si>
     <t>block_id</t>
   </si>
   <si>
@@ -886,6 +978,356 @@
 A longer tenure lowers the EMI but increases the total interest paid.</t>
   </si>
   <si>
+    <t>BLK00010</t>
+  </si>
+  <si>
+    <t>A photo straight from a phone is often 3 to 8 MB. That is far more than a web page, an email or a form upload needs. Compressing the image can cut its size by 70% or more, and when it is done well, you will not see the difference.</t>
+  </si>
+  <si>
+    <t>BLK00011</t>
+  </si>
+  <si>
+    <t>Lossy and lossless compression</t>
+  </si>
+  <si>
+    <t>BLK00012</t>
+  </si>
+  <si>
+    <t>**Lossless** compression (used by PNG) makes a file smaller without throwing any detail away. **Lossy** compression (used by JPG and WebP) discards detail your eyes are unlikely to notice. Lossy files are much smaller, which is why photos are almost always saved as JPG or WebP.</t>
+  </si>
+  <si>
+    <t>BLK00013</t>
+  </si>
+  <si>
+    <t>Pick the right format</t>
+  </si>
+  <si>
+    <t>BLK00014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">**JPG** is the safe choice for photographs. It works everywhere.
+**WebP** is usually 25% to 35% smaller than JPG at the same look. Almost all current browsers show it.
+**PNG** is best for screenshots, logos and anything with sharp edges or transparency. It does not shrink with a quality slider.</t>
+  </si>
+  <si>
+    <t>BLK00015</t>
+  </si>
+  <si>
+    <t>Choose a quality setting</t>
+  </si>
+  <si>
+    <t>BLK00016</t>
+  </si>
+  <si>
+    <t>Most photos look the same at 70% to 80% quality as at 100%, and the file is a fraction of the size. Start at 75%, check the preview, and only go lower if the picture still looks clean. If you see blocky patches or fuzzy edges around text, raise the quality a little.</t>
+  </si>
+  <si>
+    <t>BLK00017</t>
+  </si>
+  <si>
+    <t>callout</t>
+  </si>
+  <si>
+    <t>**Tip:** resize first, then compress. A photo shown at 800 pixels wide does not need to be 4,000 pixels wide. Shrinking the dimensions with the image resizer saves more than any quality setting.</t>
+  </si>
+  <si>
+    <t>BLK00018</t>
+  </si>
+  <si>
+    <t>Keep your photos private</t>
+  </si>
+  <si>
+    <t>BLK00019</t>
+  </si>
+  <si>
+    <t>Many online compressors upload your pictures to a server. Our image compressor works inside your browser, so the image never leaves your device. That matters for ID scans, receipts and family photos.</t>
+  </si>
+  <si>
+    <t>BLK00030</t>
+  </si>
+  <si>
+    <t>Goods and Services Tax (GST) is added to the price of most goods and services in India. Businesses often need to do two things: add GST to a price, and work backwards from a total that already includes it.</t>
+  </si>
+  <si>
+    <t>BLK00031</t>
+  </si>
+  <si>
+    <t>Adding GST</t>
+  </si>
+  <si>
+    <t>BLK00032</t>
+  </si>
+  <si>
+    <t>Multiply the price by the rate and add the result. The formula is **GST = price × rate ÷ 100**, and the total is **price + GST**.</t>
+  </si>
+  <si>
+    <t>BLK00033</t>
+  </si>
+  <si>
+    <t>For example, a service costs ₹10,000 before tax and the rate is 18%. GST is ₹1,800, so the customer pays ₹11,800.</t>
+  </si>
+  <si>
+    <t>BLK00034</t>
+  </si>
+  <si>
+    <t>Removing GST from a total</t>
+  </si>
+  <si>
+    <t>BLK00035</t>
+  </si>
+  <si>
+    <t>This is where mistakes happen. You cannot just take 18% off ₹11,800, because the 18% was worked out on the smaller, pre-tax price. Instead use **price before GST = total × 100 ÷ (100 + rate)**.</t>
+  </si>
+  <si>
+    <t>BLK00036</t>
+  </si>
+  <si>
+    <t>From ₹11,800 at 18%: 11,800 × 100 ÷ 118 = ₹10,000. The GST part is the difference, ₹1,800. Taking 18% off ₹11,800 would give ₹2,124, which is wrong.</t>
+  </si>
+  <si>
+    <t>BLK00037</t>
+  </si>
+  <si>
+    <t>CGST, SGST and IGST</t>
+  </si>
+  <si>
+    <t>BLK00038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For a sale within one state, GST is split equally between the central government (CGST) and the state government (SGST). At 18%, that is 9% each.
+For a sale between states, the whole amount is charged as IGST.</t>
+  </si>
+  <si>
+    <t>BLK00039</t>
+  </si>
+  <si>
+    <t>Common GST rates</t>
+  </si>
+  <si>
+    <t>BLK00040</t>
+  </si>
+  <si>
+    <t>GST is charged at 0%, 5%, 12%, 18% or 28% depending on the goods or services. Always check the official rate schedule for what you sell, because rates and classifications change.</t>
+  </si>
+  <si>
+    <t>BLK00041</t>
+  </si>
+  <si>
+    <t>Our GST calculator does both calculations and shows the CGST and SGST halves. It is a calculator, not tax advice. Confirm the rate that applies to you with an accountant or the official GST portal.</t>
+  </si>
+  <si>
+    <t>BLK00050</t>
+  </si>
+  <si>
+    <t>When you open a fixed deposit (FD), the bank pays interest on your money. How that interest is calculated decides how much you get at the end.</t>
+  </si>
+  <si>
+    <t>BLK00051</t>
+  </si>
+  <si>
+    <t>Simple interest</t>
+  </si>
+  <si>
+    <t>BLK00052</t>
+  </si>
+  <si>
+    <t>With simple interest, you earn interest only on the amount you put in. The formula is **maturity = principal × (1 + rate × years)**.</t>
+  </si>
+  <si>
+    <t>BLK00053</t>
+  </si>
+  <si>
+    <t>₹1,00,000 at 7% for 3 years earns ₹21,000 of interest, so you receive ₹1,21,000.</t>
+  </si>
+  <si>
+    <t>BLK00054</t>
+  </si>
+  <si>
+    <t>Compound interest</t>
+  </si>
+  <si>
+    <t>BLK00055</t>
+  </si>
+  <si>
+    <t>With compound interest, interest is added to the deposit at regular intervals, and then that interest earns interest too. The formula is **maturity = principal × (1 + rate ÷ n)^(n × years)**, where n is how many times a year interest is added.</t>
+  </si>
+  <si>
+    <t>BLK00056</t>
+  </si>
+  <si>
+    <t>The same ₹1,00,000 at 7% for 3 years, compounded quarterly, grows to about ₹1,23,144. That is ₹2,144 more than simple interest.</t>
+  </si>
+  <si>
+    <t>BLK00057</t>
+  </si>
+  <si>
+    <t>Does compounding frequency matter?</t>
+  </si>
+  <si>
+    <t>BLK00058</t>
+  </si>
+  <si>
+    <t>A little. For the same ₹1,00,000 at 7% over 3 years:</t>
+  </si>
+  <si>
+    <t>BLK00059</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yearly compounding gives about ₹1,22,504.
+Quarterly compounding gives about ₹1,23,144.
+Monthly compounding gives about ₹1,23,293.</t>
+  </si>
+  <si>
+    <t>BLK00060</t>
+  </si>
+  <si>
+    <t>The more often interest is added, the more you earn, but the gains get smaller each step. Most banks compound fixed deposits quarterly.</t>
+  </si>
+  <si>
+    <t>BLK00061</t>
+  </si>
+  <si>
+    <t>Interest on fixed deposits is usually taxable, and your bank may deduct tax at source. Our FD calculator does not include tax, so your actual take-home will be lower.</t>
+  </si>
+  <si>
+    <t>BLK00070</t>
+  </si>
+  <si>
+    <t>A QR code stores text, usually a web address, as a pattern of squares. Phone cameras read it in a fraction of a second, as long as the pattern is clear. Most scanning problems come from a few avoidable mistakes.</t>
+  </si>
+  <si>
+    <t>BLK00071</t>
+  </si>
+  <si>
+    <t>Keep the text short</t>
+  </si>
+  <si>
+    <t>BLK00072</t>
+  </si>
+  <si>
+    <t>The more you put in a code, the denser and harder to read it becomes. A short link makes a simpler code than a long one. If your address is long, use a shorter page address.</t>
+  </si>
+  <si>
+    <t>BLK00073</t>
+  </si>
+  <si>
+    <t>Use strong contrast</t>
+  </si>
+  <si>
+    <t>BLK00074</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dark squares on a light background scan best. Black on white is the safest.
+Do not invert the colours (light on dark). Many scanners fail on that.
+A very dark green, like our brand colour, is fine. Pale colours are not.</t>
+  </si>
+  <si>
+    <t>BLK00075</t>
+  </si>
+  <si>
+    <t>Leave a quiet zone</t>
+  </si>
+  <si>
+    <t>BLK00076</t>
+  </si>
+  <si>
+    <t>Keep an empty margin of at least four squares around the code. Our generator adds it for you. Do not crop it off, and do not print the code right against other graphics.</t>
+  </si>
+  <si>
+    <t>BLK00077</t>
+  </si>
+  <si>
+    <t>Pick the error correction level</t>
+  </si>
+  <si>
+    <t>BLK00078</t>
+  </si>
+  <si>
+    <t>Error correction lets a code still scan when part of it is dirty or damaged. Higher levels survive more damage but make the code denser. **Medium** suits most uses. Choose **High** for codes on stickers or outdoor signs that may get scratched.</t>
+  </si>
+  <si>
+    <t>BLK00079</t>
+  </si>
+  <si>
+    <t>Size and format</t>
+  </si>
+  <si>
+    <t>BLK00080</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For print, download the SVG, which stays sharp at any size, or a large PNG.
+For screens, a 512 pixel PNG is plenty.
+As a rule of thumb, a printed code should be at least 2 cm wide, and bigger if people will scan from a distance.</t>
+  </si>
+  <si>
+    <t>BLK00081</t>
+  </si>
+  <si>
+    <t>**Always test before you print.** Scan the code with two different phones, then print one copy and test that too.</t>
+  </si>
+  <si>
+    <t>BLK00090</t>
+  </si>
+  <si>
+    <t>When you use an online tool, the work has to happen somewhere. Either your file travels to someone else's computer (a server) and comes back, or the work happens on your own device, inside the browser.</t>
+  </si>
+  <si>
+    <t>BLK00091</t>
+  </si>
+  <si>
+    <t>Server-based tools</t>
+  </si>
+  <si>
+    <t>BLK00092</t>
+  </si>
+  <si>
+    <t>A server-based tool receives a copy of your file. That is not always a problem, but you have to trust the service to delete it, protect it and not use it for anything else. It also takes longer, because large files must be uploaded and downloaded.</t>
+  </si>
+  <si>
+    <t>BLK00093</t>
+  </si>
+  <si>
+    <t>Browser-based tools</t>
+  </si>
+  <si>
+    <t>BLK00094</t>
+  </si>
+  <si>
+    <t>Modern browsers can resize images, format data, generate codes and run calculations directly. A browser-based tool loads once and then does the work locally. Your file never goes anywhere, and it works as fast as your device allows.</t>
+  </si>
+  <si>
+    <t>BLK00095</t>
+  </si>
+  <si>
+    <t>How to check</t>
+  </si>
+  <si>
+    <t>BLK00096</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open your browser's developer tools and look at the Network tab while you use the tool. If your file is being sent, you will see a large request go out.
+Try turning off your internet connection after the page loads. A browser-based tool will keep working.
+Read the privacy policy. Honest tools say plainly whether files are uploaded.</t>
+  </si>
+  <si>
+    <t>BLK00097</t>
+  </si>
+  <si>
+    <t>How OEWER Tools works</t>
+  </si>
+  <si>
+    <t>BLK00098</t>
+  </si>
+  <si>
+    <t>All of our tools run in your browser. We test this: our automated tests watch the network while every tool is used and fail if anything is sent. That is the kind of promise you should be able to verify.</t>
+  </si>
+  <si>
+    <t>BLK00099</t>
+  </si>
+  <si>
+    <t>Private does not mean unlimited. Very large images can be slow on older phones, because your device is doing the work.</t>
+  </si>
+  <si>
     <t>tag_id</t>
   </si>
   <si>
@@ -907,6 +1349,42 @@
     <t>calculators</t>
   </si>
   <si>
+    <t>TAG0003</t>
+  </si>
+  <si>
+    <t>Images</t>
+  </si>
+  <si>
+    <t>images</t>
+  </si>
+  <si>
+    <t>TAG0004</t>
+  </si>
+  <si>
+    <t>Tax</t>
+  </si>
+  <si>
+    <t>tax</t>
+  </si>
+  <si>
+    <t>TAG0005</t>
+  </si>
+  <si>
+    <t>Savings</t>
+  </si>
+  <si>
+    <t>savings</t>
+  </si>
+  <si>
+    <t>TAG0006</t>
+  </si>
+  <si>
+    <t>Privacy</t>
+  </si>
+  <si>
+    <t>privacy</t>
+  </si>
+  <si>
     <t>relation_id</t>
   </si>
   <si>
@@ -916,6 +1394,30 @@
     <t>PTAG0002</t>
   </si>
   <si>
+    <t>PTAG0010</t>
+  </si>
+  <si>
+    <t>PTAG0011</t>
+  </si>
+  <si>
+    <t>PTAG0014</t>
+  </si>
+  <si>
+    <t>PTAG0015</t>
+  </si>
+  <si>
+    <t>PTAG0018</t>
+  </si>
+  <si>
+    <t>PTAG0019</t>
+  </si>
+  <si>
+    <t>PTAG0022</t>
+  </si>
+  <si>
+    <t>PTAG0026</t>
+  </si>
+  <si>
     <t>seo_id</t>
   </si>
   <si>
@@ -959,6 +1461,39 @@
   </si>
   <si>
     <t>Learn the EMI formula and how loan amount, interest rate and tenure change your monthly payment.</t>
+  </si>
+  <si>
+    <t>SEO0010</t>
+  </si>
+  <si>
+    <t>Choose the right format and quality setting to shrink JPG, PNG and WebP images while keeping them sharp, using a free in-browser tool.</t>
+  </si>
+  <si>
+    <t>SEO0011</t>
+  </si>
+  <si>
+    <t>Learn how to add GST to a price and remove it from a GST-inclusive total, with the formulas and worked examples for the 5%, 12%, 18% and 28% slabs.</t>
+  </si>
+  <si>
+    <t>SEO0012</t>
+  </si>
+  <si>
+    <t>Fixed Deposit Interest: Simple vs Compound Explained</t>
+  </si>
+  <si>
+    <t>See how simple and compound interest differ on a fixed deposit, with a worked ₹1,00,000 example and how compounding frequency changes the maturity amount.</t>
+  </si>
+  <si>
+    <t>SEO0013</t>
+  </si>
+  <si>
+    <t>Practical tips for QR codes that scan reliably: size, contrast, quiet zone, error correction and what to test before you print.</t>
+  </si>
+  <si>
+    <t>SEO0014</t>
+  </si>
+  <si>
+    <t>Understand the difference between tools that upload your files and tools that run in your browser, and how to check which kind you are using.</t>
   </si>
   <si>
     <t>SEO0003</t>
@@ -1560,7 +2095,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="12" customWidth="1"/>
@@ -1570,7 +2105,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>255</v>
+        <v>280</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>248</v>
@@ -1579,18 +2114,18 @@
         <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>256</v>
+        <v>281</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>26</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>257</v>
+        <v>282</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>258</v>
+        <v>283</v>
       </c>
       <c r="B2" t="s">
         <v>251</v>
@@ -1599,10 +2134,10 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>259</v>
+        <v>284</v>
       </c>
       <c r="E2" t="s">
-        <v>260</v>
+        <v>285</v>
       </c>
       <c r="F2" t="s">
         <v>247</v>
@@ -1610,7 +2145,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>261</v>
+        <v>286</v>
       </c>
       <c r="B3" t="s">
         <v>251</v>
@@ -1619,10 +2154,10 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>262</v>
+        <v>287</v>
       </c>
       <c r="E3" t="s">
-        <v>263</v>
+        <v>288</v>
       </c>
       <c r="F3" t="s">
         <v>247</v>
@@ -1630,7 +2165,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>264</v>
+        <v>289</v>
       </c>
       <c r="B4" t="s">
         <v>251</v>
@@ -1639,10 +2174,10 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>259</v>
+        <v>284</v>
       </c>
       <c r="E4" t="s">
-        <v>265</v>
+        <v>290</v>
       </c>
       <c r="F4" t="s">
         <v>247</v>
@@ -1650,7 +2185,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>266</v>
+        <v>291</v>
       </c>
       <c r="B5" t="s">
         <v>251</v>
@@ -1659,10 +2194,10 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>262</v>
+        <v>287</v>
       </c>
       <c r="E5" t="s">
-        <v>267</v>
+        <v>292</v>
       </c>
       <c r="F5" t="s">
         <v>247</v>
@@ -1670,7 +2205,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>268</v>
+        <v>293</v>
       </c>
       <c r="B6" t="s">
         <v>251</v>
@@ -1679,12 +2214,1132 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>269</v>
+        <v>294</v>
       </c>
       <c r="E6" t="s">
+        <v>295</v>
+      </c>
+      <c r="F6" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>296</v>
+      </c>
+      <c r="B7" t="s">
+        <v>255</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>284</v>
+      </c>
+      <c r="E7" t="s">
+        <v>297</v>
+      </c>
+      <c r="F7" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>298</v>
+      </c>
+      <c r="B8" t="s">
+        <v>255</v>
+      </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8" t="s">
+        <v>287</v>
+      </c>
+      <c r="E8" t="s">
+        <v>299</v>
+      </c>
+      <c r="F8" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>300</v>
+      </c>
+      <c r="B9" t="s">
+        <v>255</v>
+      </c>
+      <c r="C9">
+        <v>3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>284</v>
+      </c>
+      <c r="E9" t="s">
+        <v>301</v>
+      </c>
+      <c r="F9" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>302</v>
+      </c>
+      <c r="B10" t="s">
+        <v>255</v>
+      </c>
+      <c r="C10">
+        <v>4</v>
+      </c>
+      <c r="D10" t="s">
+        <v>287</v>
+      </c>
+      <c r="E10" t="s">
+        <v>303</v>
+      </c>
+      <c r="F10" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>304</v>
+      </c>
+      <c r="B11" t="s">
+        <v>255</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>294</v>
+      </c>
+      <c r="E11" t="s">
+        <v>305</v>
+      </c>
+      <c r="F11" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>306</v>
+      </c>
+      <c r="B12" t="s">
+        <v>255</v>
+      </c>
+      <c r="C12">
+        <v>6</v>
+      </c>
+      <c r="D12" t="s">
+        <v>287</v>
+      </c>
+      <c r="E12" t="s">
+        <v>307</v>
+      </c>
+      <c r="F12" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>308</v>
+      </c>
+      <c r="B13" t="s">
+        <v>255</v>
+      </c>
+      <c r="C13">
+        <v>7</v>
+      </c>
+      <c r="D13" t="s">
+        <v>284</v>
+      </c>
+      <c r="E13" t="s">
+        <v>309</v>
+      </c>
+      <c r="F13" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>310</v>
+      </c>
+      <c r="B14" t="s">
+        <v>255</v>
+      </c>
+      <c r="C14">
+        <v>8</v>
+      </c>
+      <c r="D14" t="s">
+        <v>311</v>
+      </c>
+      <c r="E14" t="s">
+        <v>312</v>
+      </c>
+      <c r="F14" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>313</v>
+      </c>
+      <c r="B15" t="s">
+        <v>255</v>
+      </c>
+      <c r="C15">
+        <v>9</v>
+      </c>
+      <c r="D15" t="s">
+        <v>287</v>
+      </c>
+      <c r="E15" t="s">
+        <v>314</v>
+      </c>
+      <c r="F15" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>315</v>
+      </c>
+      <c r="B16" t="s">
+        <v>255</v>
+      </c>
+      <c r="C16">
+        <v>10</v>
+      </c>
+      <c r="D16" t="s">
+        <v>284</v>
+      </c>
+      <c r="E16" t="s">
+        <v>316</v>
+      </c>
+      <c r="F16" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>317</v>
+      </c>
+      <c r="B17" t="s">
+        <v>260</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>284</v>
+      </c>
+      <c r="E17" t="s">
+        <v>318</v>
+      </c>
+      <c r="F17" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>319</v>
+      </c>
+      <c r="B18" t="s">
+        <v>260</v>
+      </c>
+      <c r="C18">
+        <v>2</v>
+      </c>
+      <c r="D18" t="s">
+        <v>287</v>
+      </c>
+      <c r="E18" t="s">
+        <v>320</v>
+      </c>
+      <c r="F18" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>321</v>
+      </c>
+      <c r="B19" t="s">
+        <v>260</v>
+      </c>
+      <c r="C19">
+        <v>3</v>
+      </c>
+      <c r="D19" t="s">
+        <v>284</v>
+      </c>
+      <c r="E19" t="s">
+        <v>322</v>
+      </c>
+      <c r="F19" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>323</v>
+      </c>
+      <c r="B20" t="s">
+        <v>260</v>
+      </c>
+      <c r="C20">
+        <v>4</v>
+      </c>
+      <c r="D20" t="s">
+        <v>284</v>
+      </c>
+      <c r="E20" t="s">
+        <v>324</v>
+      </c>
+      <c r="F20" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>325</v>
+      </c>
+      <c r="B21" t="s">
+        <v>260</v>
+      </c>
+      <c r="C21">
+        <v>5</v>
+      </c>
+      <c r="D21" t="s">
+        <v>287</v>
+      </c>
+      <c r="E21" t="s">
+        <v>326</v>
+      </c>
+      <c r="F21" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>327</v>
+      </c>
+      <c r="B22" t="s">
+        <v>260</v>
+      </c>
+      <c r="C22">
+        <v>6</v>
+      </c>
+      <c r="D22" t="s">
+        <v>284</v>
+      </c>
+      <c r="E22" t="s">
+        <v>328</v>
+      </c>
+      <c r="F22" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>329</v>
+      </c>
+      <c r="B23" t="s">
+        <v>260</v>
+      </c>
+      <c r="C23">
+        <v>7</v>
+      </c>
+      <c r="D23" t="s">
+        <v>284</v>
+      </c>
+      <c r="E23" t="s">
+        <v>330</v>
+      </c>
+      <c r="F23" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>331</v>
+      </c>
+      <c r="B24" t="s">
+        <v>260</v>
+      </c>
+      <c r="C24">
+        <v>8</v>
+      </c>
+      <c r="D24" t="s">
+        <v>287</v>
+      </c>
+      <c r="E24" t="s">
+        <v>332</v>
+      </c>
+      <c r="F24" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>333</v>
+      </c>
+      <c r="B25" t="s">
+        <v>260</v>
+      </c>
+      <c r="C25">
+        <v>9</v>
+      </c>
+      <c r="D25" t="s">
+        <v>294</v>
+      </c>
+      <c r="E25" t="s">
+        <v>334</v>
+      </c>
+      <c r="F25" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>335</v>
+      </c>
+      <c r="B26" t="s">
+        <v>260</v>
+      </c>
+      <c r="C26">
+        <v>10</v>
+      </c>
+      <c r="D26" t="s">
+        <v>287</v>
+      </c>
+      <c r="E26" t="s">
+        <v>336</v>
+      </c>
+      <c r="F26" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>337</v>
+      </c>
+      <c r="B27" t="s">
+        <v>260</v>
+      </c>
+      <c r="C27">
+        <v>11</v>
+      </c>
+      <c r="D27" t="s">
+        <v>284</v>
+      </c>
+      <c r="E27" t="s">
+        <v>338</v>
+      </c>
+      <c r="F27" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>339</v>
+      </c>
+      <c r="B28" t="s">
+        <v>260</v>
+      </c>
+      <c r="C28">
+        <v>12</v>
+      </c>
+      <c r="D28" t="s">
+        <v>311</v>
+      </c>
+      <c r="E28" t="s">
+        <v>340</v>
+      </c>
+      <c r="F28" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>341</v>
+      </c>
+      <c r="B29" t="s">
+        <v>265</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+      <c r="D29" t="s">
+        <v>284</v>
+      </c>
+      <c r="E29" t="s">
+        <v>342</v>
+      </c>
+      <c r="F29" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>343</v>
+      </c>
+      <c r="B30" t="s">
+        <v>265</v>
+      </c>
+      <c r="C30">
+        <v>2</v>
+      </c>
+      <c r="D30" t="s">
+        <v>287</v>
+      </c>
+      <c r="E30" t="s">
+        <v>344</v>
+      </c>
+      <c r="F30" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>345</v>
+      </c>
+      <c r="B31" t="s">
+        <v>265</v>
+      </c>
+      <c r="C31">
+        <v>3</v>
+      </c>
+      <c r="D31" t="s">
+        <v>284</v>
+      </c>
+      <c r="E31" t="s">
+        <v>346</v>
+      </c>
+      <c r="F31" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>347</v>
+      </c>
+      <c r="B32" t="s">
+        <v>265</v>
+      </c>
+      <c r="C32">
+        <v>4</v>
+      </c>
+      <c r="D32" t="s">
+        <v>284</v>
+      </c>
+      <c r="E32" t="s">
+        <v>348</v>
+      </c>
+      <c r="F32" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>349</v>
+      </c>
+      <c r="B33" t="s">
+        <v>265</v>
+      </c>
+      <c r="C33">
+        <v>5</v>
+      </c>
+      <c r="D33" t="s">
+        <v>287</v>
+      </c>
+      <c r="E33" t="s">
+        <v>350</v>
+      </c>
+      <c r="F33" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>351</v>
+      </c>
+      <c r="B34" t="s">
+        <v>265</v>
+      </c>
+      <c r="C34">
+        <v>6</v>
+      </c>
+      <c r="D34" t="s">
+        <v>284</v>
+      </c>
+      <c r="E34" t="s">
+        <v>352</v>
+      </c>
+      <c r="F34" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>353</v>
+      </c>
+      <c r="B35" t="s">
+        <v>265</v>
+      </c>
+      <c r="C35">
+        <v>7</v>
+      </c>
+      <c r="D35" t="s">
+        <v>284</v>
+      </c>
+      <c r="E35" t="s">
+        <v>354</v>
+      </c>
+      <c r="F35" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>355</v>
+      </c>
+      <c r="B36" t="s">
+        <v>265</v>
+      </c>
+      <c r="C36">
+        <v>8</v>
+      </c>
+      <c r="D36" t="s">
+        <v>287</v>
+      </c>
+      <c r="E36" t="s">
+        <v>356</v>
+      </c>
+      <c r="F36" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>357</v>
+      </c>
+      <c r="B37" t="s">
+        <v>265</v>
+      </c>
+      <c r="C37">
+        <v>9</v>
+      </c>
+      <c r="D37" t="s">
+        <v>284</v>
+      </c>
+      <c r="E37" t="s">
+        <v>358</v>
+      </c>
+      <c r="F37" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>359</v>
+      </c>
+      <c r="B38" t="s">
+        <v>265</v>
+      </c>
+      <c r="C38">
+        <v>10</v>
+      </c>
+      <c r="D38" t="s">
+        <v>294</v>
+      </c>
+      <c r="E38" t="s">
+        <v>360</v>
+      </c>
+      <c r="F38" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>361</v>
+      </c>
+      <c r="B39" t="s">
+        <v>265</v>
+      </c>
+      <c r="C39">
+        <v>11</v>
+      </c>
+      <c r="D39" t="s">
+        <v>284</v>
+      </c>
+      <c r="E39" t="s">
+        <v>362</v>
+      </c>
+      <c r="F39" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>363</v>
+      </c>
+      <c r="B40" t="s">
+        <v>265</v>
+      </c>
+      <c r="C40">
+        <v>12</v>
+      </c>
+      <c r="D40" t="s">
+        <v>311</v>
+      </c>
+      <c r="E40" t="s">
+        <v>364</v>
+      </c>
+      <c r="F40" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>365</v>
+      </c>
+      <c r="B41" t="s">
         <v>270</v>
       </c>
-      <c r="F6" t="s">
+      <c r="C41">
+        <v>1</v>
+      </c>
+      <c r="D41" t="s">
+        <v>284</v>
+      </c>
+      <c r="E41" t="s">
+        <v>366</v>
+      </c>
+      <c r="F41" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>367</v>
+      </c>
+      <c r="B42" t="s">
+        <v>270</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="D42" t="s">
+        <v>287</v>
+      </c>
+      <c r="E42" t="s">
+        <v>368</v>
+      </c>
+      <c r="F42" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>369</v>
+      </c>
+      <c r="B43" t="s">
+        <v>270</v>
+      </c>
+      <c r="C43">
+        <v>3</v>
+      </c>
+      <c r="D43" t="s">
+        <v>284</v>
+      </c>
+      <c r="E43" t="s">
+        <v>370</v>
+      </c>
+      <c r="F43" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>371</v>
+      </c>
+      <c r="B44" t="s">
+        <v>270</v>
+      </c>
+      <c r="C44">
+        <v>4</v>
+      </c>
+      <c r="D44" t="s">
+        <v>287</v>
+      </c>
+      <c r="E44" t="s">
+        <v>372</v>
+      </c>
+      <c r="F44" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>373</v>
+      </c>
+      <c r="B45" t="s">
+        <v>270</v>
+      </c>
+      <c r="C45">
+        <v>5</v>
+      </c>
+      <c r="D45" t="s">
+        <v>294</v>
+      </c>
+      <c r="E45" t="s">
+        <v>374</v>
+      </c>
+      <c r="F45" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>375</v>
+      </c>
+      <c r="B46" t="s">
+        <v>270</v>
+      </c>
+      <c r="C46">
+        <v>6</v>
+      </c>
+      <c r="D46" t="s">
+        <v>287</v>
+      </c>
+      <c r="E46" t="s">
+        <v>376</v>
+      </c>
+      <c r="F46" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>377</v>
+      </c>
+      <c r="B47" t="s">
+        <v>270</v>
+      </c>
+      <c r="C47">
+        <v>7</v>
+      </c>
+      <c r="D47" t="s">
+        <v>284</v>
+      </c>
+      <c r="E47" t="s">
+        <v>378</v>
+      </c>
+      <c r="F47" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>379</v>
+      </c>
+      <c r="B48" t="s">
+        <v>270</v>
+      </c>
+      <c r="C48">
+        <v>8</v>
+      </c>
+      <c r="D48" t="s">
+        <v>287</v>
+      </c>
+      <c r="E48" t="s">
+        <v>380</v>
+      </c>
+      <c r="F48" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>381</v>
+      </c>
+      <c r="B49" t="s">
+        <v>270</v>
+      </c>
+      <c r="C49">
+        <v>9</v>
+      </c>
+      <c r="D49" t="s">
+        <v>284</v>
+      </c>
+      <c r="E49" t="s">
+        <v>382</v>
+      </c>
+      <c r="F49" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>383</v>
+      </c>
+      <c r="B50" t="s">
+        <v>270</v>
+      </c>
+      <c r="C50">
+        <v>10</v>
+      </c>
+      <c r="D50" t="s">
+        <v>287</v>
+      </c>
+      <c r="E50" t="s">
+        <v>384</v>
+      </c>
+      <c r="F50" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>385</v>
+      </c>
+      <c r="B51" t="s">
+        <v>270</v>
+      </c>
+      <c r="C51">
+        <v>11</v>
+      </c>
+      <c r="D51" t="s">
+        <v>294</v>
+      </c>
+      <c r="E51" t="s">
+        <v>386</v>
+      </c>
+      <c r="F51" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>387</v>
+      </c>
+      <c r="B52" t="s">
+        <v>270</v>
+      </c>
+      <c r="C52">
+        <v>12</v>
+      </c>
+      <c r="D52" t="s">
+        <v>311</v>
+      </c>
+      <c r="E52" t="s">
+        <v>388</v>
+      </c>
+      <c r="F52" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>389</v>
+      </c>
+      <c r="B53" t="s">
+        <v>275</v>
+      </c>
+      <c r="C53">
+        <v>1</v>
+      </c>
+      <c r="D53" t="s">
+        <v>284</v>
+      </c>
+      <c r="E53" t="s">
+        <v>390</v>
+      </c>
+      <c r="F53" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>391</v>
+      </c>
+      <c r="B54" t="s">
+        <v>275</v>
+      </c>
+      <c r="C54">
+        <v>2</v>
+      </c>
+      <c r="D54" t="s">
+        <v>287</v>
+      </c>
+      <c r="E54" t="s">
+        <v>392</v>
+      </c>
+      <c r="F54" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>393</v>
+      </c>
+      <c r="B55" t="s">
+        <v>275</v>
+      </c>
+      <c r="C55">
+        <v>3</v>
+      </c>
+      <c r="D55" t="s">
+        <v>284</v>
+      </c>
+      <c r="E55" t="s">
+        <v>394</v>
+      </c>
+      <c r="F55" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>395</v>
+      </c>
+      <c r="B56" t="s">
+        <v>275</v>
+      </c>
+      <c r="C56">
+        <v>4</v>
+      </c>
+      <c r="D56" t="s">
+        <v>287</v>
+      </c>
+      <c r="E56" t="s">
+        <v>396</v>
+      </c>
+      <c r="F56" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>397</v>
+      </c>
+      <c r="B57" t="s">
+        <v>275</v>
+      </c>
+      <c r="C57">
+        <v>5</v>
+      </c>
+      <c r="D57" t="s">
+        <v>284</v>
+      </c>
+      <c r="E57" t="s">
+        <v>398</v>
+      </c>
+      <c r="F57" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>399</v>
+      </c>
+      <c r="B58" t="s">
+        <v>275</v>
+      </c>
+      <c r="C58">
+        <v>6</v>
+      </c>
+      <c r="D58" t="s">
+        <v>287</v>
+      </c>
+      <c r="E58" t="s">
+        <v>400</v>
+      </c>
+      <c r="F58" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>401</v>
+      </c>
+      <c r="B59" t="s">
+        <v>275</v>
+      </c>
+      <c r="C59">
+        <v>7</v>
+      </c>
+      <c r="D59" t="s">
+        <v>294</v>
+      </c>
+      <c r="E59" t="s">
+        <v>402</v>
+      </c>
+      <c r="F59" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>403</v>
+      </c>
+      <c r="B60" t="s">
+        <v>275</v>
+      </c>
+      <c r="C60">
+        <v>8</v>
+      </c>
+      <c r="D60" t="s">
+        <v>287</v>
+      </c>
+      <c r="E60" t="s">
+        <v>404</v>
+      </c>
+      <c r="F60" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>405</v>
+      </c>
+      <c r="B61" t="s">
+        <v>275</v>
+      </c>
+      <c r="C61">
+        <v>9</v>
+      </c>
+      <c r="D61" t="s">
+        <v>284</v>
+      </c>
+      <c r="E61" t="s">
+        <v>406</v>
+      </c>
+      <c r="F61" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>407</v>
+      </c>
+      <c r="B62" t="s">
+        <v>275</v>
+      </c>
+      <c r="C62">
+        <v>10</v>
+      </c>
+      <c r="D62" t="s">
+        <v>311</v>
+      </c>
+      <c r="E62" t="s">
+        <v>408</v>
+      </c>
+      <c r="F62" t="s">
         <v>247</v>
       </c>
     </row>
@@ -1696,7 +3351,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1705,7 +3360,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>271</v>
+        <v>409</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>72</v>
@@ -1716,24 +3371,68 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>272</v>
+        <v>410</v>
       </c>
       <c r="B2" t="s">
-        <v>273</v>
+        <v>411</v>
       </c>
       <c r="C2" t="s">
-        <v>274</v>
+        <v>412</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>275</v>
+        <v>413</v>
       </c>
       <c r="B3" t="s">
-        <v>276</v>
+        <v>414</v>
       </c>
       <c r="C3" t="s">
-        <v>277</v>
+        <v>415</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>416</v>
+      </c>
+      <c r="B4" t="s">
+        <v>417</v>
+      </c>
+      <c r="C4" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>419</v>
+      </c>
+      <c r="B5" t="s">
+        <v>420</v>
+      </c>
+      <c r="C5" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>422</v>
+      </c>
+      <c r="B6" t="s">
+        <v>423</v>
+      </c>
+      <c r="C6" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>425</v>
+      </c>
+      <c r="B7" t="s">
+        <v>426</v>
+      </c>
+      <c r="C7" t="s">
+        <v>427</v>
       </c>
     </row>
   </sheetData>
@@ -1744,7 +3443,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1753,35 +3452,123 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>278</v>
+        <v>428</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>248</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>271</v>
+        <v>409</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>279</v>
+        <v>429</v>
       </c>
       <c r="B2" t="s">
         <v>251</v>
       </c>
       <c r="C2" t="s">
-        <v>272</v>
+        <v>410</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>280</v>
+        <v>430</v>
       </c>
       <c r="B3" t="s">
         <v>251</v>
       </c>
       <c r="C3" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>431</v>
+      </c>
+      <c r="B4" t="s">
+        <v>255</v>
+      </c>
+      <c r="C4" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>432</v>
+      </c>
+      <c r="B5" t="s">
+        <v>255</v>
+      </c>
+      <c r="C5" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>433</v>
+      </c>
+      <c r="B6" t="s">
+        <v>260</v>
+      </c>
+      <c r="C6" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>434</v>
+      </c>
+      <c r="B7" t="s">
+        <v>260</v>
+      </c>
+      <c r="C7" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>435</v>
+      </c>
+      <c r="B8" t="s">
+        <v>265</v>
+      </c>
+      <c r="C8" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>436</v>
+      </c>
+      <c r="B9" t="s">
+        <v>265</v>
+      </c>
+      <c r="C9" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>437</v>
+      </c>
+      <c r="B10" t="s">
+        <v>270</v>
+      </c>
+      <c r="C10" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>438</v>
+      </c>
+      <c r="B11" t="s">
         <v>275</v>
+      </c>
+      <c r="C11" t="s">
+        <v>425</v>
       </c>
     </row>
   </sheetData>
@@ -1792,13 +3579,13 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="43" customWidth="1"/>
+    <col min="4" max="4" width="54" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
@@ -1806,42 +3593,42 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>281</v>
+        <v>439</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>282</v>
+        <v>440</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>283</v>
+        <v>441</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>284</v>
+        <v>442</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>285</v>
+        <v>443</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>286</v>
+        <v>444</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>287</v>
+        <v>445</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>288</v>
+        <v>446</v>
       </c>
       <c r="B2" t="s">
-        <v>289</v>
+        <v>447</v>
       </c>
       <c r="C2" t="s">
         <v>105</v>
       </c>
       <c r="D2" t="s">
-        <v>290</v>
+        <v>448</v>
       </c>
       <c r="E2" t="s">
-        <v>291</v>
+        <v>449</v>
       </c>
       <c r="F2" t="s">
         <v>247</v>
@@ -1852,19 +3639,19 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>292</v>
+        <v>450</v>
       </c>
       <c r="B3" t="s">
-        <v>293</v>
+        <v>451</v>
       </c>
       <c r="C3" t="s">
         <v>251</v>
       </c>
       <c r="D3" t="s">
-        <v>294</v>
+        <v>452</v>
       </c>
       <c r="E3" t="s">
-        <v>295</v>
+        <v>453</v>
       </c>
       <c r="F3" t="s">
         <v>247</v>
@@ -1875,24 +3662,139 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>296</v>
+        <v>454</v>
       </c>
       <c r="B4" t="s">
-        <v>297</v>
+        <v>451</v>
       </c>
       <c r="C4" t="s">
+        <v>255</v>
+      </c>
+      <c r="D4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E4" t="s">
+        <v>455</v>
+      </c>
+      <c r="F4" t="s">
+        <v>247</v>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>456</v>
+      </c>
+      <c r="B5" t="s">
+        <v>451</v>
+      </c>
+      <c r="C5" t="s">
+        <v>260</v>
+      </c>
+      <c r="D5" t="s">
+        <v>261</v>
+      </c>
+      <c r="E5" t="s">
+        <v>457</v>
+      </c>
+      <c r="F5" t="s">
+        <v>247</v>
+      </c>
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>458</v>
+      </c>
+      <c r="B6" t="s">
+        <v>451</v>
+      </c>
+      <c r="C6" t="s">
+        <v>265</v>
+      </c>
+      <c r="D6" t="s">
+        <v>459</v>
+      </c>
+      <c r="E6" t="s">
+        <v>460</v>
+      </c>
+      <c r="F6" t="s">
+        <v>247</v>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>461</v>
+      </c>
+      <c r="B7" t="s">
+        <v>451</v>
+      </c>
+      <c r="C7" t="s">
+        <v>270</v>
+      </c>
+      <c r="D7" t="s">
+        <v>271</v>
+      </c>
+      <c r="E7" t="s">
+        <v>462</v>
+      </c>
+      <c r="F7" t="s">
+        <v>247</v>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>463</v>
+      </c>
+      <c r="B8" t="s">
+        <v>451</v>
+      </c>
+      <c r="C8" t="s">
+        <v>275</v>
+      </c>
+      <c r="D8" t="s">
+        <v>276</v>
+      </c>
+      <c r="E8" t="s">
+        <v>464</v>
+      </c>
+      <c r="F8" t="s">
+        <v>247</v>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>465</v>
+      </c>
+      <c r="B9" t="s">
+        <v>466</v>
+      </c>
+      <c r="C9" t="s">
         <v>28</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D9" t="s">
         <v>30</v>
       </c>
-      <c r="E4" t="s">
-        <v>298</v>
-      </c>
-      <c r="F4" t="s">
-        <v>247</v>
-      </c>
-      <c r="G4" t="b">
+      <c r="E9" t="s">
+        <v>467</v>
+      </c>
+      <c r="F9" t="s">
+        <v>247</v>
+      </c>
+      <c r="G9" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1914,30 +3816,30 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>299</v>
+        <v>468</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>300</v>
+        <v>469</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>301</v>
+        <v>470</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>302</v>
+        <v>471</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>303</v>
+        <v>472</v>
       </c>
       <c r="B2" t="s">
-        <v>304</v>
+        <v>473</v>
       </c>
       <c r="C2" t="s">
-        <v>305</v>
+        <v>474</v>
       </c>
       <c r="D2" t="b">
         <v>0</v>
@@ -1948,13 +3850,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>306</v>
+        <v>475</v>
       </c>
       <c r="B3" t="s">
-        <v>307</v>
+        <v>476</v>
       </c>
       <c r="C3" t="s">
-        <v>289</v>
+        <v>447</v>
       </c>
       <c r="D3" t="b">
         <v>0</v>
@@ -1965,13 +3867,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>308</v>
+        <v>477</v>
       </c>
       <c r="B4" t="s">
-        <v>309</v>
+        <v>478</v>
       </c>
       <c r="C4" t="s">
-        <v>310</v>
+        <v>479</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
@@ -2000,16 +3902,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>311</v>
+        <v>480</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>312</v>
+        <v>481</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>313</v>
+        <v>482</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>314</v>
+        <v>483</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>51</v>
@@ -2017,16 +3919,16 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>315</v>
+        <v>484</v>
       </c>
       <c r="B2" t="s">
-        <v>316</v>
+        <v>485</v>
       </c>
       <c r="C2" t="s">
-        <v>317</v>
+        <v>486</v>
       </c>
       <c r="D2" t="s">
-        <v>318</v>
+        <v>487</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -2060,7 +3962,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>319</v>
+        <v>488</v>
       </c>
       <c r="B2" t="s">
         <v>136</v>
@@ -3695,11 +5597,11 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="3" width="23" customWidth="1"/>
+    <col min="2" max="3" width="49" customWidth="1"/>
     <col min="4" max="4" width="60" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="7" width="12" customWidth="1"/>
@@ -3764,6 +5666,151 @@
         <v>7</v>
       </c>
     </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>255</v>
+      </c>
+      <c r="B3" t="s">
+        <v>256</v>
+      </c>
+      <c r="C3" t="s">
+        <v>257</v>
+      </c>
+      <c r="D3" t="s">
+        <v>258</v>
+      </c>
+      <c r="E3" t="s">
+        <v>236</v>
+      </c>
+      <c r="F3" t="s">
+        <v>244</v>
+      </c>
+      <c r="G3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" t="s">
+        <v>259</v>
+      </c>
+      <c r="I3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>260</v>
+      </c>
+      <c r="B4" t="s">
+        <v>261</v>
+      </c>
+      <c r="C4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D4" t="s">
+        <v>263</v>
+      </c>
+      <c r="E4" t="s">
+        <v>232</v>
+      </c>
+      <c r="F4" t="s">
+        <v>244</v>
+      </c>
+      <c r="G4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H4" t="s">
+        <v>264</v>
+      </c>
+      <c r="I4" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>265</v>
+      </c>
+      <c r="B5" t="s">
+        <v>266</v>
+      </c>
+      <c r="C5" t="s">
+        <v>267</v>
+      </c>
+      <c r="D5" t="s">
+        <v>268</v>
+      </c>
+      <c r="E5" t="s">
+        <v>232</v>
+      </c>
+      <c r="F5" t="s">
+        <v>244</v>
+      </c>
+      <c r="G5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" t="s">
+        <v>269</v>
+      </c>
+      <c r="I5" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>270</v>
+      </c>
+      <c r="B6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C6" t="s">
+        <v>272</v>
+      </c>
+      <c r="D6" t="s">
+        <v>273</v>
+      </c>
+      <c r="E6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F6" t="s">
+        <v>244</v>
+      </c>
+      <c r="G6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" t="s">
+        <v>274</v>
+      </c>
+      <c r="I6" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>275</v>
+      </c>
+      <c r="B7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C7" t="s">
+        <v>277</v>
+      </c>
+      <c r="D7" t="s">
+        <v>278</v>
+      </c>
+      <c r="E7" t="s">
+        <v>236</v>
+      </c>
+      <c r="F7" t="s">
+        <v>244</v>
+      </c>
+      <c r="G7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" t="s">
+        <v>279</v>
+      </c>
+      <c r="I7" t="s">
+        <v>279</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Blog engine: anchors, tags, authors, RSS, statuses, related links (T4.1-T4.4)
Article anchors and outline, Article structured data, image checks, tag and
author pages, RSS feed, archived/draft handling with preview builds, and
two-way tool-to-article links with automatic related articles.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="957" uniqueCount="489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="507">
   <si>
     <t>setting_key</t>
   </si>
@@ -533,6 +533,15 @@
     <t>TSET0009</t>
   </si>
   <si>
+    <t>guides</t>
+  </si>
+  <si>
+    <t>["POST0002","POST0006"]</t>
+  </si>
+  <si>
+    <t>TSET0010</t>
+  </si>
+  <si>
     <t xml:space="preserve">Follow these steps:
 - Choose a JPG, PNG or WebP image. Its current size is filled in for you.
 - Either type a new width or height in pixels, or switch to a percentage of the original.
@@ -540,25 +549,31 @@
 - Download the resized image.</t>
   </si>
   <si>
-    <t>TSET0010</t>
+    <t>TSET0011</t>
   </si>
   <si>
     <t>[{"title":"Profile picture","text":"Set the width to 400 with proportions kept. A 2000 × 1500 photo becomes 400 × 300."},{"title":"Half size","text":"Switch to percentage and enter 50 to halve both width and height."}]</t>
   </si>
   <si>
-    <t>TSET0011</t>
+    <t>TSET0012</t>
   </si>
   <si>
     <t>[{"q":"Does resizing reduce quality?","a":"Making an image smaller keeps it sharp. Making it larger cannot add detail, so enlarged images look soft."},{"q":"Which format is the result?","a":"The same format as the image you chose. Use the image converter to change format."},{"q":"Is my image uploaded anywhere?","a":"No. Everything happens in your browser on your own device."}]</t>
   </si>
   <si>
-    <t>TSET0012</t>
+    <t>TSET0013</t>
   </si>
   <si>
     <t>["TOOL0001","TOOL0003"]</t>
   </si>
   <si>
-    <t>TSET0013</t>
+    <t>TSET0014</t>
+  </si>
+  <si>
+    <t>["POST0002"]</t>
+  </si>
+  <si>
+    <t>TSET0015</t>
   </si>
   <si>
     <t xml:space="preserve">Follow these steps:
@@ -568,25 +583,28 @@
 - Download the converted image.</t>
   </si>
   <si>
-    <t>TSET0014</t>
+    <t>TSET0016</t>
   </si>
   <si>
     <t>[{"title":"PNG to JPG","text":"Convert a PNG screenshot to JPG for a smaller file. Transparent areas turn white."},{"title":"JPG to WebP","text":"Convert a JPG to WebP at 90% quality for a smaller file with similar looks."}]</t>
   </si>
   <si>
-    <t>TSET0015</t>
+    <t>TSET0017</t>
   </si>
   <si>
     <t>[{"q":"What happens to transparency?","a":"PNG and WebP keep transparent areas. JPG cannot, so transparent areas become white."},{"q":"Can it convert GIF, HEIC or other types?","a":"Not yet. Only JPG, PNG and WebP are supported."},{"q":"Is my image uploaded anywhere?","a":"No. Everything happens in your browser on your own device."}]</t>
   </si>
   <si>
-    <t>TSET0016</t>
+    <t>TSET0018</t>
   </si>
   <si>
     <t>["TOOL0001","TOOL0002"]</t>
   </si>
   <si>
-    <t>TSET0017</t>
+    <t>TSET0019</t>
+  </si>
+  <si>
+    <t>TSET0020</t>
   </si>
   <si>
     <t xml:space="preserve">Follow these steps:
@@ -597,25 +615,31 @@
 EMI = P × r × (1 + r)^n ÷ ((1 + r)^n − 1), where P is the loan amount, r is the monthly rate (yearly rate ÷ 12 ÷ 100) and n is the number of months.</t>
   </si>
   <si>
-    <t>TSET0018</t>
+    <t>TSET0021</t>
   </si>
   <si>
     <t>[{"title":"Home loan","text":"₹50,00,000 at 8.5% for 20 years gives a monthly EMI of about ₹43,391."},{"title":"Car loan","text":"₹8,00,000 at 9% for 5 years gives a monthly EMI of about ₹16,607."}]</t>
   </si>
   <si>
-    <t>TSET0019</t>
+    <t>TSET0022</t>
   </si>
   <si>
     <t>[{"q":"Does this match my bank's figure?","a":"It uses the standard reducing-balance formula. Banks may differ slightly because of rounding, processing fees or the day the first instalment falls."},{"q":"Does it include processing fees or insurance?","a":"No. It only calculates principal and interest."},{"q":"Is the information I type saved?","a":"No. The calculation runs in your browser and nothing is sent or stored."}]</t>
   </si>
   <si>
-    <t>TSET0020</t>
+    <t>TSET0023</t>
   </si>
   <si>
     <t>["TOOL0005","TOOL0007"]</t>
   </si>
   <si>
-    <t>TSET0021</t>
+    <t>TSET0024</t>
+  </si>
+  <si>
+    <t>["POST0001"]</t>
+  </si>
+  <si>
+    <t>TSET0025</t>
   </si>
   <si>
     <t xml:space="preserve">Follow these steps:
@@ -626,25 +650,31 @@
 Maturity = P × (1 + r ÷ n)^(n × t), where P is the deposit, r the yearly rate, n the compounding periods per year and t the years. With simple interest, maturity = P × (1 + r × t).</t>
   </si>
   <si>
-    <t>TSET0022</t>
+    <t>TSET0026</t>
   </si>
   <si>
     <t>[{"title":"Three-year deposit","text":"₹1,00,000 at 7% compounded quarterly for 3 years matures to about ₹1,23,144."},{"title":"Simple interest","text":"₹1,00,000 at 7% simple interest for 2 years earns ₹14,000."}]</t>
   </si>
   <si>
-    <t>TSET0023</t>
+    <t>TSET0027</t>
   </si>
   <si>
     <t>[{"q":"Is the interest taxable?","a":"Interest on fixed deposits is usually taxable. This calculator does not include tax or TDS."},{"q":"Why is my bank's maturity amount a little different?","a":"Banks round each period and may count days exactly. Use this as a close estimate."},{"q":"Is the information I type saved?","a":"No. The calculation runs in your browser and nothing is sent or stored."}]</t>
   </si>
   <si>
-    <t>TSET0024</t>
+    <t>TSET0028</t>
   </si>
   <si>
     <t>["TOOL0004","TOOL0007"]</t>
   </si>
   <si>
-    <t>TSET0025</t>
+    <t>TSET0029</t>
+  </si>
+  <si>
+    <t>["POST0004"]</t>
+  </si>
+  <si>
+    <t>TSET0030</t>
   </si>
   <si>
     <t xml:space="preserve">Follow these steps:
@@ -653,25 +683,31 @@
 - See the amount without GST, the GST, and the CGST and SGST halves.</t>
   </si>
   <si>
-    <t>TSET0026</t>
+    <t>TSET0031</t>
   </si>
   <si>
     <t>[{"title":"Add GST","text":"₹1,000 plus 18% GST gives ₹180 of GST and a total of ₹1,180."},{"title":"Remove GST","text":"A bill of ₹1,180 that includes 18% GST is ₹1,000 before tax, with ₹180 of GST."}]</t>
   </si>
   <si>
-    <t>TSET0027</t>
+    <t>TSET0032</t>
   </si>
   <si>
     <t>[{"q":"What are CGST and SGST?","a":"For a sale within one state, GST is split equally between the central (CGST) and state (SGST) governments. For a sale between states, the whole amount is IGST."},{"q":"Does it check the correct rate for my goods?","a":"No. Enter the rate that applies to your goods or services. Check the official GST rate schedule if you are unsure."},{"q":"Is the information I type saved?","a":"No. The calculation runs in your browser and nothing is sent or stored."}]</t>
   </si>
   <si>
-    <t>TSET0028</t>
+    <t>TSET0033</t>
   </si>
   <si>
     <t>["TOOL0007","TOOL0004"]</t>
   </si>
   <si>
-    <t>TSET0029</t>
+    <t>TSET0034</t>
+  </si>
+  <si>
+    <t>["POST0003"]</t>
+  </si>
+  <si>
+    <t>TSET0035</t>
   </si>
   <si>
     <t xml:space="preserve">Pick the kind of calculation, then enter two numbers:
@@ -681,25 +717,28 @@
 - **Increase or decrease X by Y%**: for example, a price rise of 10%.</t>
   </si>
   <si>
-    <t>TSET0030</t>
+    <t>TSET0036</t>
   </si>
   <si>
     <t>[{"title":"Discount","text":"Decrease 2,000 by 25% to get 1,500."},{"title":"Marks","text":"42 out of 60 is 70%."},{"title":"Price change","text":"From 80 to 100 is a 25% increase."}]</t>
   </si>
   <si>
-    <t>TSET0031</t>
+    <t>TSET0037</t>
   </si>
   <si>
     <t>[{"q":"Why can't the old value be 0 for a % change?","a":"A change from zero cannot be shown as a percentage because dividing by zero is undefined."},{"q":"Can I use decimals and negative numbers?","a":"Yes for most modes. Commas in numbers such as 1,00,000 are fine."},{"q":"Is the information I type saved?","a":"No. The calculation runs in your browser and nothing is sent or stored."}]</t>
   </si>
   <si>
-    <t>TSET0032</t>
+    <t>TSET0038</t>
   </si>
   <si>
     <t>["TOOL0006","TOOL0004"]</t>
   </si>
   <si>
-    <t>TSET0033</t>
+    <t>TSET0039</t>
+  </si>
+  <si>
+    <t>TSET0040</t>
   </si>
   <si>
     <t xml:space="preserve">Follow these steps:
@@ -710,25 +749,31 @@
 If the JSON is invalid, the message says what is wrong and, where your browser gives it, the line and column.</t>
   </si>
   <si>
-    <t>TSET0034</t>
+    <t>TSET0041</t>
   </si>
   <si>
     <t>[{"title":"Tidy a response","text":"Paste {\"name\":\"OEWER\",\"tools\":[1,2]} and choose Format to see it spread over several indented lines."},{"title":"Find a mistake","text":"A trailing comma such as {\"a\": 1,} is not valid JSON. The error message points to where it goes wrong."}]</t>
   </si>
   <si>
-    <t>TSET0035</t>
+    <t>TSET0042</t>
   </si>
   <si>
     <t>[{"q":"Is my JSON sent to a server?","a":"No. It is checked and formatted in your browser and never leaves your device."},{"q":"Why is my JSON invalid when it works in my code?","a":"JSON is stricter than JavaScript: keys need double quotes, single quotes are not allowed, and trailing commas and comments are not allowed."},{"q":"How large can the input be?","a":"Up to 5 million characters."}]</t>
   </si>
   <si>
-    <t>TSET0036</t>
+    <t>TSET0043</t>
   </si>
   <si>
     <t>["TOOL0010","TOOL0009"]</t>
   </si>
   <si>
-    <t>TSET0037</t>
+    <t>TSET0044</t>
+  </si>
+  <si>
+    <t>["POST0006"]</t>
+  </si>
+  <si>
+    <t>TSET0045</t>
   </si>
   <si>
     <t xml:space="preserve">Follow these steps:
@@ -739,25 +784,31 @@
 Always test the code with a phone before you print it.</t>
   </si>
   <si>
-    <t>TSET0038</t>
+    <t>TSET0046</t>
   </si>
   <si>
     <t>[{"title":"Website link","text":"Enter https://example.com to make a code that opens the site when scanned."},{"title":"Wi-Fi details","text":"Enter WIFI:T:WPA;S:MyNetwork;P:mypassword;; and phones can join the network by scanning."}]</t>
   </si>
   <si>
-    <t>TSET0039</t>
+    <t>TSET0047</t>
   </si>
   <si>
     <t>[{"q":"Do the codes expire?","a":"No. The text is stored in the code itself, so it works as long as it is readable."},{"q":"Is my text sent to a server?","a":"No. The code is generated in your browser and your text never leaves your device."},{"q":"PNG or SVG?","a":"Use PNG for screens and documents. Use SVG when you need it to stay sharp at any size, for example for print."}]</t>
   </si>
   <si>
-    <t>TSET0040</t>
+    <t>TSET0048</t>
   </si>
   <si>
     <t>["TOOL0010","TOOL0008"]</t>
   </si>
   <si>
-    <t>TSET0041</t>
+    <t>TSET0049</t>
+  </si>
+  <si>
+    <t>["POST0005","POST0006"]</t>
+  </si>
+  <si>
+    <t>TSET0050</t>
   </si>
   <si>
     <t xml:space="preserve">Follow these steps:
@@ -766,22 +817,25 @@
 - Reading and speaking time are estimates based on average speeds.</t>
   </si>
   <si>
-    <t>TSET0042</t>
+    <t>TSET0051</t>
   </si>
   <si>
     <t>[{"title":"Essay limit","text":"Paste your essay to check it is within a 500-word limit."},{"title":"Social post","text":"Check a post stays under a character limit, counting spaces."}]</t>
   </si>
   <si>
-    <t>TSET0043</t>
+    <t>TSET0052</t>
   </si>
   <si>
     <t>[{"q":"How are words counted?","a":"A word is a run of letters or numbers separated by spaces or punctuation. Hyphenated words and numbers each count as words."},{"q":"How are reading and speaking time worked out?","a":"Reading time assumes 200 words a minute and speaking time 130 words a minute."},{"q":"Is my text sent to a server?","a":"No. The count happens in your browser and your text never leaves your device."}]</t>
   </si>
   <si>
-    <t>TSET0044</t>
+    <t>TSET0053</t>
   </si>
   <si>
     <t>["TOOL0008","TOOL0009"]</t>
+  </si>
+  <si>
+    <t>TSET0054</t>
   </si>
   <si>
     <t>BCAT0001</t>
@@ -2105,1242 +2159,1242 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>280</v>
+        <v>298</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>281</v>
+        <v>299</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>26</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>282</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>283</v>
+        <v>301</v>
       </c>
       <c r="B2" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E2" t="s">
-        <v>285</v>
+        <v>303</v>
       </c>
       <c r="F2" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>286</v>
+        <v>304</v>
       </c>
       <c r="B3" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E3" t="s">
-        <v>288</v>
+        <v>306</v>
       </c>
       <c r="F3" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>289</v>
+        <v>307</v>
       </c>
       <c r="B4" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E4" t="s">
-        <v>290</v>
+        <v>308</v>
       </c>
       <c r="F4" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>291</v>
+        <v>309</v>
       </c>
       <c r="B5" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E5" t="s">
-        <v>292</v>
+        <v>310</v>
       </c>
       <c r="F5" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>293</v>
+        <v>311</v>
       </c>
       <c r="B6" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>294</v>
+        <v>312</v>
       </c>
       <c r="E6" t="s">
-        <v>295</v>
+        <v>313</v>
       </c>
       <c r="F6" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>296</v>
+        <v>314</v>
       </c>
       <c r="B7" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E7" t="s">
-        <v>297</v>
+        <v>315</v>
       </c>
       <c r="F7" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>298</v>
+        <v>316</v>
       </c>
       <c r="B8" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E8" t="s">
-        <v>299</v>
+        <v>317</v>
       </c>
       <c r="F8" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>300</v>
+        <v>318</v>
       </c>
       <c r="B9" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="C9">
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E9" t="s">
-        <v>301</v>
+        <v>319</v>
       </c>
       <c r="F9" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>302</v>
+        <v>320</v>
       </c>
       <c r="B10" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="C10">
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E10" t="s">
-        <v>303</v>
+        <v>321</v>
       </c>
       <c r="F10" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>304</v>
+        <v>322</v>
       </c>
       <c r="B11" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="C11">
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>294</v>
+        <v>312</v>
       </c>
       <c r="E11" t="s">
-        <v>305</v>
+        <v>323</v>
       </c>
       <c r="F11" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>306</v>
+        <v>324</v>
       </c>
       <c r="B12" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="C12">
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E12" t="s">
-        <v>307</v>
+        <v>325</v>
       </c>
       <c r="F12" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>308</v>
+        <v>326</v>
       </c>
       <c r="B13" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="C13">
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E13" t="s">
-        <v>309</v>
+        <v>327</v>
       </c>
       <c r="F13" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="B14" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="C14">
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>311</v>
+        <v>329</v>
       </c>
       <c r="E14" t="s">
-        <v>312</v>
+        <v>330</v>
       </c>
       <c r="F14" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>313</v>
+        <v>331</v>
       </c>
       <c r="B15" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="C15">
         <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E15" t="s">
-        <v>314</v>
+        <v>332</v>
       </c>
       <c r="F15" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>315</v>
+        <v>333</v>
       </c>
       <c r="B16" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="C16">
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E16" t="s">
-        <v>316</v>
+        <v>334</v>
       </c>
       <c r="F16" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>317</v>
+        <v>335</v>
       </c>
       <c r="B17" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E17" t="s">
-        <v>318</v>
+        <v>336</v>
       </c>
       <c r="F17" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>319</v>
+        <v>337</v>
       </c>
       <c r="B18" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C18">
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E18" t="s">
-        <v>320</v>
+        <v>338</v>
       </c>
       <c r="F18" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>321</v>
+        <v>339</v>
       </c>
       <c r="B19" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E19" t="s">
-        <v>322</v>
+        <v>340</v>
       </c>
       <c r="F19" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>323</v>
+        <v>341</v>
       </c>
       <c r="B20" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C20">
         <v>4</v>
       </c>
       <c r="D20" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E20" t="s">
-        <v>324</v>
+        <v>342</v>
       </c>
       <c r="F20" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>325</v>
+        <v>343</v>
       </c>
       <c r="B21" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C21">
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E21" t="s">
-        <v>326</v>
+        <v>344</v>
       </c>
       <c r="F21" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="B22" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C22">
         <v>6</v>
       </c>
       <c r="D22" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E22" t="s">
-        <v>328</v>
+        <v>346</v>
       </c>
       <c r="F22" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>329</v>
+        <v>347</v>
       </c>
       <c r="B23" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C23">
         <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E23" t="s">
-        <v>330</v>
+        <v>348</v>
       </c>
       <c r="F23" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>331</v>
+        <v>349</v>
       </c>
       <c r="B24" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C24">
         <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E24" t="s">
-        <v>332</v>
+        <v>350</v>
       </c>
       <c r="F24" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>333</v>
+        <v>351</v>
       </c>
       <c r="B25" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C25">
         <v>9</v>
       </c>
       <c r="D25" t="s">
-        <v>294</v>
+        <v>312</v>
       </c>
       <c r="E25" t="s">
-        <v>334</v>
+        <v>352</v>
       </c>
       <c r="F25" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>335</v>
+        <v>353</v>
       </c>
       <c r="B26" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C26">
         <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E26" t="s">
-        <v>336</v>
+        <v>354</v>
       </c>
       <c r="F26" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="B27" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C27">
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E27" t="s">
-        <v>338</v>
+        <v>356</v>
       </c>
       <c r="F27" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="B28" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C28">
         <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>311</v>
+        <v>329</v>
       </c>
       <c r="E28" t="s">
-        <v>340</v>
+        <v>358</v>
       </c>
       <c r="F28" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>341</v>
+        <v>359</v>
       </c>
       <c r="B29" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E29" t="s">
-        <v>342</v>
+        <v>360</v>
       </c>
       <c r="F29" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>343</v>
+        <v>361</v>
       </c>
       <c r="B30" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="C30">
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E30" t="s">
-        <v>344</v>
+        <v>362</v>
       </c>
       <c r="F30" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>345</v>
+        <v>363</v>
       </c>
       <c r="B31" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="C31">
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E31" t="s">
-        <v>346</v>
+        <v>364</v>
       </c>
       <c r="F31" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>347</v>
+        <v>365</v>
       </c>
       <c r="B32" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="C32">
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E32" t="s">
-        <v>348</v>
+        <v>366</v>
       </c>
       <c r="F32" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>349</v>
+        <v>367</v>
       </c>
       <c r="B33" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="C33">
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E33" t="s">
-        <v>350</v>
+        <v>368</v>
       </c>
       <c r="F33" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>351</v>
+        <v>369</v>
       </c>
       <c r="B34" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="C34">
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E34" t="s">
-        <v>352</v>
+        <v>370</v>
       </c>
       <c r="F34" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>353</v>
+        <v>371</v>
       </c>
       <c r="B35" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="C35">
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E35" t="s">
-        <v>354</v>
+        <v>372</v>
       </c>
       <c r="F35" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>355</v>
+        <v>373</v>
       </c>
       <c r="B36" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="C36">
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E36" t="s">
-        <v>356</v>
+        <v>374</v>
       </c>
       <c r="F36" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>357</v>
+        <v>375</v>
       </c>
       <c r="B37" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="C37">
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E37" t="s">
-        <v>358</v>
+        <v>376</v>
       </c>
       <c r="F37" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>359</v>
+        <v>377</v>
       </c>
       <c r="B38" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="C38">
         <v>10</v>
       </c>
       <c r="D38" t="s">
-        <v>294</v>
+        <v>312</v>
       </c>
       <c r="E38" t="s">
-        <v>360</v>
+        <v>378</v>
       </c>
       <c r="F38" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>361</v>
+        <v>379</v>
       </c>
       <c r="B39" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="C39">
         <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E39" t="s">
-        <v>362</v>
+        <v>380</v>
       </c>
       <c r="F39" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>363</v>
+        <v>381</v>
       </c>
       <c r="B40" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="C40">
         <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>311</v>
+        <v>329</v>
       </c>
       <c r="E40" t="s">
-        <v>364</v>
+        <v>382</v>
       </c>
       <c r="F40" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>365</v>
+        <v>383</v>
       </c>
       <c r="B41" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C41">
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E41" t="s">
-        <v>366</v>
+        <v>384</v>
       </c>
       <c r="F41" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>367</v>
+        <v>385</v>
       </c>
       <c r="B42" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C42">
         <v>2</v>
       </c>
       <c r="D42" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E42" t="s">
-        <v>368</v>
+        <v>386</v>
       </c>
       <c r="F42" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>369</v>
+        <v>387</v>
       </c>
       <c r="B43" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C43">
         <v>3</v>
       </c>
       <c r="D43" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E43" t="s">
-        <v>370</v>
+        <v>388</v>
       </c>
       <c r="F43" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>371</v>
+        <v>389</v>
       </c>
       <c r="B44" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C44">
         <v>4</v>
       </c>
       <c r="D44" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E44" t="s">
-        <v>372</v>
+        <v>390</v>
       </c>
       <c r="F44" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>373</v>
+        <v>391</v>
       </c>
       <c r="B45" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C45">
         <v>5</v>
       </c>
       <c r="D45" t="s">
-        <v>294</v>
+        <v>312</v>
       </c>
       <c r="E45" t="s">
-        <v>374</v>
+        <v>392</v>
       </c>
       <c r="F45" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>375</v>
+        <v>393</v>
       </c>
       <c r="B46" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C46">
         <v>6</v>
       </c>
       <c r="D46" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E46" t="s">
-        <v>376</v>
+        <v>394</v>
       </c>
       <c r="F46" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>377</v>
+        <v>395</v>
       </c>
       <c r="B47" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C47">
         <v>7</v>
       </c>
       <c r="D47" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E47" t="s">
-        <v>378</v>
+        <v>396</v>
       </c>
       <c r="F47" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>379</v>
+        <v>397</v>
       </c>
       <c r="B48" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C48">
         <v>8</v>
       </c>
       <c r="D48" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E48" t="s">
-        <v>380</v>
+        <v>398</v>
       </c>
       <c r="F48" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>381</v>
+        <v>399</v>
       </c>
       <c r="B49" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C49">
         <v>9</v>
       </c>
       <c r="D49" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E49" t="s">
-        <v>382</v>
+        <v>400</v>
       </c>
       <c r="F49" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>383</v>
+        <v>401</v>
       </c>
       <c r="B50" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C50">
         <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E50" t="s">
-        <v>384</v>
+        <v>402</v>
       </c>
       <c r="F50" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>385</v>
+        <v>403</v>
       </c>
       <c r="B51" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C51">
         <v>11</v>
       </c>
       <c r="D51" t="s">
-        <v>294</v>
+        <v>312</v>
       </c>
       <c r="E51" t="s">
-        <v>386</v>
+        <v>404</v>
       </c>
       <c r="F51" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>387</v>
+        <v>405</v>
       </c>
       <c r="B52" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C52">
         <v>12</v>
       </c>
       <c r="D52" t="s">
-        <v>311</v>
+        <v>329</v>
       </c>
       <c r="E52" t="s">
-        <v>388</v>
+        <v>406</v>
       </c>
       <c r="F52" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>389</v>
+        <v>407</v>
       </c>
       <c r="B53" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="C53">
         <v>1</v>
       </c>
       <c r="D53" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E53" t="s">
-        <v>390</v>
+        <v>408</v>
       </c>
       <c r="F53" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>391</v>
+        <v>409</v>
       </c>
       <c r="B54" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="C54">
         <v>2</v>
       </c>
       <c r="D54" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E54" t="s">
-        <v>392</v>
+        <v>410</v>
       </c>
       <c r="F54" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>393</v>
+        <v>411</v>
       </c>
       <c r="B55" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="C55">
         <v>3</v>
       </c>
       <c r="D55" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E55" t="s">
-        <v>394</v>
+        <v>412</v>
       </c>
       <c r="F55" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>395</v>
+        <v>413</v>
       </c>
       <c r="B56" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="C56">
         <v>4</v>
       </c>
       <c r="D56" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E56" t="s">
-        <v>396</v>
+        <v>414</v>
       </c>
       <c r="F56" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>397</v>
+        <v>415</v>
       </c>
       <c r="B57" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="C57">
         <v>5</v>
       </c>
       <c r="D57" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E57" t="s">
-        <v>398</v>
+        <v>416</v>
       </c>
       <c r="F57" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>399</v>
+        <v>417</v>
       </c>
       <c r="B58" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="C58">
         <v>6</v>
       </c>
       <c r="D58" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E58" t="s">
-        <v>400</v>
+        <v>418</v>
       </c>
       <c r="F58" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>401</v>
+        <v>419</v>
       </c>
       <c r="B59" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="C59">
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>294</v>
+        <v>312</v>
       </c>
       <c r="E59" t="s">
-        <v>402</v>
+        <v>420</v>
       </c>
       <c r="F59" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>403</v>
+        <v>421</v>
       </c>
       <c r="B60" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="C60">
         <v>8</v>
       </c>
       <c r="D60" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="E60" t="s">
-        <v>404</v>
+        <v>422</v>
       </c>
       <c r="F60" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>405</v>
+        <v>423</v>
       </c>
       <c r="B61" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="C61">
         <v>9</v>
       </c>
       <c r="D61" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
       <c r="E61" t="s">
-        <v>406</v>
+        <v>424</v>
       </c>
       <c r="F61" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>407</v>
+        <v>425</v>
       </c>
       <c r="B62" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="C62">
         <v>10</v>
       </c>
       <c r="D62" t="s">
-        <v>311</v>
+        <v>329</v>
       </c>
       <c r="E62" t="s">
-        <v>408</v>
+        <v>426</v>
       </c>
       <c r="F62" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -3360,7 +3414,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>409</v>
+        <v>427</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>72</v>
@@ -3371,68 +3425,68 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>410</v>
+        <v>428</v>
       </c>
       <c r="B2" t="s">
-        <v>411</v>
+        <v>429</v>
       </c>
       <c r="C2" t="s">
-        <v>412</v>
+        <v>430</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>413</v>
+        <v>431</v>
       </c>
       <c r="B3" t="s">
-        <v>414</v>
+        <v>432</v>
       </c>
       <c r="C3" t="s">
-        <v>415</v>
+        <v>433</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>416</v>
+        <v>434</v>
       </c>
       <c r="B4" t="s">
-        <v>417</v>
+        <v>435</v>
       </c>
       <c r="C4" t="s">
-        <v>418</v>
+        <v>436</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>419</v>
+        <v>437</v>
       </c>
       <c r="B5" t="s">
-        <v>420</v>
+        <v>438</v>
       </c>
       <c r="C5" t="s">
-        <v>421</v>
+        <v>439</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>422</v>
+        <v>440</v>
       </c>
       <c r="B6" t="s">
-        <v>423</v>
+        <v>441</v>
       </c>
       <c r="C6" t="s">
-        <v>424</v>
+        <v>442</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>425</v>
+        <v>443</v>
       </c>
       <c r="B7" t="s">
-        <v>426</v>
+        <v>444</v>
       </c>
       <c r="C7" t="s">
-        <v>427</v>
+        <v>445</v>
       </c>
     </row>
   </sheetData>
@@ -3452,123 +3506,123 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>428</v>
+        <v>446</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>409</v>
+        <v>427</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>429</v>
+        <v>447</v>
       </c>
       <c r="B2" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="C2" t="s">
-        <v>410</v>
+        <v>428</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>430</v>
+        <v>448</v>
       </c>
       <c r="B3" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="C3" t="s">
-        <v>413</v>
+        <v>431</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>431</v>
+        <v>449</v>
       </c>
       <c r="B4" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="C4" t="s">
-        <v>416</v>
+        <v>434</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>432</v>
+        <v>450</v>
       </c>
       <c r="B5" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="C5" t="s">
-        <v>425</v>
+        <v>443</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>433</v>
+        <v>451</v>
       </c>
       <c r="B6" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C6" t="s">
-        <v>419</v>
+        <v>437</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>434</v>
+        <v>452</v>
       </c>
       <c r="B7" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C7" t="s">
-        <v>413</v>
+        <v>431</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>435</v>
+        <v>453</v>
       </c>
       <c r="B8" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="C8" t="s">
-        <v>422</v>
+        <v>440</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>436</v>
+        <v>454</v>
       </c>
       <c r="B9" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="C9" t="s">
-        <v>413</v>
+        <v>431</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>437</v>
+        <v>455</v>
       </c>
       <c r="B10" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="C10" t="s">
-        <v>425</v>
+        <v>443</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>438</v>
+        <v>456</v>
       </c>
       <c r="B11" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="C11" t="s">
-        <v>425</v>
+        <v>443</v>
       </c>
     </row>
   </sheetData>
@@ -3593,45 +3647,45 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>439</v>
+        <v>457</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>440</v>
+        <v>458</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>441</v>
+        <v>459</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>443</v>
+        <v>461</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>444</v>
+        <v>462</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>445</v>
+        <v>463</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>446</v>
+        <v>464</v>
       </c>
       <c r="B2" t="s">
-        <v>447</v>
+        <v>465</v>
       </c>
       <c r="C2" t="s">
         <v>105</v>
       </c>
       <c r="D2" t="s">
-        <v>448</v>
+        <v>466</v>
       </c>
       <c r="E2" t="s">
-        <v>449</v>
+        <v>467</v>
       </c>
       <c r="F2" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
       <c r="G2" t="b">
         <v>0</v>
@@ -3639,22 +3693,22 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>450</v>
+        <v>468</v>
       </c>
       <c r="B3" t="s">
-        <v>451</v>
+        <v>469</v>
       </c>
       <c r="C3" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="D3" t="s">
-        <v>452</v>
+        <v>470</v>
       </c>
       <c r="E3" t="s">
-        <v>453</v>
+        <v>471</v>
       </c>
       <c r="F3" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
       <c r="G3" t="b">
         <v>0</v>
@@ -3662,22 +3716,22 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>454</v>
+        <v>472</v>
       </c>
       <c r="B4" t="s">
-        <v>451</v>
+        <v>469</v>
       </c>
       <c r="C4" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="D4" t="s">
-        <v>256</v>
+        <v>274</v>
       </c>
       <c r="E4" t="s">
-        <v>455</v>
+        <v>473</v>
       </c>
       <c r="F4" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
       <c r="G4" t="b">
         <v>0</v>
@@ -3685,22 +3739,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>456</v>
+        <v>474</v>
       </c>
       <c r="B5" t="s">
-        <v>451</v>
+        <v>469</v>
       </c>
       <c r="C5" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="D5" t="s">
-        <v>261</v>
+        <v>279</v>
       </c>
       <c r="E5" t="s">
-        <v>457</v>
+        <v>475</v>
       </c>
       <c r="F5" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
       <c r="G5" t="b">
         <v>0</v>
@@ -3708,22 +3762,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>458</v>
+        <v>476</v>
       </c>
       <c r="B6" t="s">
-        <v>451</v>
+        <v>469</v>
       </c>
       <c r="C6" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="D6" t="s">
-        <v>459</v>
+        <v>477</v>
       </c>
       <c r="E6" t="s">
-        <v>460</v>
+        <v>478</v>
       </c>
       <c r="F6" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
       <c r="G6" t="b">
         <v>0</v>
@@ -3731,22 +3785,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>461</v>
+        <v>479</v>
       </c>
       <c r="B7" t="s">
-        <v>451</v>
+        <v>469</v>
       </c>
       <c r="C7" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="D7" t="s">
-        <v>271</v>
+        <v>289</v>
       </c>
       <c r="E7" t="s">
-        <v>462</v>
+        <v>480</v>
       </c>
       <c r="F7" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
       <c r="G7" t="b">
         <v>0</v>
@@ -3754,22 +3808,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>463</v>
+        <v>481</v>
       </c>
       <c r="B8" t="s">
-        <v>451</v>
+        <v>469</v>
       </c>
       <c r="C8" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="D8" t="s">
-        <v>276</v>
+        <v>294</v>
       </c>
       <c r="E8" t="s">
-        <v>464</v>
+        <v>482</v>
       </c>
       <c r="F8" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
       <c r="G8" t="b">
         <v>0</v>
@@ -3777,10 +3831,10 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>465</v>
+        <v>483</v>
       </c>
       <c r="B9" t="s">
-        <v>466</v>
+        <v>484</v>
       </c>
       <c r="C9" t="s">
         <v>28</v>
@@ -3789,10 +3843,10 @@
         <v>30</v>
       </c>
       <c r="E9" t="s">
-        <v>467</v>
+        <v>485</v>
       </c>
       <c r="F9" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
       <c r="G9" t="b">
         <v>0</v>
@@ -3816,70 +3870,70 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>468</v>
+        <v>486</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>469</v>
+        <v>487</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>470</v>
+        <v>488</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>471</v>
+        <v>489</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>472</v>
+        <v>490</v>
       </c>
       <c r="B2" t="s">
-        <v>473</v>
+        <v>491</v>
       </c>
       <c r="C2" t="s">
-        <v>474</v>
+        <v>492</v>
       </c>
       <c r="D2" t="b">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>475</v>
+        <v>493</v>
       </c>
       <c r="B3" t="s">
-        <v>476</v>
+        <v>494</v>
       </c>
       <c r="C3" t="s">
-        <v>447</v>
+        <v>465</v>
       </c>
       <c r="D3" t="b">
         <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>477</v>
+        <v>495</v>
       </c>
       <c r="B4" t="s">
-        <v>478</v>
+        <v>496</v>
       </c>
       <c r="C4" t="s">
-        <v>479</v>
+        <v>497</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -3902,16 +3956,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>480</v>
+        <v>498</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>481</v>
+        <v>499</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>482</v>
+        <v>500</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>483</v>
+        <v>501</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>51</v>
@@ -3919,16 +3973,16 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>484</v>
+        <v>502</v>
       </c>
       <c r="B2" t="s">
-        <v>485</v>
+        <v>503</v>
       </c>
       <c r="C2" t="s">
-        <v>486</v>
+        <v>504</v>
       </c>
       <c r="D2" t="s">
-        <v>487</v>
+        <v>505</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -3962,7 +4016,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>488</v>
+        <v>506</v>
       </c>
       <c r="B2" t="s">
         <v>136</v>
@@ -4712,7 +4766,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -4879,47 +4933,47 @@
         <v>160</v>
       </c>
       <c r="B10" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C10" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E10" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B11" t="s">
         <v>97</v>
       </c>
       <c r="C11" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D11" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E11" t="s">
-        <v>153</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B12" t="s">
         <v>97</v>
       </c>
       <c r="C12" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D12" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E12" t="s">
         <v>153</v>
@@ -4927,16 +4981,16 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B13" t="s">
         <v>97</v>
       </c>
       <c r="C13" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D13" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E13" t="s">
         <v>153</v>
@@ -4944,33 +4998,33 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B14" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C14" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="D14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E14" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B15" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C15" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="D15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E15" t="s">
         <v>153</v>
@@ -4978,33 +5032,33 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B16" t="s">
         <v>101</v>
       </c>
       <c r="C16" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="D16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E16" t="s">
-        <v>153</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B17" t="s">
         <v>101</v>
       </c>
       <c r="C17" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="D17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E17" t="s">
         <v>153</v>
@@ -5012,33 +5066,33 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B18" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C18" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="D18" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E18" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B19" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C19" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="D19" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E19" t="s">
         <v>153</v>
@@ -5046,16 +5100,16 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B20" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C20" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="D20" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="E20" t="s">
         <v>153</v>
@@ -5069,13 +5123,13 @@
         <v>105</v>
       </c>
       <c r="C21" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="D21" t="s">
         <v>183</v>
       </c>
       <c r="E21" t="s">
-        <v>153</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -5083,16 +5137,16 @@
         <v>184</v>
       </c>
       <c r="B22" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C22" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D22" t="s">
         <v>185</v>
       </c>
       <c r="E22" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -5100,10 +5154,10 @@
         <v>186</v>
       </c>
       <c r="B23" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C23" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D23" t="s">
         <v>187</v>
@@ -5117,10 +5171,10 @@
         <v>188</v>
       </c>
       <c r="B24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C24" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D24" t="s">
         <v>189</v>
@@ -5134,10 +5188,10 @@
         <v>190</v>
       </c>
       <c r="B25" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C25" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D25" t="s">
         <v>191</v>
@@ -5151,7 +5205,7 @@
         <v>192</v>
       </c>
       <c r="B26" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C26" t="s">
         <v>148</v>
@@ -5168,7 +5222,7 @@
         <v>194</v>
       </c>
       <c r="B27" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C27" t="s">
         <v>151</v>
@@ -5185,7 +5239,7 @@
         <v>196</v>
       </c>
       <c r="B28" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C28" t="s">
         <v>155</v>
@@ -5202,7 +5256,7 @@
         <v>198</v>
       </c>
       <c r="B29" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C29" t="s">
         <v>158</v>
@@ -5219,16 +5273,16 @@
         <v>200</v>
       </c>
       <c r="B30" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C30" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D30" t="s">
         <v>201</v>
       </c>
       <c r="E30" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -5236,16 +5290,16 @@
         <v>202</v>
       </c>
       <c r="B31" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C31" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D31" t="s">
         <v>203</v>
       </c>
       <c r="E31" t="s">
-        <v>153</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -5253,10 +5307,10 @@
         <v>204</v>
       </c>
       <c r="B32" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C32" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D32" t="s">
         <v>205</v>
@@ -5270,10 +5324,10 @@
         <v>206</v>
       </c>
       <c r="B33" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C33" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D33" t="s">
         <v>207</v>
@@ -5287,16 +5341,16 @@
         <v>208</v>
       </c>
       <c r="B34" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="C34" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="D34" t="s">
         <v>209</v>
       </c>
       <c r="E34" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -5304,10 +5358,10 @@
         <v>210</v>
       </c>
       <c r="B35" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="C35" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="D35" t="s">
         <v>211</v>
@@ -5321,16 +5375,16 @@
         <v>212</v>
       </c>
       <c r="B36" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C36" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="D36" t="s">
         <v>213</v>
       </c>
       <c r="E36" t="s">
-        <v>153</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -5338,10 +5392,10 @@
         <v>214</v>
       </c>
       <c r="B37" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C37" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="D37" t="s">
         <v>215</v>
@@ -5355,16 +5409,16 @@
         <v>216</v>
       </c>
       <c r="B38" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="C38" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="D38" t="s">
         <v>217</v>
       </c>
       <c r="E38" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -5372,10 +5426,10 @@
         <v>218</v>
       </c>
       <c r="B39" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="C39" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="D39" t="s">
         <v>219</v>
@@ -5389,13 +5443,13 @@
         <v>220</v>
       </c>
       <c r="B40" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="C40" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="D40" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="E40" t="s">
         <v>153</v>
@@ -5403,50 +5457,50 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>221</v>
+      </c>
+      <c r="B41" t="s">
+        <v>121</v>
+      </c>
+      <c r="C41" t="s">
+        <v>148</v>
+      </c>
+      <c r="D41" t="s">
         <v>222</v>
       </c>
-      <c r="B41" t="s">
-        <v>125</v>
-      </c>
-      <c r="C41" t="s">
-        <v>158</v>
-      </c>
-      <c r="D41" t="s">
-        <v>223</v>
-      </c>
       <c r="E41" t="s">
-        <v>153</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>223</v>
+      </c>
+      <c r="B42" t="s">
+        <v>121</v>
+      </c>
+      <c r="C42" t="s">
+        <v>151</v>
+      </c>
+      <c r="D42" t="s">
         <v>224</v>
       </c>
-      <c r="B42" t="s">
-        <v>129</v>
-      </c>
-      <c r="C42" t="s">
-        <v>148</v>
-      </c>
-      <c r="D42" t="s">
-        <v>225</v>
-      </c>
       <c r="E42" t="s">
-        <v>6</v>
+        <v>153</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>225</v>
+      </c>
+      <c r="B43" t="s">
+        <v>121</v>
+      </c>
+      <c r="C43" t="s">
+        <v>155</v>
+      </c>
+      <c r="D43" t="s">
         <v>226</v>
-      </c>
-      <c r="B43" t="s">
-        <v>129</v>
-      </c>
-      <c r="C43" t="s">
-        <v>151</v>
-      </c>
-      <c r="D43" t="s">
-        <v>227</v>
       </c>
       <c r="E43" t="s">
         <v>153</v>
@@ -5454,16 +5508,16 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>227</v>
+      </c>
+      <c r="B44" t="s">
+        <v>121</v>
+      </c>
+      <c r="C44" t="s">
+        <v>158</v>
+      </c>
+      <c r="D44" t="s">
         <v>228</v>
-      </c>
-      <c r="B44" t="s">
-        <v>129</v>
-      </c>
-      <c r="C44" t="s">
-        <v>155</v>
-      </c>
-      <c r="D44" t="s">
-        <v>229</v>
       </c>
       <c r="E44" t="s">
         <v>153</v>
@@ -5471,18 +5525,188 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>229</v>
+      </c>
+      <c r="B45" t="s">
+        <v>121</v>
+      </c>
+      <c r="C45" t="s">
+        <v>161</v>
+      </c>
+      <c r="D45" t="s">
         <v>230</v>
       </c>
-      <c r="B45" t="s">
+      <c r="E45" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>231</v>
+      </c>
+      <c r="B46" t="s">
+        <v>125</v>
+      </c>
+      <c r="C46" t="s">
+        <v>148</v>
+      </c>
+      <c r="D46" t="s">
+        <v>232</v>
+      </c>
+      <c r="E46" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>233</v>
+      </c>
+      <c r="B47" t="s">
+        <v>125</v>
+      </c>
+      <c r="C47" t="s">
+        <v>151</v>
+      </c>
+      <c r="D47" t="s">
+        <v>234</v>
+      </c>
+      <c r="E47" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>235</v>
+      </c>
+      <c r="B48" t="s">
+        <v>125</v>
+      </c>
+      <c r="C48" t="s">
+        <v>155</v>
+      </c>
+      <c r="D48" t="s">
+        <v>236</v>
+      </c>
+      <c r="E48" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>237</v>
+      </c>
+      <c r="B49" t="s">
+        <v>125</v>
+      </c>
+      <c r="C49" t="s">
+        <v>158</v>
+      </c>
+      <c r="D49" t="s">
+        <v>238</v>
+      </c>
+      <c r="E49" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>239</v>
+      </c>
+      <c r="B50" t="s">
+        <v>125</v>
+      </c>
+      <c r="C50" t="s">
+        <v>161</v>
+      </c>
+      <c r="D50" t="s">
+        <v>240</v>
+      </c>
+      <c r="E50" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>241</v>
+      </c>
+      <c r="B51" t="s">
         <v>129</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C51" t="s">
+        <v>148</v>
+      </c>
+      <c r="D51" t="s">
+        <v>242</v>
+      </c>
+      <c r="E51" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>243</v>
+      </c>
+      <c r="B52" t="s">
+        <v>129</v>
+      </c>
+      <c r="C52" t="s">
+        <v>151</v>
+      </c>
+      <c r="D52" t="s">
+        <v>244</v>
+      </c>
+      <c r="E52" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>245</v>
+      </c>
+      <c r="B53" t="s">
+        <v>129</v>
+      </c>
+      <c r="C53" t="s">
+        <v>155</v>
+      </c>
+      <c r="D53" t="s">
+        <v>246</v>
+      </c>
+      <c r="E53" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>247</v>
+      </c>
+      <c r="B54" t="s">
+        <v>129</v>
+      </c>
+      <c r="C54" t="s">
         <v>158</v>
       </c>
-      <c r="D45" t="s">
-        <v>231</v>
-      </c>
-      <c r="E45" t="s">
+      <c r="D54" t="s">
+        <v>248</v>
+      </c>
+      <c r="E54" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>249</v>
+      </c>
+      <c r="B55" t="s">
+        <v>129</v>
+      </c>
+      <c r="C55" t="s">
+        <v>161</v>
+      </c>
+      <c r="D55" t="s">
+        <v>230</v>
+      </c>
+      <c r="E55" t="s">
         <v>153</v>
       </c>
     </row>
@@ -5518,30 +5742,30 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>232</v>
+        <v>250</v>
       </c>
       <c r="B2" t="s">
-        <v>233</v>
+        <v>251</v>
       </c>
       <c r="C2" t="s">
-        <v>234</v>
+        <v>252</v>
       </c>
       <c r="D2" t="s">
-        <v>235</v>
+        <v>253</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>236</v>
+        <v>254</v>
       </c>
       <c r="B3" t="s">
-        <v>237</v>
+        <v>255</v>
       </c>
       <c r="C3" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="D3" t="s">
-        <v>239</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>
@@ -5563,30 +5787,30 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>240</v>
+        <v>258</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>241</v>
+        <v>259</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>242</v>
+        <v>260</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>243</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>244</v>
+        <v>262</v>
       </c>
       <c r="B2" t="s">
-        <v>245</v>
+        <v>263</v>
       </c>
       <c r="C2" t="s">
-        <v>246</v>
+        <v>264</v>
       </c>
       <c r="D2" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -5610,7 +5834,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>25</v>
@@ -5619,19 +5843,19 @@
         <v>24</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>249</v>
+        <v>267</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>240</v>
+        <v>258</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>27</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>250</v>
+        <v>268</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>3</v>
@@ -5639,22 +5863,22 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="B2" t="s">
-        <v>252</v>
+        <v>270</v>
       </c>
       <c r="C2" t="s">
-        <v>253</v>
+        <v>271</v>
       </c>
       <c r="D2" t="s">
-        <v>254</v>
+        <v>272</v>
       </c>
       <c r="E2" t="s">
-        <v>232</v>
+        <v>250</v>
       </c>
       <c r="F2" t="s">
-        <v>244</v>
+        <v>262</v>
       </c>
       <c r="G2" t="s">
         <v>32</v>
@@ -5668,147 +5892,147 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="B3" t="s">
-        <v>256</v>
+        <v>274</v>
       </c>
       <c r="C3" t="s">
-        <v>257</v>
+        <v>275</v>
       </c>
       <c r="D3" t="s">
-        <v>258</v>
+        <v>276</v>
       </c>
       <c r="E3" t="s">
-        <v>236</v>
+        <v>254</v>
       </c>
       <c r="F3" t="s">
-        <v>244</v>
+        <v>262</v>
       </c>
       <c r="G3" t="s">
         <v>32</v>
       </c>
       <c r="H3" t="s">
-        <v>259</v>
+        <v>277</v>
       </c>
       <c r="I3" t="s">
-        <v>259</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="B4" t="s">
-        <v>261</v>
+        <v>279</v>
       </c>
       <c r="C4" t="s">
+        <v>280</v>
+      </c>
+      <c r="D4" t="s">
+        <v>281</v>
+      </c>
+      <c r="E4" t="s">
+        <v>250</v>
+      </c>
+      <c r="F4" t="s">
         <v>262</v>
-      </c>
-      <c r="D4" t="s">
-        <v>263</v>
-      </c>
-      <c r="E4" t="s">
-        <v>232</v>
-      </c>
-      <c r="F4" t="s">
-        <v>244</v>
       </c>
       <c r="G4" t="s">
         <v>32</v>
       </c>
       <c r="H4" t="s">
-        <v>264</v>
+        <v>282</v>
       </c>
       <c r="I4" t="s">
-        <v>264</v>
+        <v>282</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="B5" t="s">
-        <v>266</v>
+        <v>284</v>
       </c>
       <c r="C5" t="s">
-        <v>267</v>
+        <v>285</v>
       </c>
       <c r="D5" t="s">
-        <v>268</v>
+        <v>286</v>
       </c>
       <c r="E5" t="s">
-        <v>232</v>
+        <v>250</v>
       </c>
       <c r="F5" t="s">
-        <v>244</v>
+        <v>262</v>
       </c>
       <c r="G5" t="s">
         <v>32</v>
       </c>
       <c r="H5" t="s">
-        <v>269</v>
+        <v>287</v>
       </c>
       <c r="I5" t="s">
-        <v>269</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="B6" t="s">
-        <v>271</v>
+        <v>289</v>
       </c>
       <c r="C6" t="s">
-        <v>272</v>
+        <v>290</v>
       </c>
       <c r="D6" t="s">
-        <v>273</v>
+        <v>291</v>
       </c>
       <c r="E6" t="s">
-        <v>236</v>
+        <v>254</v>
       </c>
       <c r="F6" t="s">
-        <v>244</v>
+        <v>262</v>
       </c>
       <c r="G6" t="s">
         <v>32</v>
       </c>
       <c r="H6" t="s">
-        <v>274</v>
+        <v>292</v>
       </c>
       <c r="I6" t="s">
-        <v>274</v>
+        <v>292</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="B7" t="s">
-        <v>276</v>
+        <v>294</v>
       </c>
       <c r="C7" t="s">
-        <v>277</v>
+        <v>295</v>
       </c>
       <c r="D7" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="E7" t="s">
-        <v>236</v>
+        <v>254</v>
       </c>
       <c r="F7" t="s">
-        <v>244</v>
+        <v>262</v>
       </c>
       <c r="G7" t="s">
         <v>32</v>
       </c>
       <c r="H7" t="s">
-        <v>279</v>
+        <v>297</v>
       </c>
       <c r="I7" t="s">
-        <v>279</v>
+        <v>297</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Analytics: GA4 behind a Measurement ID and consent, page views and tool events (T6.1)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1010" uniqueCount="509">
   <si>
     <t>setting_key</t>
   </si>
@@ -95,6 +95,12 @@
   </si>
   <si>
     <t>false</t>
+  </si>
+  <si>
+    <t>analytics_measurement_id</t>
+  </si>
+  <si>
+    <t>2026-10-30T08:39:16Z</t>
   </si>
   <si>
     <t>page_id</t>
@@ -2006,7 +2012,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -2141,9 +2147,20 @@
         <v>7</v>
       </c>
     </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2159,1247 +2176,1247 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="F2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E3" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="F3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B4" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E4" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="F4" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B5" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E5" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="F5" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B6" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E6" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="F6" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B7" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E7" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="F7" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B8" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E8" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="F8" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B9" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C9">
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E9" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="F9" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B10" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C10">
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E10" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="F10" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B11" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C11">
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E11" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="F11" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B12" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C12">
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E12" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="F12" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B13" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C13">
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E13" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="F13" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B14" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C14">
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E14" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="F14" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B15" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C15">
         <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E15" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="F15" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B16" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C16">
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E16" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="F16" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B17" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E17" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="F17" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B18" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C18">
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E18" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F18" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B19" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E19" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="F19" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B20" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C20">
         <v>4</v>
       </c>
       <c r="D20" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E20" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="F20" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B21" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C21">
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E21" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="F21" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B22" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C22">
         <v>6</v>
       </c>
       <c r="D22" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E22" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="F22" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B23" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C23">
         <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E23" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="F23" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B24" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C24">
         <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E24" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="F24" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B25" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C25">
         <v>9</v>
       </c>
       <c r="D25" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E25" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="F25" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B26" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C26">
         <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E26" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="F26" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B27" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C27">
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E27" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="F27" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B28" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C28">
         <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E28" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="F28" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B29" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E29" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="F29" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B30" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C30">
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E30" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="F30" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B31" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C31">
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E31" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="F31" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B32" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C32">
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E32" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="F32" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B33" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C33">
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E33" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="F33" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B34" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C34">
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E34" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F34" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B35" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C35">
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E35" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="F35" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B36" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C36">
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E36" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="F36" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B37" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C37">
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E37" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="F37" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B38" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C38">
         <v>10</v>
       </c>
       <c r="D38" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E38" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="F38" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B39" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C39">
         <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E39" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="F39" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B40" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C40">
         <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E40" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="F40" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B41" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C41">
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E41" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="F41" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B42" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C42">
         <v>2</v>
       </c>
       <c r="D42" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E42" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="F42" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B43" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C43">
         <v>3</v>
       </c>
       <c r="D43" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E43" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="F43" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B44" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C44">
         <v>4</v>
       </c>
       <c r="D44" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E44" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F44" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B45" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C45">
         <v>5</v>
       </c>
       <c r="D45" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E45" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F45" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B46" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C46">
         <v>6</v>
       </c>
       <c r="D46" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E46" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="F46" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B47" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C47">
         <v>7</v>
       </c>
       <c r="D47" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E47" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="F47" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B48" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C48">
         <v>8</v>
       </c>
       <c r="D48" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E48" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="F48" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B49" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C49">
         <v>9</v>
       </c>
       <c r="D49" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E49" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="F49" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B50" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C50">
         <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E50" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="F50" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B51" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C51">
         <v>11</v>
       </c>
       <c r="D51" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E51" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="F51" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B52" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C52">
         <v>12</v>
       </c>
       <c r="D52" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E52" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="F52" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B53" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C53">
         <v>1</v>
       </c>
       <c r="D53" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E53" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="F53" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B54" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C54">
         <v>2</v>
       </c>
       <c r="D54" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E54" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="F54" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B55" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C55">
         <v>3</v>
       </c>
       <c r="D55" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E55" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="F55" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B56" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C56">
         <v>4</v>
       </c>
       <c r="D56" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E56" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="F56" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B57" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C57">
         <v>5</v>
       </c>
       <c r="D57" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E57" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="F57" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B58" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C58">
         <v>6</v>
       </c>
       <c r="D58" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E58" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="F58" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B59" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C59">
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E59" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="F59" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B60" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C60">
         <v>8</v>
       </c>
       <c r="D60" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E60" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="F60" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B61" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C61">
         <v>9</v>
       </c>
       <c r="D61" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E61" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="F61" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B62" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C62">
         <v>10</v>
       </c>
       <c r="D62" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E62" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="F62" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3414,84 +3431,84 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B2" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C2" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B3" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="C3" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B4" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="C4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B5" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="C5" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B6" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C6" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B7" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="C7" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3506,128 +3523,128 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C2" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C3" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B4" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C4" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B5" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C5" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B6" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C6" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B7" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C7" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B8" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C8" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B9" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C9" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B10" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C10" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B11" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C11" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3647,45 +3664,45 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B2" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="C2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D2" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="E2" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="F2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="G2" t="b">
         <v>0</v>
@@ -3693,22 +3710,22 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B3" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="C3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D3" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="E3" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="F3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="G3" t="b">
         <v>0</v>
@@ -3716,22 +3733,22 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B4" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="C4" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D4" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E4" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="F4" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="G4" t="b">
         <v>0</v>
@@ -3739,22 +3756,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B5" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="C5" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D5" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E5" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="F5" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="G5" t="b">
         <v>0</v>
@@ -3762,22 +3779,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B6" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="C6" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="D6" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="E6" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="F6" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="G6" t="b">
         <v>0</v>
@@ -3785,22 +3802,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B7" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="C7" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D7" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="E7" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="F7" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="G7" t="b">
         <v>0</v>
@@ -3808,22 +3825,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B8" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="C8" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D8" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E8" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="F8" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="G8" t="b">
         <v>0</v>
@@ -3831,22 +3848,22 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B9" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E9" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="F9" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="G9" t="b">
         <v>0</v>
@@ -3854,7 +3871,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3870,75 +3887,75 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B2" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="C2" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="D2" t="b">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B3" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="C3" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="D3" t="b">
         <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B4" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="C4" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3956,33 +3973,33 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B2" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="C2" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="D2" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -3990,7 +4007,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4016,10 +4033,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -4027,7 +4044,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4046,19 +4063,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4066,19 +4083,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F2" t="s">
         <v>7</v>
@@ -4086,19 +4103,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F3" t="s">
         <v>7</v>
@@ -4106,19 +4123,19 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E4" t="s">
         <v>39</v>
-      </c>
-      <c r="C4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E4" t="s">
-        <v>37</v>
       </c>
       <c r="F4" t="s">
         <v>7</v>
@@ -4126,19 +4143,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s">
         <v>7</v>
@@ -4146,7 +4163,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4164,36 +4181,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -4204,16 +4221,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" t="s">
         <v>57</v>
-      </c>
-      <c r="C3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D3" t="s">
-        <v>55</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -4224,16 +4241,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -4244,16 +4261,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -4264,16 +4281,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -4284,16 +4301,16 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" t="s">
         <v>70</v>
-      </c>
-      <c r="D7" t="s">
-        <v>68</v>
       </c>
       <c r="E7">
         <v>2</v>
@@ -4304,7 +4321,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4321,36 +4338,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -4361,16 +4378,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -4381,16 +4398,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -4401,16 +4418,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -4421,7 +4438,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4441,54 +4458,54 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -4499,25 +4516,25 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H3" t="b">
         <v>0</v>
@@ -4528,25 +4545,25 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
@@ -4557,25 +4574,25 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -4586,25 +4603,25 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -4615,25 +4632,25 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="G7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
@@ -4644,25 +4661,25 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
@@ -4673,25 +4690,25 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E9" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H9" t="b">
         <v>1</v>
@@ -4702,25 +4719,25 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C10" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E10" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -4731,25 +4748,25 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C11" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E11" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H11" t="b">
         <v>0</v>
@@ -4760,7 +4777,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4777,10 +4794,10 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -4794,50 +4811,50 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C3" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" t="s">
+        <v>142</v>
+      </c>
+      <c r="E3" t="s">
         <v>139</v>
-      </c>
-      <c r="D3" t="s">
-        <v>140</v>
-      </c>
-      <c r="E3" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C4" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E4" t="s">
         <v>6</v>
@@ -4845,33 +4862,33 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E6" t="s">
         <v>6</v>
@@ -4879,84 +4896,84 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C7" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D7" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C8" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" t="s">
+        <v>158</v>
+      </c>
+      <c r="E8" t="s">
         <v>155</v>
-      </c>
-      <c r="D8" t="s">
-        <v>156</v>
-      </c>
-      <c r="E8" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B9" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C9" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D9" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E9" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B10" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C10" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D10" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E10" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B11" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D11" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E11" t="s">
         <v>6</v>
@@ -4964,84 +4981,84 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B12" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C12" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D12" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E12" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C13" t="s">
+        <v>157</v>
+      </c>
+      <c r="D13" t="s">
+        <v>170</v>
+      </c>
+      <c r="E13" t="s">
         <v>155</v>
-      </c>
-      <c r="D13" t="s">
-        <v>168</v>
-      </c>
-      <c r="E13" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B14" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C14" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D14" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E14" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B15" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C15" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D15" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E15" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C16" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D16" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E16" t="s">
         <v>6</v>
@@ -5049,84 +5066,84 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B17" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C17" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D17" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E17" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B18" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C18" t="s">
+        <v>157</v>
+      </c>
+      <c r="D18" t="s">
+        <v>180</v>
+      </c>
+      <c r="E18" t="s">
         <v>155</v>
-      </c>
-      <c r="D18" t="s">
-        <v>178</v>
-      </c>
-      <c r="E18" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B19" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C19" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D19" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E19" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B20" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C20" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D20" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E20" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B21" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C21" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D21" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E21" t="s">
         <v>6</v>
@@ -5134,84 +5151,84 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B22" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C22" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D22" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E22" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B23" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C23" t="s">
+        <v>157</v>
+      </c>
+      <c r="D23" t="s">
+        <v>189</v>
+      </c>
+      <c r="E23" t="s">
         <v>155</v>
-      </c>
-      <c r="D23" t="s">
-        <v>187</v>
-      </c>
-      <c r="E23" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B24" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C24" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D24" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E24" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B25" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C25" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D25" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E25" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B26" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C26" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D26" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E26" t="s">
         <v>6</v>
@@ -5219,84 +5236,84 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B27" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C27" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D27" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E27" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B28" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C28" t="s">
+        <v>157</v>
+      </c>
+      <c r="D28" t="s">
+        <v>199</v>
+      </c>
+      <c r="E28" t="s">
         <v>155</v>
-      </c>
-      <c r="D28" t="s">
-        <v>197</v>
-      </c>
-      <c r="E28" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B29" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C29" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D29" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E29" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B30" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C30" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D30" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E30" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B31" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C31" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D31" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E31" t="s">
         <v>6</v>
@@ -5304,84 +5321,84 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B32" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C32" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D32" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E32" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B33" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C33" t="s">
+        <v>157</v>
+      </c>
+      <c r="D33" t="s">
+        <v>209</v>
+      </c>
+      <c r="E33" t="s">
         <v>155</v>
-      </c>
-      <c r="D33" t="s">
-        <v>207</v>
-      </c>
-      <c r="E33" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B34" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C34" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D34" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E34" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B35" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C35" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D35" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="E35" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B36" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C36" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D36" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="E36" t="s">
         <v>6</v>
@@ -5389,84 +5406,84 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B37" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C37" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D37" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E37" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B38" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C38" t="s">
+        <v>157</v>
+      </c>
+      <c r="D38" t="s">
+        <v>219</v>
+      </c>
+      <c r="E38" t="s">
         <v>155</v>
-      </c>
-      <c r="D38" t="s">
-        <v>217</v>
-      </c>
-      <c r="E38" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B39" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C39" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D39" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E39" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B40" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C40" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D40" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="E40" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B41" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C41" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D41" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E41" t="s">
         <v>6</v>
@@ -5474,84 +5491,84 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B42" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C42" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D42" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E42" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B43" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C43" t="s">
+        <v>157</v>
+      </c>
+      <c r="D43" t="s">
+        <v>228</v>
+      </c>
+      <c r="E43" t="s">
         <v>155</v>
-      </c>
-      <c r="D43" t="s">
-        <v>226</v>
-      </c>
-      <c r="E43" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B44" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C44" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D44" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E44" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B45" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C45" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D45" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E45" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B46" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C46" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D46" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E46" t="s">
         <v>6</v>
@@ -5559,84 +5576,84 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B47" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C47" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D47" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E47" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B48" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C48" t="s">
+        <v>157</v>
+      </c>
+      <c r="D48" t="s">
+        <v>238</v>
+      </c>
+      <c r="E48" t="s">
         <v>155</v>
-      </c>
-      <c r="D48" t="s">
-        <v>236</v>
-      </c>
-      <c r="E48" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B49" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C49" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D49" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E49" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B50" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C50" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D50" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E50" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B51" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C51" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D51" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E51" t="s">
         <v>6</v>
@@ -5644,75 +5661,75 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B52" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C52" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D52" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E52" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B53" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C53" t="s">
+        <v>157</v>
+      </c>
+      <c r="D53" t="s">
+        <v>248</v>
+      </c>
+      <c r="E53" t="s">
         <v>155</v>
-      </c>
-      <c r="D53" t="s">
-        <v>246</v>
-      </c>
-      <c r="E53" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B54" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C54" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D54" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E54" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B55" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C55" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D55" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E55" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -5728,49 +5745,49 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B2" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="D2" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B3" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C3" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D3" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -5787,35 +5804,35 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B2" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -5834,28 +5851,28 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>3</v>
@@ -5863,25 +5880,25 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B2" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D2" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E2" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F2" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="G2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H2" t="s">
         <v>7</v>
@@ -5892,151 +5909,151 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B3" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D3" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F3" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="G3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H3" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="I3" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B4" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C4" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D4" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E4" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F4" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="G4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H4" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I4" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B5" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C5" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="E5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F5" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="G5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H5" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="I5" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B6" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C6" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D6" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F6" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="G6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H6" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="I6" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B7" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C7" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D7" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E7" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F7" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="G7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H7" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="I7" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Admin dashboard: analytics status and link to the reports (T6.4)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1010" uniqueCount="509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="511">
   <si>
     <t>setting_key</t>
   </si>
@@ -101,6 +101,12 @@
   </si>
   <si>
     <t>2026-10-30T08:39:16Z</t>
+  </si>
+  <si>
+    <t>analytics_dashboard_url</t>
+  </si>
+  <si>
+    <t>2026-10-30T10:15:15Z</t>
   </si>
   <si>
     <t>page_id</t>
@@ -2012,7 +2018,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -2156,6 +2162,17 @@
       </c>
       <c r="D10" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -2176,1242 +2193,1242 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E2" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="F2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B3" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E3" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="F3" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B4" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E4" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="F4" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B5" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E5" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="F5" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B6" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E6" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="F6" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B7" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E7" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="F7" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B8" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E8" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="F8" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B9" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C9">
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E9" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="F9" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B10" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C10">
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E10" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="F10" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B11" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C11">
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E11" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="F11" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B12" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C12">
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E12" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="F12" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B13" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C13">
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E13" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="F13" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B14" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C14">
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E14" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="F14" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B15" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C15">
         <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E15" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="F15" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B16" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C16">
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E16" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="F16" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B17" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E17" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F17" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C18">
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E18" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="F18" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B19" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E19" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="F19" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B20" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C20">
         <v>4</v>
       </c>
       <c r="D20" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E20" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="F20" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B21" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C21">
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E21" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="F21" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B22" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C22">
         <v>6</v>
       </c>
       <c r="D22" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E22" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="F22" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B23" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C23">
         <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E23" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="F23" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B24" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C24">
         <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E24" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="F24" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B25" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C25">
         <v>9</v>
       </c>
       <c r="D25" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E25" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="F25" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B26" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C26">
         <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E26" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="F26" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B27" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C27">
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E27" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="F27" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B28" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C28">
         <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E28" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="F28" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B29" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E29" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="F29" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B30" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C30">
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E30" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="F30" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B31" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C31">
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E31" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="F31" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B32" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C32">
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E32" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="F32" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B33" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C33">
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E33" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F33" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B34" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C34">
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E34" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="F34" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B35" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C35">
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E35" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="F35" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B36" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C36">
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E36" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="F36" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B37" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C37">
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E37" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="F37" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B38" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C38">
         <v>10</v>
       </c>
       <c r="D38" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E38" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="F38" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B39" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C39">
         <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E39" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="F39" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B40" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C40">
         <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E40" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="F40" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B41" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C41">
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E41" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="F41" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B42" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C42">
         <v>2</v>
       </c>
       <c r="D42" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E42" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="F42" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B43" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C43">
         <v>3</v>
       </c>
       <c r="D43" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E43" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F43" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B44" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C44">
         <v>4</v>
       </c>
       <c r="D44" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E44" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F44" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B45" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C45">
         <v>5</v>
       </c>
       <c r="D45" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E45" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="F45" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B46" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C46">
         <v>6</v>
       </c>
       <c r="D46" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E46" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="F46" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B47" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C47">
         <v>7</v>
       </c>
       <c r="D47" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E47" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="F47" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B48" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C48">
         <v>8</v>
       </c>
       <c r="D48" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E48" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="F48" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B49" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C49">
         <v>9</v>
       </c>
       <c r="D49" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E49" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="F49" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B50" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C50">
         <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E50" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="F50" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B51" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C51">
         <v>11</v>
       </c>
       <c r="D51" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E51" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="F51" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B52" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C52">
         <v>12</v>
       </c>
       <c r="D52" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E52" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="F52" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B53" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C53">
         <v>1</v>
       </c>
       <c r="D53" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E53" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="F53" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B54" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C54">
         <v>2</v>
       </c>
       <c r="D54" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E54" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="F54" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B55" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C55">
         <v>3</v>
       </c>
       <c r="D55" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E55" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="F55" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B56" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C56">
         <v>4</v>
       </c>
       <c r="D56" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E56" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="F56" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B57" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C57">
         <v>5</v>
       </c>
       <c r="D57" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E57" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="F57" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B58" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C58">
         <v>6</v>
       </c>
       <c r="D58" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E58" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="F58" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B59" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C59">
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E59" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="F59" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B60" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C60">
         <v>8</v>
       </c>
       <c r="D60" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E60" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="F60" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B61" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C61">
         <v>9</v>
       </c>
       <c r="D61" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E61" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="F61" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B62" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C62">
         <v>10</v>
       </c>
       <c r="D62" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E62" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="F62" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -3431,79 +3448,79 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B2" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="C2" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B3" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="C3" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B4" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="C4" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B5" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="C5" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B6" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C6" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B7" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="C7" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
     </row>
   </sheetData>
@@ -3523,123 +3540,123 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C2" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B3" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C3" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B4" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B5" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C5" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B6" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C6" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B7" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C7" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B8" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C8" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B9" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C9" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B10" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C10" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B11" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C11" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
     </row>
   </sheetData>
@@ -3664,45 +3681,45 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B2" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="C2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D2" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="E2" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="F2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="G2" t="b">
         <v>0</v>
@@ -3710,22 +3727,22 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B3" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C3" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D3" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="E3" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="F3" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="G3" t="b">
         <v>0</v>
@@ -3733,22 +3750,22 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B4" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C4" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D4" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E4" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="F4" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="G4" t="b">
         <v>0</v>
@@ -3756,22 +3773,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B5" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C5" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D5" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E5" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="F5" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="G5" t="b">
         <v>0</v>
@@ -3779,22 +3796,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B6" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C6" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D6" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="E6" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="F6" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="G6" t="b">
         <v>0</v>
@@ -3802,22 +3819,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B7" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C7" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D7" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E7" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="F7" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="G7" t="b">
         <v>0</v>
@@ -3825,22 +3842,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B8" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C8" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D8" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E8" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="F8" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="G8" t="b">
         <v>0</v>
@@ -3848,22 +3865,22 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B9" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="C9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="F9" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="G9" t="b">
         <v>0</v>
@@ -3887,70 +3904,70 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B2" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="C2" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="D2" t="b">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B3" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="C3" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="D3" t="b">
         <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B4" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="C4" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -3973,33 +3990,33 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B2" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="C2" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="D2" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -4033,10 +4050,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -4063,19 +4080,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4083,19 +4100,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F2" t="s">
         <v>7</v>
@@ -4103,19 +4120,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F3" t="s">
         <v>7</v>
@@ -4123,19 +4140,19 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" t="s">
         <v>41</v>
-      </c>
-      <c r="C4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E4" t="s">
-        <v>39</v>
       </c>
       <c r="F4" t="s">
         <v>7</v>
@@ -4143,19 +4160,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F5" t="s">
         <v>7</v>
@@ -4181,36 +4198,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -4221,16 +4238,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D3" t="s">
         <v>59</v>
-      </c>
-      <c r="C3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D3" t="s">
-        <v>57</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -4241,16 +4258,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -4261,16 +4278,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -4281,16 +4298,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -4301,16 +4318,16 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" t="s">
         <v>72</v>
-      </c>
-      <c r="D7" t="s">
-        <v>70</v>
       </c>
       <c r="E7">
         <v>2</v>
@@ -4338,36 +4355,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -4378,16 +4395,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -4398,16 +4415,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -4418,16 +4435,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -4458,54 +4475,54 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -4516,25 +4533,25 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H3" t="b">
         <v>0</v>
@@ -4545,25 +4562,25 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E4" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
@@ -4574,25 +4591,25 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -4603,25 +4620,25 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -4632,25 +4649,25 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="G7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
@@ -4661,25 +4678,25 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B8" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E8" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
@@ -4690,25 +4707,25 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B9" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C9" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E9" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H9" t="b">
         <v>1</v>
@@ -4719,25 +4736,25 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B10" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C10" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D10" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E10" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F10" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -4748,25 +4765,25 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B11" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C11" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E11" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H11" t="b">
         <v>0</v>
@@ -4794,10 +4811,10 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -4811,50 +4828,50 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E3" t="s">
         <v>141</v>
-      </c>
-      <c r="D3" t="s">
-        <v>142</v>
-      </c>
-      <c r="E3" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C4" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E4" t="s">
         <v>6</v>
@@ -4862,33 +4879,33 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E6" t="s">
         <v>6</v>
@@ -4896,84 +4913,84 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D7" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E7" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B8" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C8" t="s">
+        <v>159</v>
+      </c>
+      <c r="D8" t="s">
+        <v>160</v>
+      </c>
+      <c r="E8" t="s">
         <v>157</v>
-      </c>
-      <c r="D8" t="s">
-        <v>158</v>
-      </c>
-      <c r="E8" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D9" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B10" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C10" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D10" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E10" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C11" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D11" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E11" t="s">
         <v>6</v>
@@ -4981,84 +4998,84 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B12" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C12" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D12" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E12" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C13" t="s">
+        <v>159</v>
+      </c>
+      <c r="D13" t="s">
+        <v>172</v>
+      </c>
+      <c r="E13" t="s">
         <v>157</v>
-      </c>
-      <c r="D13" t="s">
-        <v>170</v>
-      </c>
-      <c r="E13" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B14" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C14" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D14" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E14" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B15" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C15" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D15" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E15" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B16" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C16" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D16" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E16" t="s">
         <v>6</v>
@@ -5066,84 +5083,84 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B17" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C17" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D17" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E17" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B18" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C18" t="s">
+        <v>159</v>
+      </c>
+      <c r="D18" t="s">
+        <v>182</v>
+      </c>
+      <c r="E18" t="s">
         <v>157</v>
-      </c>
-      <c r="D18" t="s">
-        <v>180</v>
-      </c>
-      <c r="E18" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B19" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C19" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D19" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E19" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B20" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C20" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D20" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E20" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B21" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C21" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D21" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E21" t="s">
         <v>6</v>
@@ -5151,84 +5168,84 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B22" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C22" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D22" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E22" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B23" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C23" t="s">
+        <v>159</v>
+      </c>
+      <c r="D23" t="s">
+        <v>191</v>
+      </c>
+      <c r="E23" t="s">
         <v>157</v>
-      </c>
-      <c r="D23" t="s">
-        <v>189</v>
-      </c>
-      <c r="E23" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B24" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C24" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D24" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E24" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B25" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C25" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D25" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E25" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B26" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C26" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D26" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E26" t="s">
         <v>6</v>
@@ -5236,84 +5253,84 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B27" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C27" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D27" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="E27" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B28" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C28" t="s">
+        <v>159</v>
+      </c>
+      <c r="D28" t="s">
+        <v>201</v>
+      </c>
+      <c r="E28" t="s">
         <v>157</v>
-      </c>
-      <c r="D28" t="s">
-        <v>199</v>
-      </c>
-      <c r="E28" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B29" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C29" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D29" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E29" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B30" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C30" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D30" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E30" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B31" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C31" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D31" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E31" t="s">
         <v>6</v>
@@ -5321,84 +5338,84 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B32" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C32" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D32" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E32" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B33" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C33" t="s">
+        <v>159</v>
+      </c>
+      <c r="D33" t="s">
+        <v>211</v>
+      </c>
+      <c r="E33" t="s">
         <v>157</v>
-      </c>
-      <c r="D33" t="s">
-        <v>209</v>
-      </c>
-      <c r="E33" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B34" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C34" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D34" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="E34" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B35" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C35" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D35" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="E35" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B36" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C36" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D36" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E36" t="s">
         <v>6</v>
@@ -5406,84 +5423,84 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B37" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C37" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D37" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="E37" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B38" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C38" t="s">
+        <v>159</v>
+      </c>
+      <c r="D38" t="s">
+        <v>221</v>
+      </c>
+      <c r="E38" t="s">
         <v>157</v>
-      </c>
-      <c r="D38" t="s">
-        <v>219</v>
-      </c>
-      <c r="E38" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B39" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C39" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D39" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E39" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B40" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C40" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D40" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="E40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B41" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C41" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D41" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E41" t="s">
         <v>6</v>
@@ -5491,84 +5508,84 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B42" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C42" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D42" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E42" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B43" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C43" t="s">
+        <v>159</v>
+      </c>
+      <c r="D43" t="s">
+        <v>230</v>
+      </c>
+      <c r="E43" t="s">
         <v>157</v>
-      </c>
-      <c r="D43" t="s">
-        <v>228</v>
-      </c>
-      <c r="E43" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B44" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C44" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D44" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E44" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B45" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C45" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D45" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E45" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B46" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C46" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D46" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E46" t="s">
         <v>6</v>
@@ -5576,84 +5593,84 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B47" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C47" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D47" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E47" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B48" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C48" t="s">
+        <v>159</v>
+      </c>
+      <c r="D48" t="s">
+        <v>240</v>
+      </c>
+      <c r="E48" t="s">
         <v>157</v>
-      </c>
-      <c r="D48" t="s">
-        <v>238</v>
-      </c>
-      <c r="E48" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B49" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C49" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D49" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E49" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B50" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C50" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D50" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E50" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B51" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C51" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D51" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E51" t="s">
         <v>6</v>
@@ -5661,70 +5678,70 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B52" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C52" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D52" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E52" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B53" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C53" t="s">
+        <v>159</v>
+      </c>
+      <c r="D53" t="s">
+        <v>250</v>
+      </c>
+      <c r="E53" t="s">
         <v>157</v>
-      </c>
-      <c r="D53" t="s">
-        <v>248</v>
-      </c>
-      <c r="E53" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B54" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C54" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D54" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E54" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B55" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C55" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D55" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E55" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -5745,44 +5762,44 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B2" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C2" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D2" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B3" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D3" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>
@@ -5804,30 +5821,30 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C2" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -5851,28 +5868,28 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>3</v>
@@ -5880,25 +5897,25 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B2" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D2" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="G2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H2" t="s">
         <v>7</v>
@@ -5909,147 +5926,147 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B3" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C3" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="D3" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E3" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="F3" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="G3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H3" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="I3" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B4" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C4" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D4" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E4" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F4" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="G4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H4" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="I4" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C5" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D5" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F5" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="G5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H5" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="I5" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B6" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C6" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="D6" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="E6" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="F6" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="G6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="I6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B7" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C7" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D7" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E7" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="F7" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="G7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H7" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="I7" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final Privacy Policy, Terms and Contact pages with the real contact email (T7.1)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -79,7 +79,10 @@
     <t>contact_email</t>
   </si>
   <si>
-    <t>hello@example.com</t>
+    <t>oewersolutions@gmail.com</t>
+  </si>
+  <si>
+    <t>2026-10-30T10:27:50Z</t>
   </si>
   <si>
     <t>search_enabled</t>
@@ -158,10 +161,41 @@
     <t>Privacy Policy</t>
   </si>
   <si>
-    <t>Draft placeholder. Replace with the final privacy policy before launch (see task T7.1).</t>
-  </si>
-  <si>
-    <t>draft</t>
+    <t xml:space="preserve">Last updated: 30 October 2026
+We built OEWER Tools to be private by design. This page explains, in plain words, what happens to your information when you use the site.
+# The short version
+- Our tools run in your browser. The images, text, numbers and files you use in them stay on your device and are never uploaded to us.
+- We do not ask you to create an account.
+- We use Google Analytics to count visits, but only if you say yes. If you decline, the site works exactly the same.
+- We may show ads. Where the law requires it, personalised ads only follow your consent.
+# What stays on your device
+When you use a tool, for example the image compressor, the JSON formatter or an EMI calculator, the work is done by your browser. We do not receive, see or store what you type, paste or choose. We check this with automated tests that watch the network while each tool is used.
+The site stores one small note in your browser, called a local storage entry, to remember your analytics choice. It holds only whether you allowed analytics and when you chose.
+# Analytics (only with your permission)
+If you click **Allow analytics**, we load Google Analytics, a service from Google. It uses cookies to count visits and sends Google anonymous usage figures such as:
+- which pages you view and which tools you open or finish (by name only, never what you entered);
+- the approximate area you are in, your browser, device type and screen size;
+- how you arrived at the site, for example from a search engine.
+We use these figures to see which tools and guides are useful and what to improve. We do not use them to identify you, and we do not turn on Google's advertising features for analytics.
+If you click **Decline**, or do not answer, no analytics script is loaded and no analytics cookies are set. You can change your mind at any time with **Analytics settings** at the bottom of every page. Declining stops counting immediately and removes the analytics cookies.
+Google's own handling of this data is described in its privacy policy: [policies.google.com/privacy](https://policies.google.com/privacy).
+# Advertising
+We may show ads on the site to cover its costs, using Google AdSense. To show ads, Google and its partners may use cookies or similar technologies, and may use your approximate location and the page you are viewing. Personalised ads, where they are offered, are shown only if you consent where the law requires it. You can control Google's ad personalisation at [adssettings.google.com](https://adssettings.google.com).
+# Where the site is hosted
+The site is hosted on GitHub Pages. Like any web host, GitHub receives technical information when your browser requests a page, such as your IP address, and may keep it in its logs. We do not receive that information from GitHub. See GitHub's privacy statement at [docs.github.com/site-policy/privacy-policies](https://docs.github.com/site-policy/privacy-policies/github-general-privacy-statement).
+The fonts on this site are served from the site itself, so your browser does not contact Google Fonts.
+# When you contact us
+If you email us, we receive your email address and what you wrote. We use it only to reply and to improve the site, and we keep it for as long as it is useful for that. We do not sell it or share it for marketing.
+# Your choices and rights
+- You can allow, decline or change your analytics choice at any time, as described above.
+- You can clear cookies and site data in your browser settings.
+- You can ask us what we hold about you, and ask us to correct or delete it, by emailing [oewersolutions@gmail.com](mailto:oewersolutions@gmail.com). Depending on where you live, you may have further rights under your local data protection law, and we will honour them.
+# Children
+The site is meant for a general audience and is not directed at children under 13. We do not knowingly collect information from children.
+# Changes to this policy
+If we change how the site handles information, we will update this page and the date at the top. Please check back from time to time.
+# Contact
+Questions about privacy? Email [oewersolutions@gmail.com](mailto:oewersolutions@gmail.com).</t>
   </si>
   <si>
     <t>PAGE0003</t>
@@ -173,7 +207,28 @@
     <t>Terms of Use</t>
   </si>
   <si>
-    <t>Draft placeholder. Replace with the final terms of use before launch (see task T7.1).</t>
+    <t xml:space="preserve">Last updated: 30 October 2026
+By using OEWER Tools you agree to these terms. If you do not agree, please do not use the site.
+# Using the site
+OEWER Tools is free to use. You may use the tools and read the guides for personal or business purposes. Please do not misuse the site: do not try to break it, overload it, or interfere with how it works for others.
+# Results are for information only
+Our calculators and tools use standard formulas and we test them, but results are estimates for general information. They are not financial, tax, legal or professional advice. A real loan, deposit or tax figure may differ because of fees, rounding, rate changes and rules that apply to you. Check important numbers with your bank or a qualified professional before you rely on them.
+# Your content stays yours
+The files and text you use in a tool stay on your device. We do not receive them and we claim no rights over them. You are responsible for having the right to use anything you process with the tools.
+# Our content
+The site, its design, the guides and the tool descriptions belong to OEWER Tools. You may link to our pages and quote short extracts with a link back to the source. Please do not copy whole pages or republish our guides without asking us first.
+# Availability and changes
+We work to keep the site available and accurate, but we provide it as it is, without a promise that it will always be available, error-free or suited to a particular purpose. We may change, add or remove tools and pages at any time.
+# Limits of our responsibility
+To the extent the law allows, we are not responsible for losses that come from using, or being unable to use, the site or its results. Nothing in these terms limits any right you have by law that cannot be limited.
+# Ads and links to other sites
+The site may show ads and may link to other sites. We do not control those sites or their content and are not responsible for them. Their own terms and privacy policies apply.
+# Privacy
+How we handle information is explained in our [Privacy Policy](/privacy-policy).
+# Changes to these terms
+We may update these terms. The date at the top shows when they last changed. If you keep using the site after a change, you accept the updated terms.
+# Contact
+Questions about these terms? Email [oewersolutions@gmail.com](mailto:oewersolutions@gmail.com).</t>
   </si>
   <si>
     <t>PAGE0004</t>
@@ -186,14 +241,16 @@
   </si>
   <si>
     <t xml:space="preserve">Questions, bug reports or ideas for a new tool? We would like to hear from you.
-Email us at hello@example.com.
+Email us at [oewersolutions@gmail.com](mailto:oewersolutions@gmail.com).
 # Helpful details to include
 - The name of the tool and what you were trying to do.
 - What you expected to happen, and what happened instead.
 - Your browser and device, for example Chrome on Android.
 Please do not send passwords, bank details or files containing personal information. We do not need them to help.
 # Suggest a tool
-Tell us what you would use it for and how often. Tools that save people the most time go to the top of our list.</t>
+Tell us what you would use it for and how often. Tools that save people the most time go to the top of our list.
+# How we handle your email
+We use your message and email address only to reply to you and to improve the site. We do not add you to a mailing list or share your details. See the [Privacy Policy](/privacy-policy) for more.</t>
   </si>
   <si>
     <t>nav_id</t>
@@ -2122,18 +2179,18 @@
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D8" t="s">
         <v>7</v>
@@ -2141,13 +2198,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
         <v>21</v>
-      </c>
-      <c r="B9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" t="s">
-        <v>20</v>
       </c>
       <c r="D9" t="s">
         <v>7</v>
@@ -2155,24 +2212,24 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C10" t="s">
         <v>6</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C11" t="s">
         <v>6</v>
       </c>
       <c r="D11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -2205,7 +2262,7 @@
         <v>303</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>304</v>
@@ -3454,7 +3511,7 @@
         <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -3871,10 +3928,10 @@
         <v>488</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E9" t="s">
         <v>489</v>
@@ -4080,19 +4137,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4100,19 +4157,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
         <v>7</v>
@@ -4120,22 +4177,22 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" t="s">
         <v>37</v>
       </c>
-      <c r="B3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D3" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" t="s">
-        <v>41</v>
-      </c>
       <c r="F3" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -4152,10 +4209,10 @@
         <v>45</v>
       </c>
       <c r="E4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -4172,10 +4229,10 @@
         <v>49</v>
       </c>
       <c r="E5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -4301,7 +4358,7 @@
         <v>70</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s">
         <v>71</v>
@@ -4361,7 +4418,7 @@
         <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>77</v>
@@ -4484,7 +4541,7 @@
         <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>77</v>
@@ -4493,7 +4550,7 @@
         <v>95</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>96</v>
@@ -4522,7 +4579,7 @@
         <v>99</v>
       </c>
       <c r="G2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -4551,7 +4608,7 @@
         <v>103</v>
       </c>
       <c r="G3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H3" t="b">
         <v>0</v>
@@ -4580,7 +4637,7 @@
         <v>107</v>
       </c>
       <c r="G4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
@@ -4609,7 +4666,7 @@
         <v>111</v>
       </c>
       <c r="G5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -4638,7 +4695,7 @@
         <v>115</v>
       </c>
       <c r="G6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -4667,7 +4724,7 @@
         <v>119</v>
       </c>
       <c r="G7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
@@ -4696,7 +4753,7 @@
         <v>123</v>
       </c>
       <c r="G8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
@@ -4725,7 +4782,7 @@
         <v>127</v>
       </c>
       <c r="G9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H9" t="b">
         <v>1</v>
@@ -4754,7 +4811,7 @@
         <v>131</v>
       </c>
       <c r="G10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -4783,7 +4840,7 @@
         <v>135</v>
       </c>
       <c r="G11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H11" t="b">
         <v>0</v>
@@ -5768,7 +5825,7 @@
         <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>77</v>
@@ -5871,10 +5928,10 @@
         <v>270</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>271</v>
@@ -5886,7 +5943,7 @@
         <v>262</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>272</v>
@@ -5915,7 +5972,7 @@
         <v>266</v>
       </c>
       <c r="G2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H2" t="s">
         <v>7</v>
@@ -5944,7 +6001,7 @@
         <v>266</v>
       </c>
       <c r="G3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H3" t="s">
         <v>281</v>
@@ -5973,7 +6030,7 @@
         <v>266</v>
       </c>
       <c r="G4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H4" t="s">
         <v>286</v>
@@ -6002,7 +6059,7 @@
         <v>266</v>
       </c>
       <c r="G5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H5" t="s">
         <v>291</v>
@@ -6031,7 +6088,7 @@
         <v>266</v>
       </c>
       <c r="G6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H6" t="s">
         <v>296</v>
@@ -6060,7 +6117,7 @@
         <v>266</v>
       </c>
       <c r="G7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H7" t="s">
         <v>301</v>

</xml_diff>

<commit_message>
Ad placements: labelled reserved slots with layout rules, off by default (T7.2)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="520">
   <si>
     <t>setting_key</t>
   </si>
@@ -110,6 +110,12 @@
   </si>
   <si>
     <t>2026-10-30T10:15:15Z</t>
+  </si>
+  <si>
+    <t>adsense_publisher_id</t>
+  </si>
+  <si>
+    <t>2026-10-30T10:47:37Z</t>
   </si>
   <si>
     <t>page_id</t>
@@ -1662,6 +1668,27 @@
   </si>
   <si>
     <t>blog_post</t>
+  </si>
+  <si>
+    <t>AD0004</t>
+  </si>
+  <si>
+    <t>mid_page</t>
+  </si>
+  <si>
+    <t>AD0005</t>
+  </si>
+  <si>
+    <t>list_bottom</t>
+  </si>
+  <si>
+    <t>tool_category</t>
+  </si>
+  <si>
+    <t>AD0006</t>
+  </si>
+  <si>
+    <t>blog_index</t>
   </si>
   <si>
     <t>redirect_id</t>
@@ -2075,7 +2102,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -2230,6 +2257,17 @@
       </c>
       <c r="D11" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -2250,1242 +2288,1242 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="F2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B3" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E3" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="F3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B4" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E4" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="F4" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B5" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E5" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="F5" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B6" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E6" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="F6" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B7" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E7" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="F7" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B8" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E8" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="F8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B9" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C9">
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E9" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="F9" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B10" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C10">
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E10" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="F10" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B11" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C11">
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E11" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="F11" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B12" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C12">
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E12" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="F12" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B13" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C13">
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E13" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="F13" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B14" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C14">
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E14" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="F14" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B15" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C15">
         <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E15" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="F15" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B16" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C16">
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E16" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F16" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B17" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E17" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="F17" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B18" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C18">
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E18" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="F18" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B19" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E19" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="F19" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B20" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C20">
         <v>4</v>
       </c>
       <c r="D20" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E20" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="F20" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B21" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C21">
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E21" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="F21" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B22" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C22">
         <v>6</v>
       </c>
       <c r="D22" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E22" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="F22" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B23" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C23">
         <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E23" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="F23" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B24" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C24">
         <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E24" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="F24" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B25" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C25">
         <v>9</v>
       </c>
       <c r="D25" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E25" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="F25" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B26" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C26">
         <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E26" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="F26" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B27" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C27">
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E27" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="F27" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B28" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C28">
         <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E28" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="F28" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B29" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E29" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="F29" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B30" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C30">
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E30" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="F30" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B31" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C31">
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E31" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="F31" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B32" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C32">
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E32" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F32" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B33" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C33">
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E33" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="F33" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B34" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C34">
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E34" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="F34" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B35" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C35">
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E35" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="F35" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B36" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C36">
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E36" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="F36" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B37" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C37">
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E37" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="F37" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B38" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C38">
         <v>10</v>
       </c>
       <c r="D38" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E38" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="F38" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B39" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C39">
         <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E39" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="F39" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B40" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C40">
         <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E40" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="F40" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B41" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C41">
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E41" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="F41" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B42" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C42">
         <v>2</v>
       </c>
       <c r="D42" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E42" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F42" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B43" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C43">
         <v>3</v>
       </c>
       <c r="D43" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E43" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F43" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B44" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C44">
         <v>4</v>
       </c>
       <c r="D44" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E44" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="F44" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B45" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C45">
         <v>5</v>
       </c>
       <c r="D45" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E45" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="F45" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B46" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C46">
         <v>6</v>
       </c>
       <c r="D46" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E46" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="F46" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B47" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C47">
         <v>7</v>
       </c>
       <c r="D47" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E47" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="F47" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B48" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C48">
         <v>8</v>
       </c>
       <c r="D48" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E48" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="F48" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B49" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C49">
         <v>9</v>
       </c>
       <c r="D49" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E49" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="F49" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B50" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C50">
         <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E50" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="F50" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B51" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C51">
         <v>11</v>
       </c>
       <c r="D51" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E51" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="F51" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B52" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C52">
         <v>12</v>
       </c>
       <c r="D52" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E52" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="F52" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B53" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C53">
         <v>1</v>
       </c>
       <c r="D53" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E53" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="F53" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B54" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C54">
         <v>2</v>
       </c>
       <c r="D54" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E54" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="F54" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B55" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C55">
         <v>3</v>
       </c>
       <c r="D55" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E55" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="F55" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B56" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C56">
         <v>4</v>
       </c>
       <c r="D56" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E56" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="F56" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B57" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C57">
         <v>5</v>
       </c>
       <c r="D57" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E57" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="F57" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B58" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C58">
         <v>6</v>
       </c>
       <c r="D58" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E58" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="F58" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B59" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C59">
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E59" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="F59" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B60" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C60">
         <v>8</v>
       </c>
       <c r="D60" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E60" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="F60" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B61" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C61">
         <v>9</v>
       </c>
       <c r="D61" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E61" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="F61" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B62" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C62">
         <v>10</v>
       </c>
       <c r="D62" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E62" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="F62" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -3505,79 +3543,79 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B2" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C2" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="C3" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B4" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C4" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B5" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="C5" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B6" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="C6" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B7" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="C7" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
     </row>
   </sheetData>
@@ -3597,123 +3635,123 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C2" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B3" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C3" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B4" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C4" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B5" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C5" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C6" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B7" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C7" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B8" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C8" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B9" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C9" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B10" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C10" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B11" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C11" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
     </row>
   </sheetData>
@@ -3738,45 +3776,45 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B2" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="C2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D2" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="E2" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="F2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="G2" t="b">
         <v>0</v>
@@ -3784,22 +3822,22 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B3" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C3" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D3" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="E3" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="F3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="G3" t="b">
         <v>0</v>
@@ -3807,22 +3845,22 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B4" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C4" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="D4" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E4" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="F4" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="G4" t="b">
         <v>0</v>
@@ -3830,22 +3868,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B5" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C5" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D5" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="E5" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="F5" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="G5" t="b">
         <v>0</v>
@@ -3853,22 +3891,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B6" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C6" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D6" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="E6" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="F6" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="G6" t="b">
         <v>0</v>
@@ -3876,22 +3914,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B7" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C7" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="D7" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="E7" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="F7" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="G7" t="b">
         <v>0</v>
@@ -3899,22 +3937,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B8" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C8" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D8" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E8" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="F8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="G8" t="b">
         <v>0</v>
@@ -3922,22 +3960,22 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B9" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E9" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="F9" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="G9" t="b">
         <v>0</v>
@@ -3951,7 +3989,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -3961,70 +3999,112 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B2" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="C2" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="D2" t="b">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B3" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="C3" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="D3" t="b">
         <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B4" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="C4" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>269</v>
+        <v>271</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>504</v>
+      </c>
+      <c r="B5" t="s">
+        <v>505</v>
+      </c>
+      <c r="C5" t="s">
+        <v>498</v>
+      </c>
+      <c r="D5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>506</v>
+      </c>
+      <c r="B6" t="s">
+        <v>507</v>
+      </c>
+      <c r="C6" t="s">
+        <v>508</v>
+      </c>
+      <c r="D6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>509</v>
+      </c>
+      <c r="B7" t="s">
+        <v>507</v>
+      </c>
+      <c r="C7" t="s">
+        <v>510</v>
+      </c>
+      <c r="D7" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4047,33 +4127,33 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>503</v>
+        <v>512</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>505</v>
+        <v>514</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>506</v>
+        <v>515</v>
       </c>
       <c r="B2" t="s">
-        <v>507</v>
+        <v>516</v>
       </c>
       <c r="C2" t="s">
-        <v>508</v>
+        <v>517</v>
       </c>
       <c r="D2" t="s">
-        <v>509</v>
+        <v>518</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -4107,10 +4187,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>510</v>
+        <v>519</v>
       </c>
       <c r="B2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -4137,19 +4217,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4157,19 +4237,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F2" t="s">
         <v>7</v>
@@ -4177,19 +4257,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E3" t="s">
         <v>39</v>
-      </c>
-      <c r="C3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E3" t="s">
-        <v>37</v>
       </c>
       <c r="F3" t="s">
         <v>18</v>
@@ -4197,19 +4277,19 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F4" t="s">
         <v>18</v>
@@ -4217,19 +4297,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F5" t="s">
         <v>18</v>
@@ -4255,36 +4335,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -4295,16 +4375,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D3" t="s">
         <v>61</v>
-      </c>
-      <c r="C3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D3" t="s">
-        <v>59</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -4315,16 +4395,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -4335,16 +4415,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -4355,16 +4435,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -4375,16 +4455,16 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7" t="s">
         <v>74</v>
-      </c>
-      <c r="D7" t="s">
-        <v>72</v>
       </c>
       <c r="E7">
         <v>2</v>
@@ -4412,36 +4492,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -4452,16 +4532,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -4472,16 +4552,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -4492,16 +4572,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -4532,54 +4612,54 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -4590,25 +4670,25 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H3" t="b">
         <v>0</v>
@@ -4619,25 +4699,25 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C4" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E4" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
@@ -4648,25 +4728,25 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -4677,25 +4757,25 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="G6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -4706,25 +4786,25 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D7" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E7" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F7" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
@@ -4735,25 +4815,25 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C8" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D8" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E8" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F8" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
@@ -4764,25 +4844,25 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B9" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C9" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D9" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F9" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H9" t="b">
         <v>1</v>
@@ -4793,25 +4873,25 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C10" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D10" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F10" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G10" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -4822,25 +4902,25 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C11" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E11" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H11" t="b">
         <v>0</v>
@@ -4868,10 +4948,10 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -4885,50 +4965,50 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C3" t="s">
+        <v>145</v>
+      </c>
+      <c r="D3" t="s">
+        <v>146</v>
+      </c>
+      <c r="E3" t="s">
         <v>143</v>
-      </c>
-      <c r="D3" t="s">
-        <v>144</v>
-      </c>
-      <c r="E3" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C4" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D4" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E4" t="s">
         <v>6</v>
@@ -4936,33 +5016,33 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E6" t="s">
         <v>6</v>
@@ -4970,84 +5050,84 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C7" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D7" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C8" t="s">
+        <v>161</v>
+      </c>
+      <c r="D8" t="s">
+        <v>162</v>
+      </c>
+      <c r="E8" t="s">
         <v>159</v>
-      </c>
-      <c r="D8" t="s">
-        <v>160</v>
-      </c>
-      <c r="E8" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C9" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D9" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E9" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B10" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C10" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D10" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E10" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C11" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D11" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E11" t="s">
         <v>6</v>
@@ -5055,84 +5135,84 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B12" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C12" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D12" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E12" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D13" t="s">
+        <v>174</v>
+      </c>
+      <c r="E13" t="s">
         <v>159</v>
-      </c>
-      <c r="D13" t="s">
-        <v>172</v>
-      </c>
-      <c r="E13" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B14" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C14" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D14" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E14" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B15" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C15" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D15" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E15" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B16" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C16" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D16" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E16" t="s">
         <v>6</v>
@@ -5140,84 +5220,84 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B17" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C17" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D17" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E17" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B18" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C18" t="s">
+        <v>161</v>
+      </c>
+      <c r="D18" t="s">
+        <v>184</v>
+      </c>
+      <c r="E18" t="s">
         <v>159</v>
-      </c>
-      <c r="D18" t="s">
-        <v>182</v>
-      </c>
-      <c r="E18" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B19" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C19" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D19" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E19" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B20" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C20" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D20" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E20" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B21" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C21" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D21" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E21" t="s">
         <v>6</v>
@@ -5225,84 +5305,84 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B22" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C22" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D22" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E22" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B23" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C23" t="s">
+        <v>161</v>
+      </c>
+      <c r="D23" t="s">
+        <v>193</v>
+      </c>
+      <c r="E23" t="s">
         <v>159</v>
-      </c>
-      <c r="D23" t="s">
-        <v>191</v>
-      </c>
-      <c r="E23" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B24" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C24" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D24" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E24" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B25" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C25" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D25" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E25" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B26" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C26" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D26" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="E26" t="s">
         <v>6</v>
@@ -5310,84 +5390,84 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B27" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C27" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D27" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E27" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B28" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C28" t="s">
+        <v>161</v>
+      </c>
+      <c r="D28" t="s">
+        <v>203</v>
+      </c>
+      <c r="E28" t="s">
         <v>159</v>
-      </c>
-      <c r="D28" t="s">
-        <v>201</v>
-      </c>
-      <c r="E28" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C29" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D29" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E29" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B30" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C30" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D30" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E30" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B31" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C31" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D31" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E31" t="s">
         <v>6</v>
@@ -5395,84 +5475,84 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B32" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C32" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D32" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E32" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B33" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C33" t="s">
+        <v>161</v>
+      </c>
+      <c r="D33" t="s">
+        <v>213</v>
+      </c>
+      <c r="E33" t="s">
         <v>159</v>
-      </c>
-      <c r="D33" t="s">
-        <v>211</v>
-      </c>
-      <c r="E33" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B34" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C34" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D34" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="E34" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B35" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C35" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D35" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E35" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B36" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C36" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D36" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="E36" t="s">
         <v>6</v>
@@ -5480,84 +5560,84 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B37" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C37" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D37" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E37" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B38" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C38" t="s">
+        <v>161</v>
+      </c>
+      <c r="D38" t="s">
+        <v>223</v>
+      </c>
+      <c r="E38" t="s">
         <v>159</v>
-      </c>
-      <c r="D38" t="s">
-        <v>221</v>
-      </c>
-      <c r="E38" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B39" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C39" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D39" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B40" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C40" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D40" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E40" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B41" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C41" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D41" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E41" t="s">
         <v>6</v>
@@ -5565,84 +5645,84 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B42" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C42" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D42" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E42" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B43" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C43" t="s">
+        <v>161</v>
+      </c>
+      <c r="D43" t="s">
+        <v>232</v>
+      </c>
+      <c r="E43" t="s">
         <v>159</v>
-      </c>
-      <c r="D43" t="s">
-        <v>230</v>
-      </c>
-      <c r="E43" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B44" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C44" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D44" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E44" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B45" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C45" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D45" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E45" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B46" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C46" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D46" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E46" t="s">
         <v>6</v>
@@ -5650,84 +5730,84 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B47" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C47" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D47" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E47" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B48" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C48" t="s">
+        <v>161</v>
+      </c>
+      <c r="D48" t="s">
+        <v>242</v>
+      </c>
+      <c r="E48" t="s">
         <v>159</v>
-      </c>
-      <c r="D48" t="s">
-        <v>240</v>
-      </c>
-      <c r="E48" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B49" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C49" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D49" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E49" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B50" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C50" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D50" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E50" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B51" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C51" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D51" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E51" t="s">
         <v>6</v>
@@ -5735,70 +5815,70 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B52" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C52" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D52" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E52" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B53" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C53" t="s">
+        <v>161</v>
+      </c>
+      <c r="D53" t="s">
+        <v>252</v>
+      </c>
+      <c r="E53" t="s">
         <v>159</v>
-      </c>
-      <c r="D53" t="s">
-        <v>250</v>
-      </c>
-      <c r="E53" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B54" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C54" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D54" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E54" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B55" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C55" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D55" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E55" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -5819,44 +5899,44 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B2" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C2" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D2" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B3" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C3" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D3" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -5878,30 +5958,30 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C2" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -5925,28 +6005,28 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>3</v>
@@ -5954,25 +6034,25 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B2" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C2" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D2" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E2" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F2" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="G2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H2" t="s">
         <v>7</v>
@@ -5983,147 +6063,147 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B3" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C3" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="D3" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="F3" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="G3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H3" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="I3" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B4" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C4" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D4" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E4" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F4" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="G4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H4" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="I4" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B5" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C5" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D5" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E5" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F5" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="G5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H5" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="I5" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B6" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D6" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="E6" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="F6" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="G6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H6" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="I6" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B7" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C7" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D7" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E7" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="F7" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="G7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H7" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="I7" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Custom domain oewer.in verified, site_url set, restore from history verified on the real repo (T7.5)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="521">
   <si>
     <t>setting_key</t>
   </si>
@@ -67,7 +67,10 @@
     <t>site_url</t>
   </si>
   <si>
-    <t>https://example.com</t>
+    <t>https://oewer.in</t>
+  </si>
+  <si>
+    <t>2026-10-30T11:37:29Z</t>
   </si>
   <si>
     <t>primary_color</t>
@@ -2178,15 +2181,15 @@
         <v>6</v>
       </c>
       <c r="D5" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
         <v>6</v>
@@ -2197,27 +2200,27 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C7" t="s">
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D8" t="s">
         <v>7</v>
@@ -2225,13 +2228,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
         <v>22</v>
-      </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
       </c>
       <c r="D9" t="s">
         <v>7</v>
@@ -2239,35 +2242,35 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
         <v>6</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
         <v>6</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C12" t="s">
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -2288,1242 +2291,1242 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B4" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E4" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F4" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B5" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E5" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E6" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B7" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E7" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F7" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B8" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E8" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F8" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B9" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C9">
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E9" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F9" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B10" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C10">
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E10" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B11" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C11">
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F11" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B12" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C12">
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E12" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F12" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B13" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C13">
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E13" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F13" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B14" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C14">
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E14" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F14" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B15" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C15">
         <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E15" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F15" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B16" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C16">
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E16" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F16" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B17" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E17" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F17" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B18" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C18">
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E18" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F18" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B19" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E19" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F19" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B20" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C20">
         <v>4</v>
       </c>
       <c r="D20" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E20" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F20" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B21" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C21">
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E21" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F21" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B22" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C22">
         <v>6</v>
       </c>
       <c r="D22" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E22" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F22" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B23" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C23">
         <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E23" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F23" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B24" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C24">
         <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E24" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F24" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B25" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C25">
         <v>9</v>
       </c>
       <c r="D25" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E25" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F25" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B26" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C26">
         <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E26" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F26" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B27" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C27">
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E27" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F27" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B28" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C28">
         <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E28" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F28" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B29" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E29" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F29" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B30" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C30">
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E30" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F30" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B31" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C31">
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E31" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F31" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B32" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C32">
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E32" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F32" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C33">
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E33" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F33" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B34" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C34">
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E34" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F34" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B35" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C35">
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E35" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F35" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B36" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C36">
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E36" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F36" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B37" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C37">
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E37" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="F37" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B38" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C38">
         <v>10</v>
       </c>
       <c r="D38" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E38" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F38" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B39" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C39">
         <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E39" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F39" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B40" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C40">
         <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E40" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F40" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B41" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C41">
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E41" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F41" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B42" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C42">
         <v>2</v>
       </c>
       <c r="D42" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E42" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F42" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B43" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C43">
         <v>3</v>
       </c>
       <c r="D43" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E43" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F43" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B44" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C44">
         <v>4</v>
       </c>
       <c r="D44" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E44" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="F44" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B45" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C45">
         <v>5</v>
       </c>
       <c r="D45" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E45" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F45" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B46" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C46">
         <v>6</v>
       </c>
       <c r="D46" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E46" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F46" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B47" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C47">
         <v>7</v>
       </c>
       <c r="D47" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E47" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F47" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B48" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C48">
         <v>8</v>
       </c>
       <c r="D48" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E48" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F48" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B49" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C49">
         <v>9</v>
       </c>
       <c r="D49" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E49" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F49" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B50" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C50">
         <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E50" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="F50" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B51" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C51">
         <v>11</v>
       </c>
       <c r="D51" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E51" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F51" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B52" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C52">
         <v>12</v>
       </c>
       <c r="D52" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E52" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="F52" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B53" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C53">
         <v>1</v>
       </c>
       <c r="D53" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E53" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F53" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B54" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C54">
         <v>2</v>
       </c>
       <c r="D54" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E54" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="F54" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B55" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C55">
         <v>3</v>
       </c>
       <c r="D55" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E55" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F55" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B56" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C56">
         <v>4</v>
       </c>
       <c r="D56" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E56" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="F56" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B57" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C57">
         <v>5</v>
       </c>
       <c r="D57" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E57" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F57" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B58" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C58">
         <v>6</v>
       </c>
       <c r="D58" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E58" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="F58" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B59" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C59">
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E59" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F59" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B60" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C60">
         <v>8</v>
       </c>
       <c r="D60" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E60" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="F60" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B61" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C61">
         <v>9</v>
       </c>
       <c r="D61" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E61" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F61" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B62" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C62">
         <v>10</v>
       </c>
       <c r="D62" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E62" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="F62" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -3543,79 +3546,79 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B2" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C2" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B3" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C3" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B4" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C4" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B5" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C5" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B6" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C6" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B7" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C7" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
   </sheetData>
@@ -3635,123 +3638,123 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C2" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C3" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C4" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B5" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C5" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B6" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C6" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B7" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C7" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B8" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C8" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B9" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C9" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B10" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C10" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C11" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
   </sheetData>
@@ -3776,45 +3779,45 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B2" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="F2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G2" t="b">
         <v>0</v>
@@ -3822,22 +3825,22 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B3" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D3" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E3" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="F3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G3" t="b">
         <v>0</v>
@@ -3845,22 +3848,22 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B4" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E4" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F4" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G4" t="b">
         <v>0</v>
@@ -3868,22 +3871,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B5" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C5" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E5" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G5" t="b">
         <v>0</v>
@@ -3891,22 +3894,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B6" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D6" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="E6" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G6" t="b">
         <v>0</v>
@@ -3914,22 +3917,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B7" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C7" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D7" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E7" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="F7" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G7" t="b">
         <v>0</v>
@@ -3937,22 +3940,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B8" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C8" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D8" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E8" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="F8" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G8" t="b">
         <v>0</v>
@@ -3960,22 +3963,22 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B9" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E9" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F9" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G9" t="b">
         <v>0</v>
@@ -3999,81 +4002,81 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B2" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="C2" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="D2" t="b">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B3" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C3" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="D3" t="b">
         <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B4" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C4" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B5" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="C5" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="D5" t="b">
         <v>0</v>
@@ -4081,13 +4084,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B6" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="C6" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D6" t="b">
         <v>0</v>
@@ -4095,13 +4098,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B7" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="C7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="D7" t="b">
         <v>0</v>
@@ -4127,33 +4130,33 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B2" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C2" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D2" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -4187,10 +4190,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -4217,19 +4220,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4237,19 +4240,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F2" t="s">
         <v>7</v>
@@ -4257,62 +4260,62 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E3" t="s">
         <v>40</v>
       </c>
-      <c r="B3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E3" t="s">
-        <v>39</v>
-      </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -4335,36 +4338,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -4375,16 +4378,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" t="s">
         <v>62</v>
-      </c>
-      <c r="B3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D3" t="s">
-        <v>61</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -4395,16 +4398,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -4415,16 +4418,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -4435,16 +4438,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -4455,16 +4458,16 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" t="s">
         <v>75</v>
-      </c>
-      <c r="B7" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" t="s">
-        <v>76</v>
-      </c>
-      <c r="D7" t="s">
-        <v>74</v>
       </c>
       <c r="E7">
         <v>2</v>
@@ -4492,36 +4495,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -4532,16 +4535,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -4552,16 +4555,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -4572,16 +4575,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -4612,54 +4615,54 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E2" t="s">
+        <v>103</v>
+      </c>
+      <c r="F2" t="s">
         <v>102</v>
       </c>
-      <c r="F2" t="s">
-        <v>101</v>
-      </c>
       <c r="G2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -4670,25 +4673,25 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E3" t="s">
+        <v>107</v>
+      </c>
+      <c r="F3" t="s">
         <v>106</v>
       </c>
-      <c r="F3" t="s">
-        <v>105</v>
-      </c>
       <c r="G3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H3" t="b">
         <v>0</v>
@@ -4699,25 +4702,25 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E4" t="s">
+        <v>111</v>
+      </c>
+      <c r="F4" t="s">
         <v>110</v>
       </c>
-      <c r="F4" t="s">
-        <v>109</v>
-      </c>
       <c r="G4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
@@ -4728,25 +4731,25 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E5" t="s">
+        <v>115</v>
+      </c>
+      <c r="F5" t="s">
         <v>114</v>
       </c>
-      <c r="F5" t="s">
-        <v>113</v>
-      </c>
       <c r="G5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -4757,25 +4760,25 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E6" t="s">
+        <v>119</v>
+      </c>
+      <c r="F6" t="s">
         <v>118</v>
       </c>
-      <c r="F6" t="s">
-        <v>117</v>
-      </c>
       <c r="G6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -4786,25 +4789,25 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E7" t="s">
+        <v>123</v>
+      </c>
+      <c r="F7" t="s">
         <v>122</v>
       </c>
-      <c r="F7" t="s">
-        <v>121</v>
-      </c>
       <c r="G7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
@@ -4815,25 +4818,25 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E8" t="s">
+        <v>127</v>
+      </c>
+      <c r="F8" t="s">
         <v>126</v>
       </c>
-      <c r="F8" t="s">
-        <v>125</v>
-      </c>
       <c r="G8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
@@ -4844,25 +4847,25 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E9" t="s">
+        <v>131</v>
+      </c>
+      <c r="F9" t="s">
         <v>130</v>
       </c>
-      <c r="F9" t="s">
-        <v>129</v>
-      </c>
       <c r="G9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H9" t="b">
         <v>1</v>
@@ -4873,25 +4876,25 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E10" t="s">
+        <v>135</v>
+      </c>
+      <c r="F10" t="s">
         <v>134</v>
       </c>
-      <c r="F10" t="s">
-        <v>133</v>
-      </c>
       <c r="G10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -4902,25 +4905,25 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C11" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E11" t="s">
+        <v>139</v>
+      </c>
+      <c r="F11" t="s">
         <v>138</v>
       </c>
-      <c r="F11" t="s">
-        <v>137</v>
-      </c>
       <c r="G11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H11" t="b">
         <v>0</v>
@@ -4948,10 +4951,10 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -4965,50 +4968,50 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" t="s">
+        <v>146</v>
+      </c>
+      <c r="D3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E3" t="s">
         <v>144</v>
-      </c>
-      <c r="B3" t="s">
-        <v>99</v>
-      </c>
-      <c r="C3" t="s">
-        <v>145</v>
-      </c>
-      <c r="D3" t="s">
-        <v>146</v>
-      </c>
-      <c r="E3" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E4" t="s">
         <v>6</v>
@@ -5016,33 +5019,33 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E6" t="s">
         <v>6</v>
@@ -5050,84 +5053,84 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C8" t="s">
+        <v>162</v>
+      </c>
+      <c r="D8" t="s">
+        <v>163</v>
+      </c>
+      <c r="E8" t="s">
         <v>160</v>
-      </c>
-      <c r="B8" t="s">
-        <v>99</v>
-      </c>
-      <c r="C8" t="s">
-        <v>161</v>
-      </c>
-      <c r="D8" t="s">
-        <v>162</v>
-      </c>
-      <c r="E8" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E9" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C11" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E11" t="s">
         <v>6</v>
@@ -5135,84 +5138,84 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B12" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C12" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D12" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E12" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E13" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E14" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C15" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E15" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B16" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C16" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E16" t="s">
         <v>6</v>
@@ -5220,84 +5223,84 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B17" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C17" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D17" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E17" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B18" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C18" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D18" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E18" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B19" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C19" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D19" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E19" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C20" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D20" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E20" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B21" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C21" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D21" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E21" t="s">
         <v>6</v>
@@ -5305,84 +5308,84 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B22" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C22" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D22" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E22" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B23" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C23" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D23" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E23" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B24" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C24" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D24" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E24" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B25" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C25" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D25" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E25" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B26" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C26" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D26" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E26" t="s">
         <v>6</v>
@@ -5390,84 +5393,84 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B27" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C27" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D27" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E27" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B28" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C28" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D28" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E28" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B29" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C29" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D29" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E29" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B30" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C30" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D30" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E30" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B31" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C31" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D31" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E31" t="s">
         <v>6</v>
@@ -5475,84 +5478,84 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B32" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C32" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D32" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E32" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B33" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C33" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D33" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E33" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B34" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C34" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D34" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E34" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B35" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C35" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D35" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E35" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B36" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C36" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D36" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E36" t="s">
         <v>6</v>
@@ -5560,84 +5563,84 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B37" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C37" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D37" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E37" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B38" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D38" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E38" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B39" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C39" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D39" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B40" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C40" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D40" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E40" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B41" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C41" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D41" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E41" t="s">
         <v>6</v>
@@ -5645,84 +5648,84 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B42" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C42" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D42" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E42" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B43" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C43" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D43" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E43" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B44" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C44" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D44" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E44" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B45" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C45" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D45" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E45" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B46" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C46" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D46" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E46" t="s">
         <v>6</v>
@@ -5730,84 +5733,84 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B47" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C47" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D47" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E47" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B48" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C48" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D48" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E48" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B49" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C49" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D49" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E49" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B50" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C50" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D50" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E50" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B51" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C51" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D51" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E51" t="s">
         <v>6</v>
@@ -5815,70 +5818,70 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B52" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C52" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D52" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E52" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B53" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C53" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D53" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E53" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B54" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C54" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D54" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E54" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B55" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C55" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D55" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E55" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -5899,44 +5902,44 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -5958,30 +5961,30 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -6005,28 +6008,28 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>3</v>
@@ -6034,25 +6037,25 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H2" t="s">
         <v>7</v>
@@ -6063,147 +6066,147 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="I3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B4" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C4" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="I4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C5" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D5" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E5" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F5" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H5" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="I5" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B6" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D6" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E6" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F6" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H6" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="I6" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B7" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C7" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D7" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E7" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F7" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H7" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="I7" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AdSense readiness: ads.txt, account tag, consent-gated loader, ad choice in privacy panel, guide (T7.7)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="521">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="522">
   <si>
     <t>setting_key</t>
   </si>
@@ -176,7 +176,7 @@
 - Our tools run in your browser. The images, text, numbers and files you use in them stay on your device and are never uploaded to us.
 - We do not ask you to create an account.
 - We use Google Analytics to count visits, but only if you say yes. If you decline, the site works exactly the same.
-- We may show ads. Where the law requires it, personalised ads only follow your consent.
+- We may show ads, but only if you allow them, and they are not personalised.
 # What stays on your device
 When you use a tool, for example the image compressor, the JSON formatter or an EMI calculator, the work is done by your browser. We do not receive, see or store what you type, paste or choose. We check this with automated tests that watch the network while each tool is used.
 The site stores one small note in your browser, called a local storage entry, to remember your analytics choice. It holds only whether you allowed analytics and when you chose.
@@ -186,10 +186,10 @@
 - the approximate area you are in, your browser, device type and screen size;
 - how you arrived at the site, for example from a search engine.
 We use these figures to see which tools and guides are useful and what to improve. We do not use them to identify you, and we do not turn on Google's advertising features for analytics.
-If you click **Decline**, or do not answer, no analytics script is loaded and no analytics cookies are set. You can change your mind at any time with **Analytics settings** at the bottom of every page. Declining stops counting immediately and removes the analytics cookies.
+If you click **Decline**, or do not answer, no analytics script is loaded and no analytics cookies are set. You can change your mind at any time with **Analytics settings** at the bottom of every page (called **Privacy choices** once ads are switched on). Declining stops counting immediately and removes the analytics cookies.
 Google's own handling of this data is described in its privacy policy: [policies.google.com/privacy](https://policies.google.com/privacy).
 # Advertising
-We may show ads on the site to cover its costs, using Google AdSense. To show ads, Google and its partners may use cookies or similar technologies, and may use your approximate location and the page you are viewing. Personalised ads, where they are offered, are shown only if you consent where the law requires it. You can control Google's ad personalisation at [adssettings.google.com](https://adssettings.google.com).
+We may show ads on the site to cover its costs, using Google AdSense. We ask for your permission first: no ad is shown, and Google's ad script is not loaded, unless you choose **Ads** in the privacy choices panel. We ask Google for non-personalised ads, which are based on the page you are viewing rather than on your browsing history. Google and its partners may still use cookies or similar technologies, and your approximate location, to show and measure ads and to prevent fraud. You can change your choice at any time with **Privacy choices** at the bottom of every page (it appears once ads are switched on), and you can control Google's ad personalisation across the web at [adssettings.google.com](https://adssettings.google.com).
 # Where the site is hosted
 The site is hosted on GitHub Pages. Like any web host, GitHub receives technical information when your browser requests a page, such as your IP address, and may keep it in its logs. We do not receive that information from GitHub. See GitHub's privacy statement at [docs.github.com/site-policy/privacy-policies](https://docs.github.com/site-policy/privacy-policies/github-general-privacy-statement).
 The fonts on this site are served from the site itself, so your browser does not contact Google Fonts.
@@ -205,6 +205,9 @@
 If we change how the site handles information, we will update this page and the date at the top. Please check back from time to time.
 # Contact
 Questions about privacy? Email [oewersolutions@gmail.com](mailto:oewersolutions@gmail.com).</t>
+  </si>
+  <si>
+    <t>2026-10-30T13:00:32Z</t>
   </si>
   <si>
     <t>PAGE0003</t>
@@ -2291,1242 +2294,1242 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>34</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E4" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B5" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E5" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F5" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B6" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E6" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B7" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E7" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F7" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E8" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F8" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B9" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C9">
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E9" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C10">
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B11" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C11">
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E11" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B12" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C12">
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E12" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F12" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B13" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C13">
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E13" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F13" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B14" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C14">
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E14" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F14" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B15" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C15">
         <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E15" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F15" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B16" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C16">
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E16" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F16" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B17" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E17" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B18" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C18">
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E18" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F18" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B19" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E19" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F19" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B20" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C20">
         <v>4</v>
       </c>
       <c r="D20" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E20" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F20" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B21" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C21">
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E21" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="F21" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B22" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C22">
         <v>6</v>
       </c>
       <c r="D22" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E22" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F22" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B23" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C23">
         <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E23" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F23" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B24" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C24">
         <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E24" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F24" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B25" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C25">
         <v>9</v>
       </c>
       <c r="D25" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E25" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F25" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B26" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C26">
         <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E26" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F26" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B27" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C27">
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E27" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="F27" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B28" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C28">
         <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E28" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F28" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B29" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E29" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F29" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B30" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C30">
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E30" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F30" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B31" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C31">
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E31" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F31" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B32" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C32">
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E32" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F32" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B33" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C33">
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E33" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F33" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B34" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C34">
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E34" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F34" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B35" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C35">
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E35" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F35" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B36" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C36">
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E36" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F36" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B37" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C37">
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E37" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F37" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B38" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C38">
         <v>10</v>
       </c>
       <c r="D38" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E38" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F38" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B39" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C39">
         <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E39" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="F39" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C40">
         <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E40" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F40" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B41" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C41">
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E41" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F41" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B42" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C42">
         <v>2</v>
       </c>
       <c r="D42" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E42" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F42" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B43" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C43">
         <v>3</v>
       </c>
       <c r="D43" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E43" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="F43" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B44" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C44">
         <v>4</v>
       </c>
       <c r="D44" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E44" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F44" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B45" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C45">
         <v>5</v>
       </c>
       <c r="D45" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E45" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="F45" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B46" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C46">
         <v>6</v>
       </c>
       <c r="D46" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E46" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F46" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B47" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C47">
         <v>7</v>
       </c>
       <c r="D47" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E47" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F47" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B48" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C48">
         <v>8</v>
       </c>
       <c r="D48" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E48" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F48" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B49" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C49">
         <v>9</v>
       </c>
       <c r="D49" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E49" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F49" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B50" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C50">
         <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E50" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F50" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B51" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C51">
         <v>11</v>
       </c>
       <c r="D51" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E51" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="F51" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B52" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C52">
         <v>12</v>
       </c>
       <c r="D52" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E52" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="F52" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B53" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C53">
         <v>1</v>
       </c>
       <c r="D53" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E53" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="F53" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B54" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C54">
         <v>2</v>
       </c>
       <c r="D54" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E54" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F54" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B55" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C55">
         <v>3</v>
       </c>
       <c r="D55" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E55" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F55" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B56" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C56">
         <v>4</v>
       </c>
       <c r="D56" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E56" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="F56" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B57" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C57">
         <v>5</v>
       </c>
       <c r="D57" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E57" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="F57" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B58" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C58">
         <v>6</v>
       </c>
       <c r="D58" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E58" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="F58" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B59" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C59">
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E59" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F59" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B60" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C60">
         <v>8</v>
       </c>
       <c r="D60" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E60" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F60" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B61" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C61">
         <v>9</v>
       </c>
       <c r="D61" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E61" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F61" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B62" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C62">
         <v>10</v>
       </c>
       <c r="D62" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E62" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="F62" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>
@@ -3546,10 +3549,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>32</v>
@@ -3557,68 +3560,68 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B2" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C2" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B3" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C3" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B4" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B5" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C5" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B6" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C6" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B7" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C7" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
   </sheetData>
@@ -3638,123 +3641,123 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C2" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C3" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C4" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B5" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C5" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C6" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B7" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C7" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B8" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C8" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B9" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C9" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B10" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C10" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C11" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
   </sheetData>
@@ -3779,45 +3782,45 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="E2" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="F2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G2" t="b">
         <v>0</v>
@@ -3825,22 +3828,22 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B3" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D3" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="E3" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="F3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G3" t="b">
         <v>0</v>
@@ -3848,22 +3851,22 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B4" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D4" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E4" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G4" t="b">
         <v>0</v>
@@ -3871,22 +3874,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B5" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D5" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E5" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F5" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G5" t="b">
         <v>0</v>
@@ -3894,22 +3897,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B6" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C6" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D6" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E6" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G6" t="b">
         <v>0</v>
@@ -3917,22 +3920,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B7" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C7" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D7" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E7" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F7" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G7" t="b">
         <v>0</v>
@@ -3940,22 +3943,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B8" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C8" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D8" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E8" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="F8" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G8" t="b">
         <v>0</v>
@@ -3963,10 +3966,10 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B9" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="C9" t="s">
         <v>36</v>
@@ -3975,10 +3978,10 @@
         <v>38</v>
       </c>
       <c r="E9" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="F9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G9" t="b">
         <v>0</v>
@@ -4002,81 +4005,81 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B2" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="C2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D2" t="b">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B3" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="C3" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="D3" t="b">
         <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B4" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C4" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B5" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="C5" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D5" t="b">
         <v>0</v>
@@ -4084,13 +4087,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B6" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="C6" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="D6" t="b">
         <v>0</v>
@@ -4098,13 +4101,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B7" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="C7" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="D7" t="b">
         <v>0</v>
@@ -4130,33 +4133,33 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B2" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="C2" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="D2" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -4190,10 +4193,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -4275,21 +4278,21 @@
         <v>40</v>
       </c>
       <c r="F3" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E4" t="s">
         <v>40</v>
@@ -4300,16 +4303,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E5" t="s">
         <v>40</v>
@@ -4338,36 +4341,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -4378,16 +4381,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" t="s">
         <v>63</v>
-      </c>
-      <c r="B3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D3" t="s">
-        <v>62</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -4398,16 +4401,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -4418,16 +4421,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -4438,16 +4441,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B6" t="s">
         <v>43</v>
       </c>
       <c r="C6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -4458,16 +4461,16 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D7" t="s">
         <v>76</v>
-      </c>
-      <c r="B7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" t="s">
-        <v>77</v>
-      </c>
-      <c r="D7" t="s">
-        <v>75</v>
       </c>
       <c r="E7">
         <v>2</v>
@@ -4495,36 +4498,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>32</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -4535,16 +4538,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -4555,16 +4558,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -4575,16 +4578,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -4615,51 +4618,51 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>35</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E2" t="s">
+        <v>104</v>
+      </c>
+      <c r="F2" t="s">
         <v>103</v>
-      </c>
-      <c r="F2" t="s">
-        <v>102</v>
       </c>
       <c r="G2" t="s">
         <v>40</v>
@@ -4673,22 +4676,22 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E3" t="s">
+        <v>108</v>
+      </c>
+      <c r="F3" t="s">
         <v>107</v>
-      </c>
-      <c r="F3" t="s">
-        <v>106</v>
       </c>
       <c r="G3" t="s">
         <v>40</v>
@@ -4702,22 +4705,22 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E4" t="s">
+        <v>112</v>
+      </c>
+      <c r="F4" t="s">
         <v>111</v>
-      </c>
-      <c r="F4" t="s">
-        <v>110</v>
       </c>
       <c r="G4" t="s">
         <v>40</v>
@@ -4731,22 +4734,22 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E5" t="s">
+        <v>116</v>
+      </c>
+      <c r="F5" t="s">
         <v>115</v>
-      </c>
-      <c r="F5" t="s">
-        <v>114</v>
       </c>
       <c r="G5" t="s">
         <v>40</v>
@@ -4760,22 +4763,22 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F6" t="s">
         <v>119</v>
-      </c>
-      <c r="F6" t="s">
-        <v>118</v>
       </c>
       <c r="G6" t="s">
         <v>40</v>
@@ -4789,22 +4792,22 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E7" t="s">
+        <v>124</v>
+      </c>
+      <c r="F7" t="s">
         <v>123</v>
-      </c>
-      <c r="F7" t="s">
-        <v>122</v>
       </c>
       <c r="G7" t="s">
         <v>40</v>
@@ -4818,22 +4821,22 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E8" t="s">
+        <v>128</v>
+      </c>
+      <c r="F8" t="s">
         <v>127</v>
-      </c>
-      <c r="F8" t="s">
-        <v>126</v>
       </c>
       <c r="G8" t="s">
         <v>40</v>
@@ -4847,22 +4850,22 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E9" t="s">
+        <v>132</v>
+      </c>
+      <c r="F9" t="s">
         <v>131</v>
-      </c>
-      <c r="F9" t="s">
-        <v>130</v>
       </c>
       <c r="G9" t="s">
         <v>40</v>
@@ -4876,22 +4879,22 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B10" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E10" t="s">
+        <v>136</v>
+      </c>
+      <c r="F10" t="s">
         <v>135</v>
-      </c>
-      <c r="F10" t="s">
-        <v>134</v>
       </c>
       <c r="G10" t="s">
         <v>40</v>
@@ -4905,22 +4908,22 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D11" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E11" t="s">
+        <v>140</v>
+      </c>
+      <c r="F11" t="s">
         <v>139</v>
-      </c>
-      <c r="F11" t="s">
-        <v>138</v>
       </c>
       <c r="G11" t="s">
         <v>40</v>
@@ -4951,10 +4954,10 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -4968,50 +4971,50 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>146</v>
+      </c>
+      <c r="B3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E3" t="s">
         <v>145</v>
-      </c>
-      <c r="B3" t="s">
-        <v>100</v>
-      </c>
-      <c r="C3" t="s">
-        <v>146</v>
-      </c>
-      <c r="D3" t="s">
-        <v>147</v>
-      </c>
-      <c r="E3" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E4" t="s">
         <v>6</v>
@@ -5019,33 +5022,33 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E6" t="s">
         <v>6</v>
@@ -5053,84 +5056,84 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>162</v>
+      </c>
+      <c r="B8" t="s">
+        <v>101</v>
+      </c>
+      <c r="C8" t="s">
+        <v>163</v>
+      </c>
+      <c r="D8" t="s">
+        <v>164</v>
+      </c>
+      <c r="E8" t="s">
         <v>161</v>
-      </c>
-      <c r="B8" t="s">
-        <v>100</v>
-      </c>
-      <c r="C8" t="s">
-        <v>162</v>
-      </c>
-      <c r="D8" t="s">
-        <v>163</v>
-      </c>
-      <c r="E8" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D9" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E9" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C11" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E11" t="s">
         <v>6</v>
@@ -5138,84 +5141,84 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D12" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E12" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E13" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E14" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B15" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D15" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E15" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C16" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D16" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E16" t="s">
         <v>6</v>
@@ -5223,84 +5226,84 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B17" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C17" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D17" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E17" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C18" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D18" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E18" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B19" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C19" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D19" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E19" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C20" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D20" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E20" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B21" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C21" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D21" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E21" t="s">
         <v>6</v>
@@ -5308,84 +5311,84 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B22" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C22" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D22" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E22" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C23" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D23" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E23" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B24" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C24" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D24" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E24" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B25" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C25" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D25" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E25" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B26" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C26" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D26" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E26" t="s">
         <v>6</v>
@@ -5393,84 +5396,84 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C27" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D27" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E27" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B28" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C28" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D28" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E28" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B29" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C29" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D29" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E29" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B30" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C30" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D30" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E30" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B31" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C31" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D31" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E31" t="s">
         <v>6</v>
@@ -5478,84 +5481,84 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B32" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C32" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D32" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E32" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B33" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C33" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E33" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B34" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C34" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D34" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E34" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C35" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D35" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B36" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C36" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D36" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E36" t="s">
         <v>6</v>
@@ -5563,84 +5566,84 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B37" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C37" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D37" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E37" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B38" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C38" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D38" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E38" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B39" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C39" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D39" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E39" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B40" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C40" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D40" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E40" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B41" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C41" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D41" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E41" t="s">
         <v>6</v>
@@ -5648,84 +5651,84 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B42" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C42" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D42" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E42" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B43" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C43" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D43" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E43" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B44" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C44" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D44" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E44" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B45" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C45" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D45" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E45" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B46" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C46" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D46" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E46" t="s">
         <v>6</v>
@@ -5733,84 +5736,84 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B47" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C47" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D47" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E47" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B48" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C48" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D48" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E48" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B49" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C49" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D49" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E49" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B50" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C50" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D50" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E50" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B51" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C51" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D51" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E51" t="s">
         <v>6</v>
@@ -5818,70 +5821,70 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B52" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C52" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D52" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E52" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B53" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C53" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D53" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E53" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B54" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C54" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D54" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E54" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B55" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C55" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D55" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E55" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -5902,44 +5905,44 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>32</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -5961,30 +5964,30 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>
@@ -6008,7 +6011,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>33</v>
@@ -6017,19 +6020,19 @@
         <v>32</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>35</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>3</v>
@@ -6037,22 +6040,22 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G2" t="s">
         <v>40</v>
@@ -6066,147 +6069,147 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G3" t="s">
         <v>40</v>
       </c>
       <c r="H3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="I3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B4" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G4" t="s">
         <v>40</v>
       </c>
       <c r="H4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="I4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B5" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C5" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D5" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E5" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F5" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G5" t="s">
         <v>40</v>
       </c>
       <c r="H5" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="I5" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C6" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D6" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E6" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G6" t="s">
         <v>40</v>
       </c>
       <c r="H6" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="I6" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B7" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C7" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D7" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F7" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G7" t="s">
         <v>40</v>
       </c>
       <c r="H7" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="I7" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Admin: update site_settings ads_enabled setting_value and 1 more change
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -100,7 +100,7 @@
     <t>ads_enabled</t>
   </si>
   <si>
-    <t>false</t>
+    <t>2026-10-30T13:19:02Z</t>
   </si>
   <si>
     <t>analytics_measurement_id</t>
@@ -2234,13 +2234,13 @@
         <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C9" t="s">
         <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Admin: update site_settings adsense_publisher_id setting_value
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="523">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1026" uniqueCount="524">
   <si>
     <t>setting_key</t>
   </si>
@@ -116,6 +116,9 @@
   </si>
   <si>
     <t>adsense_publisher_id</t>
+  </si>
+  <si>
+    <t>ca-pub-1899141494693710</t>
   </si>
   <si>
     <t>2026-10-30T10:47:37Z</t>
@@ -2272,11 +2275,14 @@
       <c r="A12" t="s">
         <v>29</v>
       </c>
+      <c r="B12" t="s">
+        <v>30</v>
+      </c>
       <c r="C12" t="s">
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -2297,1242 +2303,1242 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E3" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B4" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E4" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B5" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E5" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F5" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B6" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E6" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B7" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E7" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F7" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B8" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E8" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F8" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B9" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C9">
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E9" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B10" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C10">
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E10" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B11" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C11">
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B12" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C12">
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F12" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B13" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C13">
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F13" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B14" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C14">
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E14" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F14" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B15" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C15">
         <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E15" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F15" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B16" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C16">
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E16" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F16" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B17" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E17" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B18" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C18">
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E18" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F18" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B19" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E19" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F19" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B20" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C20">
         <v>4</v>
       </c>
       <c r="D20" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E20" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F20" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B21" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C21">
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E21" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F21" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B22" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C22">
         <v>6</v>
       </c>
       <c r="D22" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E22" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F22" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B23" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C23">
         <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E23" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F23" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B24" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C24">
         <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E24" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F24" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B25" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C25">
         <v>9</v>
       </c>
       <c r="D25" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E25" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F25" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B26" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C26">
         <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E26" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F26" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B27" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C27">
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E27" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F27" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B28" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C28">
         <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E28" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F28" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B29" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E29" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F29" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B30" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C30">
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E30" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F30" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B31" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C31">
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E31" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F31" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B32" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C32">
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E32" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F32" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B33" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C33">
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E33" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B34" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C34">
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E34" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F34" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B35" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C35">
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E35" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F35" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B36" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C36">
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E36" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="F36" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B37" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C37">
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E37" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F37" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B38" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C38">
         <v>10</v>
       </c>
       <c r="D38" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E38" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F38" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B39" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C39">
         <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E39" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F39" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B40" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C40">
         <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E40" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F40" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B41" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C41">
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E41" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F41" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B42" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C42">
         <v>2</v>
       </c>
       <c r="D42" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E42" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F42" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B43" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C43">
         <v>3</v>
       </c>
       <c r="D43" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E43" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="F43" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B44" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C44">
         <v>4</v>
       </c>
       <c r="D44" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E44" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F44" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B45" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C45">
         <v>5</v>
       </c>
       <c r="D45" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E45" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F45" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B46" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C46">
         <v>6</v>
       </c>
       <c r="D46" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E46" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F46" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B47" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C47">
         <v>7</v>
       </c>
       <c r="D47" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E47" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F47" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B48" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C48">
         <v>8</v>
       </c>
       <c r="D48" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E48" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F48" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B49" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C49">
         <v>9</v>
       </c>
       <c r="D49" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E49" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="F49" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B50" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C50">
         <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E50" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F50" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B51" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C51">
         <v>11</v>
       </c>
       <c r="D51" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E51" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="F51" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B52" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C52">
         <v>12</v>
       </c>
       <c r="D52" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E52" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F52" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B53" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C53">
         <v>1</v>
       </c>
       <c r="D53" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E53" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="F53" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B54" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C54">
         <v>2</v>
       </c>
       <c r="D54" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E54" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F54" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B55" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C55">
         <v>3</v>
       </c>
       <c r="D55" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E55" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="F55" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B56" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C56">
         <v>4</v>
       </c>
       <c r="D56" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E56" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F56" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B57" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C57">
         <v>5</v>
       </c>
       <c r="D57" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E57" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="F57" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B58" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C58">
         <v>6</v>
       </c>
       <c r="D58" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E58" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F58" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B59" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C59">
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E59" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="F59" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B60" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C60">
         <v>8</v>
       </c>
       <c r="D60" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E60" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F60" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B61" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C61">
         <v>9</v>
       </c>
       <c r="D61" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E61" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="F61" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B62" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C62">
         <v>10</v>
       </c>
       <c r="D62" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E62" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F62" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -3552,79 +3558,79 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B2" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C2" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B3" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C3" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C4" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B5" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C5" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B6" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C6" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B7" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C7" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
   </sheetData>
@@ -3644,123 +3650,123 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C2" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C3" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B4" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C4" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B5" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C5" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C6" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B7" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C7" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B8" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C8" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B9" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C9" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C10" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
   </sheetData>
@@ -3785,45 +3791,45 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D2" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="E2" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="F2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G2" t="b">
         <v>0</v>
@@ -3831,22 +3837,22 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B3" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D3" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E3" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G3" t="b">
         <v>0</v>
@@ -3854,22 +3860,22 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B4" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C4" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E4" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G4" t="b">
         <v>0</v>
@@ -3877,22 +3883,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B5" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C5" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D5" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E5" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="F5" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G5" t="b">
         <v>0</v>
@@ -3900,22 +3906,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B6" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D6" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="E6" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="F6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G6" t="b">
         <v>0</v>
@@ -3923,22 +3929,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B7" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C7" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D7" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E7" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="F7" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G7" t="b">
         <v>0</v>
@@ -3946,22 +3952,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B8" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C8" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D8" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E8" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F8" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G8" t="b">
         <v>0</v>
@@ -3969,22 +3975,22 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B9" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E9" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G9" t="b">
         <v>0</v>
@@ -4008,81 +4014,81 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="B2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C2" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="D2" t="b">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B3" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C3" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D3" t="b">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B4" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="C4" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B5" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="C5" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="D5" t="b">
         <v>0</v>
@@ -4090,13 +4096,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B6" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C6" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="D6" t="b">
         <v>0</v>
@@ -4104,13 +4110,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C7" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D7" t="b">
         <v>0</v>
@@ -4136,33 +4142,33 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B2" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="C2" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="D2" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -4196,10 +4202,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -4226,19 +4232,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4246,19 +4252,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F2" t="s">
         <v>7</v>
@@ -4266,39 +4272,39 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" t="s">
         <v>41</v>
       </c>
-      <c r="B3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E3" t="s">
-        <v>40</v>
-      </c>
       <c r="F3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F4" t="s">
         <v>19</v>
@@ -4306,19 +4312,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F5" t="s">
         <v>19</v>
@@ -4344,36 +4350,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -4384,16 +4390,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" t="s">
         <v>64</v>
-      </c>
-      <c r="B3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D3" t="s">
-        <v>63</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -4404,16 +4410,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -4424,16 +4430,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -4444,16 +4450,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -4464,16 +4470,16 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D7" t="s">
         <v>77</v>
-      </c>
-      <c r="B7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C7" t="s">
-        <v>78</v>
-      </c>
-      <c r="D7" t="s">
-        <v>76</v>
       </c>
       <c r="E7">
         <v>2</v>
@@ -4501,36 +4507,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -4541,16 +4547,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -4561,16 +4567,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -4581,16 +4587,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -4621,54 +4627,54 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F2" t="s">
         <v>104</v>
       </c>
-      <c r="F2" t="s">
-        <v>103</v>
-      </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -4679,25 +4685,25 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F3" t="s">
         <v>108</v>
       </c>
-      <c r="F3" t="s">
-        <v>107</v>
-      </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H3" t="b">
         <v>0</v>
@@ -4708,25 +4714,25 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E4" t="s">
+        <v>113</v>
+      </c>
+      <c r="F4" t="s">
         <v>112</v>
       </c>
-      <c r="F4" t="s">
-        <v>111</v>
-      </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
@@ -4737,25 +4743,25 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E5" t="s">
+        <v>117</v>
+      </c>
+      <c r="F5" t="s">
         <v>116</v>
       </c>
-      <c r="F5" t="s">
-        <v>115</v>
-      </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -4766,25 +4772,25 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E6" t="s">
+        <v>121</v>
+      </c>
+      <c r="F6" t="s">
         <v>120</v>
       </c>
-      <c r="F6" t="s">
-        <v>119</v>
-      </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -4795,25 +4801,25 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E7" t="s">
+        <v>125</v>
+      </c>
+      <c r="F7" t="s">
         <v>124</v>
       </c>
-      <c r="F7" t="s">
-        <v>123</v>
-      </c>
       <c r="G7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
@@ -4824,25 +4830,25 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E8" t="s">
+        <v>129</v>
+      </c>
+      <c r="F8" t="s">
         <v>128</v>
       </c>
-      <c r="F8" t="s">
-        <v>127</v>
-      </c>
       <c r="G8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
@@ -4853,25 +4859,25 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D9" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E9" t="s">
+        <v>133</v>
+      </c>
+      <c r="F9" t="s">
         <v>132</v>
       </c>
-      <c r="F9" t="s">
-        <v>131</v>
-      </c>
       <c r="G9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H9" t="b">
         <v>1</v>
@@ -4882,25 +4888,25 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E10" t="s">
+        <v>137</v>
+      </c>
+      <c r="F10" t="s">
         <v>136</v>
       </c>
-      <c r="F10" t="s">
-        <v>135</v>
-      </c>
       <c r="G10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -4911,25 +4917,25 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B11" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C11" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E11" t="s">
+        <v>141</v>
+      </c>
+      <c r="F11" t="s">
         <v>140</v>
       </c>
-      <c r="F11" t="s">
-        <v>139</v>
-      </c>
       <c r="G11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H11" t="b">
         <v>0</v>
@@ -4957,10 +4963,10 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -4974,50 +4980,50 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" t="s">
+        <v>148</v>
+      </c>
+      <c r="D3" t="s">
+        <v>149</v>
+      </c>
+      <c r="E3" t="s">
         <v>146</v>
-      </c>
-      <c r="B3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C3" t="s">
-        <v>147</v>
-      </c>
-      <c r="D3" t="s">
-        <v>148</v>
-      </c>
-      <c r="E3" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E4" t="s">
         <v>6</v>
@@ -5025,33 +5031,33 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E6" t="s">
         <v>6</v>
@@ -5059,84 +5065,84 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>163</v>
+      </c>
+      <c r="B8" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" t="s">
+        <v>164</v>
+      </c>
+      <c r="D8" t="s">
+        <v>165</v>
+      </c>
+      <c r="E8" t="s">
         <v>162</v>
-      </c>
-      <c r="B8" t="s">
-        <v>101</v>
-      </c>
-      <c r="C8" t="s">
-        <v>163</v>
-      </c>
-      <c r="D8" t="s">
-        <v>164</v>
-      </c>
-      <c r="E8" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C9" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D9" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E9" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C11" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E11" t="s">
         <v>6</v>
@@ -5144,84 +5150,84 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C12" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E12" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D13" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D14" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E14" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D15" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E15" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C16" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D16" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E16" t="s">
         <v>6</v>
@@ -5229,84 +5235,84 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C17" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E17" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C18" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D18" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E18" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B19" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D19" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E19" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B20" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C20" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D20" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E20" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B21" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C21" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D21" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E21" t="s">
         <v>6</v>
@@ -5314,84 +5320,84 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B22" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C22" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D22" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E22" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B23" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C23" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D23" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E23" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B24" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C24" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D24" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E24" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B25" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C25" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D25" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E25" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B26" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C26" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D26" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E26" t="s">
         <v>6</v>
@@ -5399,84 +5405,84 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C27" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D27" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E27" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B28" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C28" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D28" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E28" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B29" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C29" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D29" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E29" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B30" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C30" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D30" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E30" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B31" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C31" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D31" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E31" t="s">
         <v>6</v>
@@ -5484,84 +5490,84 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B32" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C32" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D32" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E32" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B33" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C33" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E33" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B34" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C34" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D34" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E34" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B35" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C35" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D35" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E35" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B36" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C36" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D36" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E36" t="s">
         <v>6</v>
@@ -5569,84 +5575,84 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B37" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C37" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D37" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E37" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B38" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C38" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D38" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B39" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C39" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D39" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E39" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B40" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C40" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D40" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E40" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B41" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C41" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D41" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E41" t="s">
         <v>6</v>
@@ -5654,84 +5660,84 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B42" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C42" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D42" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E42" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B43" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C43" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D43" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E43" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B44" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C44" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D44" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E44" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B45" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C45" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D45" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E45" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B46" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C46" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D46" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E46" t="s">
         <v>6</v>
@@ -5739,84 +5745,84 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B47" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C47" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D47" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E47" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B48" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C48" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D48" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E48" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B49" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C49" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D49" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E49" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B50" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C50" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D50" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E50" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B51" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C51" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D51" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E51" t="s">
         <v>6</v>
@@ -5824,70 +5830,70 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B52" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C52" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D52" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E52" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B53" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C53" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D53" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E53" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B54" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C54" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D54" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E54" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B55" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C55" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D55" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E55" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -5908,44 +5914,44 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -5967,30 +5973,30 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -6014,28 +6020,28 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>3</v>
@@ -6043,25 +6049,25 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H2" t="s">
         <v>7</v>
@@ -6072,147 +6078,147 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F3" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="I3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E4" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F4" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="I4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B5" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C5" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D5" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E5" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F5" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H5" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="I5" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B6" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C6" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D6" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="I6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B7" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C7" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D7" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E7" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F7" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H7" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="I7" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Admin: update advertisements AD0002 enabled and 1 more change
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1026" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1026" uniqueCount="523">
   <si>
     <t>setting_key</t>
   </si>
@@ -1668,9 +1668,6 @@
   </si>
   <si>
     <t>below_tool</t>
-  </si>
-  <si>
-    <t>1899141494693710</t>
   </si>
   <si>
     <t>AD0003</t>
@@ -4057,21 +4054,21 @@
         <v>474</v>
       </c>
       <c r="D3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>504</v>
+        <v>274</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>504</v>
+      </c>
+      <c r="B4" t="s">
         <v>505</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>506</v>
-      </c>
-      <c r="C4" t="s">
-        <v>507</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
@@ -4082,10 +4079,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>507</v>
+      </c>
+      <c r="B5" t="s">
         <v>508</v>
-      </c>
-      <c r="B5" t="s">
-        <v>509</v>
       </c>
       <c r="C5" t="s">
         <v>501</v>
@@ -4096,13 +4093,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>509</v>
+      </c>
+      <c r="B6" t="s">
         <v>510</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>511</v>
-      </c>
-      <c r="C6" t="s">
-        <v>512</v>
       </c>
       <c r="D6" t="b">
         <v>0</v>
@@ -4110,13 +4107,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>512</v>
+      </c>
+      <c r="B7" t="s">
+        <v>510</v>
+      </c>
+      <c r="C7" t="s">
         <v>513</v>
-      </c>
-      <c r="B7" t="s">
-        <v>511</v>
-      </c>
-      <c r="C7" t="s">
-        <v>514</v>
       </c>
       <c r="D7" t="b">
         <v>0</v>
@@ -4142,16 +4139,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>515</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>516</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>517</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>518</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>60</v>
@@ -4159,16 +4156,16 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>518</v>
+      </c>
+      <c r="B2" t="s">
         <v>519</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>520</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>521</v>
-      </c>
-      <c r="D2" t="s">
-        <v>522</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -4202,7 +4199,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B2" t="s">
         <v>145</v>

</xml_diff>

<commit_message>
Admin: update site_settings analytics_measurement_id setting_value
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1026" uniqueCount="523">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1027" uniqueCount="524">
   <si>
     <t>setting_key</t>
   </si>
@@ -104,6 +104,9 @@
   </si>
   <si>
     <t>analytics_measurement_id</t>
+  </si>
+  <si>
+    <t>G-EN8KN5P8X6</t>
   </si>
   <si>
     <t>2026-10-30T08:39:16Z</t>
@@ -2250,36 +2253,39 @@
       <c r="A10" t="s">
         <v>25</v>
       </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
       <c r="C10" t="s">
         <v>6</v>
       </c>
       <c r="D10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
         <v>6</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -2300,1242 +2306,1242 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E3" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B4" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E4" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B5" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E5" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F5" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E6" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B7" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E7" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F7" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E8" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F8" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B9" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C9">
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E9" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F9" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B10" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C10">
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E10" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F10" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B11" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C11">
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E11" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F11" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B12" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C12">
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F12" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B13" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C13">
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E13" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F13" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B14" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C14">
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E14" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F14" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B15" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C15">
         <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E15" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F15" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B16" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C16">
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E16" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F16" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B17" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E17" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B18" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C18">
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E18" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F18" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B19" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E19" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F19" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B20" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C20">
         <v>4</v>
       </c>
       <c r="D20" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E20" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="F20" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B21" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C21">
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E21" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F21" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B22" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C22">
         <v>6</v>
       </c>
       <c r="D22" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E22" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F22" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B23" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C23">
         <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E23" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F23" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B24" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C24">
         <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E24" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F24" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B25" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C25">
         <v>9</v>
       </c>
       <c r="D25" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E25" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F25" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B26" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C26">
         <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E26" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="F26" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B27" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C27">
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E27" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F27" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B28" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C28">
         <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E28" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F28" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B29" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E29" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F29" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B30" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C30">
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E30" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F30" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B31" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C31">
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E31" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F31" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B32" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C32">
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E32" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F32" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B33" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C33">
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E33" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B34" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C34">
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E34" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F34" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B35" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C35">
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E35" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F35" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B36" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C36">
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E36" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F36" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B37" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C37">
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E37" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F37" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B38" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C38">
         <v>10</v>
       </c>
       <c r="D38" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E38" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="F38" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B39" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C39">
         <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E39" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F39" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B40" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C40">
         <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E40" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F40" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B41" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C41">
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E41" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F41" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B42" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C42">
         <v>2</v>
       </c>
       <c r="D42" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E42" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="F42" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B43" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C43">
         <v>3</v>
       </c>
       <c r="D43" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E43" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F43" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B44" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C44">
         <v>4</v>
       </c>
       <c r="D44" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E44" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="F44" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B45" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C45">
         <v>5</v>
       </c>
       <c r="D45" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E45" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F45" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B46" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C46">
         <v>6</v>
       </c>
       <c r="D46" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E46" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F46" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B47" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C47">
         <v>7</v>
       </c>
       <c r="D47" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E47" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F47" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B48" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C48">
         <v>8</v>
       </c>
       <c r="D48" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E48" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F48" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B49" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C49">
         <v>9</v>
       </c>
       <c r="D49" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E49" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F49" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B50" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C50">
         <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E50" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="F50" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B51" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C51">
         <v>11</v>
       </c>
       <c r="D51" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E51" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="F51" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B52" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C52">
         <v>12</v>
       </c>
       <c r="D52" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E52" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="F52" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B53" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C53">
         <v>1</v>
       </c>
       <c r="D53" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E53" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F53" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B54" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C54">
         <v>2</v>
       </c>
       <c r="D54" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E54" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F54" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B55" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C55">
         <v>3</v>
       </c>
       <c r="D55" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E55" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="F55" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B56" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C56">
         <v>4</v>
       </c>
       <c r="D56" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E56" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="F56" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B57" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C57">
         <v>5</v>
       </c>
       <c r="D57" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E57" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="F57" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B58" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C58">
         <v>6</v>
       </c>
       <c r="D58" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E58" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F58" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B59" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C59">
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E59" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F59" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B60" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C60">
         <v>8</v>
       </c>
       <c r="D60" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E60" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F60" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B61" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C61">
         <v>9</v>
       </c>
       <c r="D61" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E61" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="F61" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B62" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C62">
         <v>10</v>
       </c>
       <c r="D62" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E62" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F62" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -3555,79 +3561,79 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B2" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C2" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B3" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C3" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B4" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C4" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B5" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C5" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B6" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C6" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B7" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C7" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
   </sheetData>
@@ -3647,123 +3653,123 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C2" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C3" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B5" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C5" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C6" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B7" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C7" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B8" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C8" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B9" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C9" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B10" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C10" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
   </sheetData>
@@ -3788,45 +3794,45 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B2" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D2" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="E2" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G2" t="b">
         <v>0</v>
@@ -3834,22 +3840,22 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B3" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D3" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E3" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G3" t="b">
         <v>0</v>
@@ -3857,22 +3863,22 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B4" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D4" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E4" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G4" t="b">
         <v>0</v>
@@ -3880,22 +3886,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B5" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C5" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D5" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E5" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F5" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G5" t="b">
         <v>0</v>
@@ -3903,22 +3909,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B6" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C6" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D6" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E6" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G6" t="b">
         <v>0</v>
@@ -3926,22 +3932,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B7" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C7" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D7" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E7" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="F7" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G7" t="b">
         <v>0</v>
@@ -3949,22 +3955,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B8" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C8" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D8" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E8" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F8" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G8" t="b">
         <v>0</v>
@@ -3972,22 +3978,22 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B9" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E9" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F9" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G9" t="b">
         <v>0</v>
@@ -4011,81 +4017,81 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B2" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C2" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="D2" t="b">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B3" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C3" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="D3" t="b">
         <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B4" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="C4" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B5" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="C5" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="D5" t="b">
         <v>0</v>
@@ -4093,13 +4099,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B6" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C6" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="D6" t="b">
         <v>0</v>
@@ -4107,13 +4113,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C7" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D7" t="b">
         <v>0</v>
@@ -4139,33 +4145,33 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B2" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="C2" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="D2" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -4199,10 +4205,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -4229,19 +4235,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4249,19 +4255,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F2" t="s">
         <v>7</v>
@@ -4269,39 +4275,39 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" t="s">
         <v>42</v>
       </c>
-      <c r="B3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E3" t="s">
-        <v>41</v>
-      </c>
       <c r="F3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F4" t="s">
         <v>19</v>
@@ -4309,19 +4315,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F5" t="s">
         <v>19</v>
@@ -4347,36 +4353,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -4387,16 +4393,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" t="s">
         <v>65</v>
-      </c>
-      <c r="B3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C3" t="s">
-        <v>67</v>
-      </c>
-      <c r="D3" t="s">
-        <v>64</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -4407,16 +4413,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -4427,16 +4433,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -4447,16 +4453,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -4467,16 +4473,16 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" t="s">
         <v>78</v>
-      </c>
-      <c r="B7" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" t="s">
-        <v>79</v>
-      </c>
-      <c r="D7" t="s">
-        <v>77</v>
       </c>
       <c r="E7">
         <v>2</v>
@@ -4504,36 +4510,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -4544,16 +4550,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -4564,16 +4570,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -4584,16 +4590,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -4624,54 +4630,54 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F2" t="s">
         <v>105</v>
       </c>
-      <c r="F2" t="s">
-        <v>104</v>
-      </c>
       <c r="G2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -4682,25 +4688,25 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F3" t="s">
         <v>109</v>
       </c>
-      <c r="F3" t="s">
-        <v>108</v>
-      </c>
       <c r="G3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H3" t="b">
         <v>0</v>
@@ -4711,25 +4717,25 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E4" t="s">
+        <v>114</v>
+      </c>
+      <c r="F4" t="s">
         <v>113</v>
       </c>
-      <c r="F4" t="s">
-        <v>112</v>
-      </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
@@ -4740,25 +4746,25 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E5" t="s">
+        <v>118</v>
+      </c>
+      <c r="F5" t="s">
         <v>117</v>
       </c>
-      <c r="F5" t="s">
-        <v>116</v>
-      </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -4769,25 +4775,25 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E6" t="s">
+        <v>122</v>
+      </c>
+      <c r="F6" t="s">
         <v>121</v>
       </c>
-      <c r="F6" t="s">
-        <v>120</v>
-      </c>
       <c r="G6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -4798,25 +4804,25 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F7" t="s">
         <v>125</v>
       </c>
-      <c r="F7" t="s">
-        <v>124</v>
-      </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
@@ -4827,25 +4833,25 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E8" t="s">
+        <v>130</v>
+      </c>
+      <c r="F8" t="s">
         <v>129</v>
       </c>
-      <c r="F8" t="s">
-        <v>128</v>
-      </c>
       <c r="G8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
@@ -4856,25 +4862,25 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C9" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D9" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E9" t="s">
+        <v>134</v>
+      </c>
+      <c r="F9" t="s">
         <v>133</v>
       </c>
-      <c r="F9" t="s">
-        <v>132</v>
-      </c>
       <c r="G9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H9" t="b">
         <v>1</v>
@@ -4885,25 +4891,25 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E10" t="s">
+        <v>138</v>
+      </c>
+      <c r="F10" t="s">
         <v>137</v>
       </c>
-      <c r="F10" t="s">
-        <v>136</v>
-      </c>
       <c r="G10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -4914,25 +4920,25 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D11" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E11" t="s">
+        <v>142</v>
+      </c>
+      <c r="F11" t="s">
         <v>141</v>
       </c>
-      <c r="F11" t="s">
-        <v>140</v>
-      </c>
       <c r="G11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H11" t="b">
         <v>0</v>
@@ -4960,10 +4966,10 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -4977,50 +4983,50 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" t="s">
+        <v>149</v>
+      </c>
+      <c r="D3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E3" t="s">
         <v>147</v>
-      </c>
-      <c r="B3" t="s">
-        <v>102</v>
-      </c>
-      <c r="C3" t="s">
-        <v>148</v>
-      </c>
-      <c r="D3" t="s">
-        <v>149</v>
-      </c>
-      <c r="E3" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E4" t="s">
         <v>6</v>
@@ -5028,33 +5034,33 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E6" t="s">
         <v>6</v>
@@ -5062,84 +5068,84 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>164</v>
+      </c>
+      <c r="B8" t="s">
+        <v>103</v>
+      </c>
+      <c r="C8" t="s">
+        <v>165</v>
+      </c>
+      <c r="D8" t="s">
+        <v>166</v>
+      </c>
+      <c r="E8" t="s">
         <v>163</v>
-      </c>
-      <c r="B8" t="s">
-        <v>102</v>
-      </c>
-      <c r="C8" t="s">
-        <v>164</v>
-      </c>
-      <c r="D8" t="s">
-        <v>165</v>
-      </c>
-      <c r="E8" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C9" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D9" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E9" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E11" t="s">
         <v>6</v>
@@ -5147,84 +5153,84 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C12" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C13" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D13" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C14" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D14" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E14" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B15" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C15" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E15" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C16" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D16" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E16" t="s">
         <v>6</v>
@@ -5232,84 +5238,84 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C17" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E17" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C18" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D18" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E18" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B19" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C19" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D19" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E19" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B20" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C20" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D20" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E20" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B21" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C21" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D21" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E21" t="s">
         <v>6</v>
@@ -5317,84 +5323,84 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B22" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C22" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D22" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E22" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B23" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C23" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D23" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E23" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B24" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C24" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D24" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E24" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B25" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C25" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D25" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E25" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B26" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D26" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E26" t="s">
         <v>6</v>
@@ -5402,84 +5408,84 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C27" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D27" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E27" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B28" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C28" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E28" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B29" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C29" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D29" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E29" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B30" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C30" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D30" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E30" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B31" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C31" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D31" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E31" t="s">
         <v>6</v>
@@ -5487,84 +5493,84 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B32" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C32" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D32" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E32" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B33" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C33" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E33" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B34" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C34" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D34" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E34" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B35" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C35" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D35" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B36" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C36" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D36" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E36" t="s">
         <v>6</v>
@@ -5572,84 +5578,84 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B37" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C37" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D37" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E37" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B38" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C38" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D38" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E38" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B39" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C39" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D39" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E39" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B40" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C40" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D40" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E40" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B41" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C41" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D41" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E41" t="s">
         <v>6</v>
@@ -5657,84 +5663,84 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B42" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C42" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D42" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E42" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B43" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C43" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D43" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E43" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B44" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C44" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D44" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E44" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B45" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C45" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D45" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E45" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B46" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C46" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D46" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E46" t="s">
         <v>6</v>
@@ -5742,84 +5748,84 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B47" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C47" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D47" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E47" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B48" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C48" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D48" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E48" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B49" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C49" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D49" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E49" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B50" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C50" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D50" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E50" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B51" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C51" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D51" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E51" t="s">
         <v>6</v>
@@ -5827,70 +5833,70 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B52" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C52" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D52" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E52" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B53" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C53" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D53" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E53" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B54" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C54" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D54" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E54" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B55" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C55" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D55" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E55" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -5911,44 +5917,44 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -5970,30 +5976,30 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -6017,28 +6023,28 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>3</v>
@@ -6046,25 +6052,25 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
         <v>7</v>
@@ -6075,147 +6081,147 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="I3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F4" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H4" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="I4" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B5" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C5" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D5" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E5" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="I5" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B6" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C6" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E6" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="I6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B7" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C7" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D7" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E7" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F7" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H7" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="I7" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Article images: covers, captions, schema 1.0.2 with migration, image sizes and srcset (T9.7)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1027" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1042" uniqueCount="539">
   <si>
     <t>setting_key</t>
   </si>
@@ -43,7 +43,7 @@
     <t>schema_version</t>
   </si>
   <si>
-    <t>1.0.1</t>
+    <t>1.0.2</t>
   </si>
   <si>
     <t>string</t>
@@ -982,6 +982,12 @@
     <t>published_at</t>
   </si>
   <si>
+    <t>cover_image</t>
+  </si>
+  <si>
+    <t>cover_alt</t>
+  </si>
+  <si>
     <t>POST0001</t>
   </si>
   <si>
@@ -994,6 +1000,12 @@
     <t>Understand the formula behind your loan EMI and how interest and tenure change what you pay.</t>
   </si>
   <si>
+    <t>/images/blog/how-emi-is-calculated/cover-1600.jpg</t>
+  </si>
+  <si>
+    <t>Abstract artwork in dark purple with orange and gold glow</t>
+  </si>
+  <si>
     <t>POST0002</t>
   </si>
   <si>
@@ -1009,6 +1021,12 @@
     <t>2026-10-12T09:00:00Z</t>
   </si>
   <si>
+    <t>/images/blog/compress-images-without-losing-quality/cover-1600.jpg</t>
+  </si>
+  <si>
+    <t>Abstract artwork in navy blue with sky blue and teal light</t>
+  </si>
+  <si>
     <t>POST0003</t>
   </si>
   <si>
@@ -1024,6 +1042,12 @@
     <t>2026-10-16T09:00:00Z</t>
   </si>
   <si>
+    <t>/images/blog/gst-explained-add-and-remove-gst/cover-1600.jpg</t>
+  </si>
+  <si>
+    <t>Abstract artwork in deep red with peach and coral glow</t>
+  </si>
+  <si>
     <t>POST0004</t>
   </si>
   <si>
@@ -1039,6 +1063,12 @@
     <t>2026-10-20T09:00:00Z</t>
   </si>
   <si>
+    <t>/images/blog/fixed-deposit-interest-simple-vs-compound/cover-1600.jpg</t>
+  </si>
+  <si>
+    <t>Abstract artwork in forest green with mint and gold light</t>
+  </si>
+  <si>
     <t>POST0005</t>
   </si>
   <si>
@@ -1054,6 +1084,12 @@
     <t>2026-10-24T09:00:00Z</t>
   </si>
   <si>
+    <t>/images/blog/make-a-qr-code-that-scans-every-time/cover-1600.jpg</t>
+  </si>
+  <si>
+    <t>Abstract artwork in indigo with lilac and teal light</t>
+  </si>
+  <si>
     <t>POST0006</t>
   </si>
   <si>
@@ -1069,6 +1105,12 @@
     <t>2026-10-28T09:00:00Z</t>
   </si>
   <si>
+    <t>/images/blog/why-browser-based-tools-keep-your-files-private/cover-1600.jpg</t>
+  </si>
+  <si>
+    <t>Abstract artwork in deep green with soft gold and teal light</t>
+  </si>
+  <si>
     <t>block_id</t>
   </si>
   <si>
@@ -1076,6 +1118,9 @@
   </si>
   <si>
     <t>asset_path</t>
+  </si>
+  <si>
+    <t>caption</t>
   </si>
   <si>
     <t>BLK00001</t>
@@ -2296,17 +2341,18 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>308</v>
+        <v>322</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>276</v>
@@ -2315,30 +2361,33 @@
         <v>60</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>309</v>
+        <v>323</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>310</v>
+        <v>324</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>311</v>
+        <v>326</v>
       </c>
       <c r="B2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E2" t="s">
-        <v>313</v>
+        <v>328</v>
       </c>
       <c r="F2" t="s">
         <v>275</v>
@@ -2346,19 +2395,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>314</v>
+        <v>329</v>
       </c>
       <c r="B3" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E3" t="s">
-        <v>316</v>
+        <v>331</v>
       </c>
       <c r="F3" t="s">
         <v>275</v>
@@ -2366,19 +2415,19 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>317</v>
+        <v>332</v>
       </c>
       <c r="B4" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E4" t="s">
-        <v>318</v>
+        <v>333</v>
       </c>
       <c r="F4" t="s">
         <v>275</v>
@@ -2386,19 +2435,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>319</v>
+        <v>334</v>
       </c>
       <c r="B5" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E5" t="s">
-        <v>320</v>
+        <v>335</v>
       </c>
       <c r="F5" t="s">
         <v>275</v>
@@ -2406,19 +2455,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>321</v>
+        <v>336</v>
       </c>
       <c r="B6" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="E6" t="s">
-        <v>323</v>
+        <v>338</v>
       </c>
       <c r="F6" t="s">
         <v>275</v>
@@ -2426,19 +2475,19 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>324</v>
+        <v>339</v>
       </c>
       <c r="B7" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E7" t="s">
-        <v>325</v>
+        <v>340</v>
       </c>
       <c r="F7" t="s">
         <v>275</v>
@@ -2446,19 +2495,19 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>326</v>
+        <v>341</v>
       </c>
       <c r="B8" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E8" t="s">
-        <v>327</v>
+        <v>342</v>
       </c>
       <c r="F8" t="s">
         <v>275</v>
@@ -2466,19 +2515,19 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="B9" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C9">
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E9" t="s">
-        <v>329</v>
+        <v>344</v>
       </c>
       <c r="F9" t="s">
         <v>275</v>
@@ -2486,19 +2535,19 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>330</v>
+        <v>345</v>
       </c>
       <c r="B10" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C10">
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E10" t="s">
-        <v>331</v>
+        <v>346</v>
       </c>
       <c r="F10" t="s">
         <v>275</v>
@@ -2506,19 +2555,19 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>332</v>
+        <v>347</v>
       </c>
       <c r="B11" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C11">
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="E11" t="s">
-        <v>333</v>
+        <v>348</v>
       </c>
       <c r="F11" t="s">
         <v>275</v>
@@ -2526,19 +2575,19 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>334</v>
+        <v>349</v>
       </c>
       <c r="B12" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C12">
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E12" t="s">
-        <v>335</v>
+        <v>350</v>
       </c>
       <c r="F12" t="s">
         <v>275</v>
@@ -2546,19 +2595,19 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>336</v>
+        <v>351</v>
       </c>
       <c r="B13" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C13">
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E13" t="s">
-        <v>337</v>
+        <v>352</v>
       </c>
       <c r="F13" t="s">
         <v>275</v>
@@ -2566,19 +2615,19 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>338</v>
+        <v>353</v>
       </c>
       <c r="B14" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C14">
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>339</v>
+        <v>354</v>
       </c>
       <c r="E14" t="s">
-        <v>340</v>
+        <v>355</v>
       </c>
       <c r="F14" t="s">
         <v>275</v>
@@ -2586,19 +2635,19 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>341</v>
+        <v>356</v>
       </c>
       <c r="B15" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C15">
         <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E15" t="s">
-        <v>342</v>
+        <v>357</v>
       </c>
       <c r="F15" t="s">
         <v>275</v>
@@ -2606,19 +2655,19 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>343</v>
+        <v>358</v>
       </c>
       <c r="B16" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C16">
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E16" t="s">
-        <v>344</v>
+        <v>359</v>
       </c>
       <c r="F16" t="s">
         <v>275</v>
@@ -2626,19 +2675,19 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>345</v>
+        <v>360</v>
       </c>
       <c r="B17" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E17" t="s">
-        <v>346</v>
+        <v>361</v>
       </c>
       <c r="F17" t="s">
         <v>275</v>
@@ -2646,19 +2695,19 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>347</v>
+        <v>362</v>
       </c>
       <c r="B18" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C18">
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E18" t="s">
-        <v>348</v>
+        <v>363</v>
       </c>
       <c r="F18" t="s">
         <v>275</v>
@@ -2666,19 +2715,19 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>349</v>
+        <v>364</v>
       </c>
       <c r="B19" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E19" t="s">
-        <v>350</v>
+        <v>365</v>
       </c>
       <c r="F19" t="s">
         <v>275</v>
@@ -2686,19 +2735,19 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>351</v>
+        <v>366</v>
       </c>
       <c r="B20" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C20">
         <v>4</v>
       </c>
       <c r="D20" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E20" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="F20" t="s">
         <v>275</v>
@@ -2706,19 +2755,19 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>353</v>
+        <v>368</v>
       </c>
       <c r="B21" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C21">
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E21" t="s">
-        <v>354</v>
+        <v>369</v>
       </c>
       <c r="F21" t="s">
         <v>275</v>
@@ -2726,19 +2775,19 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>355</v>
+        <v>370</v>
       </c>
       <c r="B22" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C22">
         <v>6</v>
       </c>
       <c r="D22" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E22" t="s">
-        <v>356</v>
+        <v>371</v>
       </c>
       <c r="F22" t="s">
         <v>275</v>
@@ -2746,19 +2795,19 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>357</v>
+        <v>372</v>
       </c>
       <c r="B23" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C23">
         <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E23" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="F23" t="s">
         <v>275</v>
@@ -2766,19 +2815,19 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>359</v>
+        <v>374</v>
       </c>
       <c r="B24" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C24">
         <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E24" t="s">
-        <v>360</v>
+        <v>375</v>
       </c>
       <c r="F24" t="s">
         <v>275</v>
@@ -2786,19 +2835,19 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>361</v>
+        <v>376</v>
       </c>
       <c r="B25" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C25">
         <v>9</v>
       </c>
       <c r="D25" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="E25" t="s">
-        <v>362</v>
+        <v>377</v>
       </c>
       <c r="F25" t="s">
         <v>275</v>
@@ -2806,19 +2855,19 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>363</v>
+        <v>378</v>
       </c>
       <c r="B26" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C26">
         <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E26" t="s">
-        <v>364</v>
+        <v>379</v>
       </c>
       <c r="F26" t="s">
         <v>275</v>
@@ -2826,19 +2875,19 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>365</v>
+        <v>380</v>
       </c>
       <c r="B27" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C27">
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E27" t="s">
-        <v>366</v>
+        <v>381</v>
       </c>
       <c r="F27" t="s">
         <v>275</v>
@@ -2846,19 +2895,19 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>367</v>
+        <v>382</v>
       </c>
       <c r="B28" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C28">
         <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>339</v>
+        <v>354</v>
       </c>
       <c r="E28" t="s">
-        <v>368</v>
+        <v>383</v>
       </c>
       <c r="F28" t="s">
         <v>275</v>
@@ -2866,19 +2915,19 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>369</v>
+        <v>384</v>
       </c>
       <c r="B29" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E29" t="s">
-        <v>370</v>
+        <v>385</v>
       </c>
       <c r="F29" t="s">
         <v>275</v>
@@ -2886,19 +2935,19 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>371</v>
+        <v>386</v>
       </c>
       <c r="B30" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C30">
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E30" t="s">
-        <v>372</v>
+        <v>387</v>
       </c>
       <c r="F30" t="s">
         <v>275</v>
@@ -2906,19 +2955,19 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>373</v>
+        <v>388</v>
       </c>
       <c r="B31" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C31">
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E31" t="s">
-        <v>374</v>
+        <v>389</v>
       </c>
       <c r="F31" t="s">
         <v>275</v>
@@ -2926,19 +2975,19 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>375</v>
+        <v>390</v>
       </c>
       <c r="B32" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C32">
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E32" t="s">
-        <v>376</v>
+        <v>391</v>
       </c>
       <c r="F32" t="s">
         <v>275</v>
@@ -2946,19 +2995,19 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>377</v>
+        <v>392</v>
       </c>
       <c r="B33" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C33">
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E33" t="s">
-        <v>378</v>
+        <v>393</v>
       </c>
       <c r="F33" t="s">
         <v>275</v>
@@ -2966,19 +3015,19 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>379</v>
+        <v>394</v>
       </c>
       <c r="B34" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C34">
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E34" t="s">
-        <v>380</v>
+        <v>395</v>
       </c>
       <c r="F34" t="s">
         <v>275</v>
@@ -2986,19 +3035,19 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>381</v>
+        <v>396</v>
       </c>
       <c r="B35" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C35">
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E35" t="s">
-        <v>382</v>
+        <v>397</v>
       </c>
       <c r="F35" t="s">
         <v>275</v>
@@ -3006,19 +3055,19 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>383</v>
+        <v>398</v>
       </c>
       <c r="B36" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C36">
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E36" t="s">
-        <v>384</v>
+        <v>399</v>
       </c>
       <c r="F36" t="s">
         <v>275</v>
@@ -3026,19 +3075,19 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="B37" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C37">
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E37" t="s">
-        <v>386</v>
+        <v>401</v>
       </c>
       <c r="F37" t="s">
         <v>275</v>
@@ -3046,19 +3095,19 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>387</v>
+        <v>402</v>
       </c>
       <c r="B38" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C38">
         <v>10</v>
       </c>
       <c r="D38" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="E38" t="s">
-        <v>388</v>
+        <v>403</v>
       </c>
       <c r="F38" t="s">
         <v>275</v>
@@ -3066,19 +3115,19 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>389</v>
+        <v>404</v>
       </c>
       <c r="B39" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C39">
         <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E39" t="s">
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="F39" t="s">
         <v>275</v>
@@ -3086,19 +3135,19 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>391</v>
+        <v>406</v>
       </c>
       <c r="B40" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C40">
         <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>339</v>
+        <v>354</v>
       </c>
       <c r="E40" t="s">
-        <v>392</v>
+        <v>407</v>
       </c>
       <c r="F40" t="s">
         <v>275</v>
@@ -3106,19 +3155,19 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>393</v>
+        <v>408</v>
       </c>
       <c r="B41" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="C41">
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E41" t="s">
-        <v>394</v>
+        <v>409</v>
       </c>
       <c r="F41" t="s">
         <v>275</v>
@@ -3126,19 +3175,19 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>395</v>
+        <v>410</v>
       </c>
       <c r="B42" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="C42">
         <v>2</v>
       </c>
       <c r="D42" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E42" t="s">
-        <v>396</v>
+        <v>411</v>
       </c>
       <c r="F42" t="s">
         <v>275</v>
@@ -3146,19 +3195,19 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="B43" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="C43">
         <v>3</v>
       </c>
       <c r="D43" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E43" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="F43" t="s">
         <v>275</v>
@@ -3166,19 +3215,19 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="B44" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="C44">
         <v>4</v>
       </c>
       <c r="D44" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E44" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="F44" t="s">
         <v>275</v>
@@ -3186,19 +3235,19 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>401</v>
+        <v>416</v>
       </c>
       <c r="B45" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="C45">
         <v>5</v>
       </c>
       <c r="D45" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="E45" t="s">
-        <v>402</v>
+        <v>417</v>
       </c>
       <c r="F45" t="s">
         <v>275</v>
@@ -3206,19 +3255,19 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="B46" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="C46">
         <v>6</v>
       </c>
       <c r="D46" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E46" t="s">
-        <v>404</v>
+        <v>419</v>
       </c>
       <c r="F46" t="s">
         <v>275</v>
@@ -3226,19 +3275,19 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>405</v>
+        <v>420</v>
       </c>
       <c r="B47" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="C47">
         <v>7</v>
       </c>
       <c r="D47" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E47" t="s">
-        <v>406</v>
+        <v>421</v>
       </c>
       <c r="F47" t="s">
         <v>275</v>
@@ -3246,19 +3295,19 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>407</v>
+        <v>422</v>
       </c>
       <c r="B48" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="C48">
         <v>8</v>
       </c>
       <c r="D48" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E48" t="s">
-        <v>408</v>
+        <v>423</v>
       </c>
       <c r="F48" t="s">
         <v>275</v>
@@ -3266,19 +3315,19 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>409</v>
+        <v>424</v>
       </c>
       <c r="B49" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="C49">
         <v>9</v>
       </c>
       <c r="D49" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E49" t="s">
-        <v>410</v>
+        <v>425</v>
       </c>
       <c r="F49" t="s">
         <v>275</v>
@@ -3286,19 +3335,19 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>411</v>
+        <v>426</v>
       </c>
       <c r="B50" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="C50">
         <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E50" t="s">
-        <v>412</v>
+        <v>427</v>
       </c>
       <c r="F50" t="s">
         <v>275</v>
@@ -3306,19 +3355,19 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>413</v>
+        <v>428</v>
       </c>
       <c r="B51" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="C51">
         <v>11</v>
       </c>
       <c r="D51" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="E51" t="s">
-        <v>414</v>
+        <v>429</v>
       </c>
       <c r="F51" t="s">
         <v>275</v>
@@ -3326,19 +3375,19 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>415</v>
+        <v>430</v>
       </c>
       <c r="B52" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="C52">
         <v>12</v>
       </c>
       <c r="D52" t="s">
-        <v>339</v>
+        <v>354</v>
       </c>
       <c r="E52" t="s">
-        <v>416</v>
+        <v>431</v>
       </c>
       <c r="F52" t="s">
         <v>275</v>
@@ -3346,19 +3395,19 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>417</v>
+        <v>432</v>
       </c>
       <c r="B53" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="C53">
         <v>1</v>
       </c>
       <c r="D53" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E53" t="s">
-        <v>418</v>
+        <v>433</v>
       </c>
       <c r="F53" t="s">
         <v>275</v>
@@ -3366,19 +3415,19 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>419</v>
+        <v>434</v>
       </c>
       <c r="B54" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="C54">
         <v>2</v>
       </c>
       <c r="D54" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E54" t="s">
-        <v>420</v>
+        <v>435</v>
       </c>
       <c r="F54" t="s">
         <v>275</v>
@@ -3386,19 +3435,19 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>421</v>
+        <v>436</v>
       </c>
       <c r="B55" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="C55">
         <v>3</v>
       </c>
       <c r="D55" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E55" t="s">
-        <v>422</v>
+        <v>437</v>
       </c>
       <c r="F55" t="s">
         <v>275</v>
@@ -3406,19 +3455,19 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>423</v>
+        <v>438</v>
       </c>
       <c r="B56" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="C56">
         <v>4</v>
       </c>
       <c r="D56" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E56" t="s">
-        <v>424</v>
+        <v>439</v>
       </c>
       <c r="F56" t="s">
         <v>275</v>
@@ -3426,19 +3475,19 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>425</v>
+        <v>440</v>
       </c>
       <c r="B57" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="C57">
         <v>5</v>
       </c>
       <c r="D57" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E57" t="s">
-        <v>426</v>
+        <v>441</v>
       </c>
       <c r="F57" t="s">
         <v>275</v>
@@ -3446,19 +3495,19 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>427</v>
+        <v>442</v>
       </c>
       <c r="B58" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="C58">
         <v>6</v>
       </c>
       <c r="D58" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E58" t="s">
-        <v>428</v>
+        <v>443</v>
       </c>
       <c r="F58" t="s">
         <v>275</v>
@@ -3466,19 +3515,19 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>429</v>
+        <v>444</v>
       </c>
       <c r="B59" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="C59">
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="E59" t="s">
-        <v>430</v>
+        <v>445</v>
       </c>
       <c r="F59" t="s">
         <v>275</v>
@@ -3486,19 +3535,19 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>431</v>
+        <v>446</v>
       </c>
       <c r="B60" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="C60">
         <v>8</v>
       </c>
       <c r="D60" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="E60" t="s">
-        <v>432</v>
+        <v>447</v>
       </c>
       <c r="F60" t="s">
         <v>275</v>
@@ -3506,19 +3555,19 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>433</v>
+        <v>448</v>
       </c>
       <c r="B61" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="C61">
         <v>9</v>
       </c>
       <c r="D61" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="E61" t="s">
-        <v>434</v>
+        <v>449</v>
       </c>
       <c r="F61" t="s">
         <v>275</v>
@@ -3526,19 +3575,19 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>435</v>
+        <v>450</v>
       </c>
       <c r="B62" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="C62">
         <v>10</v>
       </c>
       <c r="D62" t="s">
-        <v>339</v>
+        <v>354</v>
       </c>
       <c r="E62" t="s">
-        <v>436</v>
+        <v>451</v>
       </c>
       <c r="F62" t="s">
         <v>275</v>
@@ -3561,7 +3610,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>437</v>
+        <v>452</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>82</v>
@@ -3572,68 +3621,68 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>438</v>
+        <v>453</v>
       </c>
       <c r="B2" t="s">
-        <v>439</v>
+        <v>454</v>
       </c>
       <c r="C2" t="s">
-        <v>440</v>
+        <v>455</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>441</v>
+        <v>456</v>
       </c>
       <c r="B3" t="s">
-        <v>442</v>
+        <v>457</v>
       </c>
       <c r="C3" t="s">
-        <v>443</v>
+        <v>458</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>444</v>
+        <v>459</v>
       </c>
       <c r="B4" t="s">
-        <v>445</v>
+        <v>460</v>
       </c>
       <c r="C4" t="s">
-        <v>446</v>
+        <v>461</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>447</v>
+        <v>462</v>
       </c>
       <c r="B5" t="s">
-        <v>448</v>
+        <v>463</v>
       </c>
       <c r="C5" t="s">
-        <v>449</v>
+        <v>464</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>450</v>
+        <v>465</v>
       </c>
       <c r="B6" t="s">
-        <v>451</v>
+        <v>466</v>
       </c>
       <c r="C6" t="s">
-        <v>452</v>
+        <v>467</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>453</v>
+        <v>468</v>
       </c>
       <c r="B7" t="s">
-        <v>454</v>
+        <v>469</v>
       </c>
       <c r="C7" t="s">
-        <v>455</v>
+        <v>470</v>
       </c>
     </row>
   </sheetData>
@@ -3653,123 +3702,123 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>456</v>
+        <v>471</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>276</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>437</v>
+        <v>452</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>457</v>
+        <v>472</v>
       </c>
       <c r="B2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C2" t="s">
-        <v>438</v>
+        <v>453</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>458</v>
+        <v>473</v>
       </c>
       <c r="B3" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C3" t="s">
-        <v>441</v>
+        <v>456</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>474</v>
+      </c>
+      <c r="B4" t="s">
+        <v>287</v>
+      </c>
+      <c r="C4" t="s">
         <v>459</v>
-      </c>
-      <c r="B4" t="s">
-        <v>283</v>
-      </c>
-      <c r="C4" t="s">
-        <v>444</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>460</v>
+        <v>475</v>
       </c>
       <c r="B5" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C5" t="s">
-        <v>453</v>
+        <v>468</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>461</v>
+        <v>476</v>
       </c>
       <c r="B6" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C6" t="s">
-        <v>447</v>
+        <v>462</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>462</v>
+        <v>477</v>
       </c>
       <c r="B7" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C7" t="s">
-        <v>441</v>
+        <v>456</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>463</v>
+        <v>478</v>
       </c>
       <c r="B8" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C8" t="s">
-        <v>450</v>
+        <v>465</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>464</v>
+        <v>479</v>
       </c>
       <c r="B9" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C9" t="s">
-        <v>441</v>
+        <v>456</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>465</v>
+        <v>480</v>
       </c>
       <c r="B10" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="C10" t="s">
-        <v>453</v>
+        <v>468</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>466</v>
+        <v>481</v>
       </c>
       <c r="B11" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="C11" t="s">
-        <v>453</v>
+        <v>468</v>
       </c>
     </row>
   </sheetData>
@@ -3794,42 +3843,42 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>467</v>
+        <v>482</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>468</v>
+        <v>483</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>469</v>
+        <v>484</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>470</v>
+        <v>485</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>471</v>
+        <v>486</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>472</v>
+        <v>487</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>473</v>
+        <v>488</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>474</v>
+        <v>489</v>
       </c>
       <c r="B2" t="s">
-        <v>475</v>
+        <v>490</v>
       </c>
       <c r="C2" t="s">
         <v>115</v>
       </c>
       <c r="D2" t="s">
-        <v>476</v>
+        <v>491</v>
       </c>
       <c r="E2" t="s">
-        <v>477</v>
+        <v>492</v>
       </c>
       <c r="F2" t="s">
         <v>275</v>
@@ -3840,19 +3889,19 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>478</v>
+        <v>493</v>
       </c>
       <c r="B3" t="s">
-        <v>479</v>
+        <v>494</v>
       </c>
       <c r="C3" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="D3" t="s">
-        <v>480</v>
+        <v>495</v>
       </c>
       <c r="E3" t="s">
-        <v>481</v>
+        <v>496</v>
       </c>
       <c r="F3" t="s">
         <v>275</v>
@@ -3863,19 +3912,19 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>482</v>
+        <v>497</v>
       </c>
       <c r="B4" t="s">
-        <v>479</v>
+        <v>494</v>
       </c>
       <c r="C4" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="D4" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="E4" t="s">
-        <v>483</v>
+        <v>498</v>
       </c>
       <c r="F4" t="s">
         <v>275</v>
@@ -3886,19 +3935,19 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>484</v>
+        <v>499</v>
       </c>
       <c r="B5" t="s">
-        <v>479</v>
+        <v>494</v>
       </c>
       <c r="C5" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="D5" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="E5" t="s">
-        <v>485</v>
+        <v>500</v>
       </c>
       <c r="F5" t="s">
         <v>275</v>
@@ -3909,19 +3958,19 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>486</v>
+        <v>501</v>
       </c>
       <c r="B6" t="s">
-        <v>479</v>
+        <v>494</v>
       </c>
       <c r="C6" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="D6" t="s">
-        <v>487</v>
+        <v>502</v>
       </c>
       <c r="E6" t="s">
-        <v>488</v>
+        <v>503</v>
       </c>
       <c r="F6" t="s">
         <v>275</v>
@@ -3932,19 +3981,19 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>489</v>
+        <v>504</v>
       </c>
       <c r="B7" t="s">
-        <v>479</v>
+        <v>494</v>
       </c>
       <c r="C7" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="D7" t="s">
-        <v>299</v>
+        <v>309</v>
       </c>
       <c r="E7" t="s">
-        <v>490</v>
+        <v>505</v>
       </c>
       <c r="F7" t="s">
         <v>275</v>
@@ -3955,19 +4004,19 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>491</v>
+        <v>506</v>
       </c>
       <c r="B8" t="s">
-        <v>479</v>
+        <v>494</v>
       </c>
       <c r="C8" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="D8" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="E8" t="s">
-        <v>492</v>
+        <v>507</v>
       </c>
       <c r="F8" t="s">
         <v>275</v>
@@ -3978,10 +4027,10 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>493</v>
+        <v>508</v>
       </c>
       <c r="B9" t="s">
-        <v>494</v>
+        <v>509</v>
       </c>
       <c r="C9" t="s">
         <v>38</v>
@@ -3990,7 +4039,7 @@
         <v>40</v>
       </c>
       <c r="E9" t="s">
-        <v>495</v>
+        <v>510</v>
       </c>
       <c r="F9" t="s">
         <v>275</v>
@@ -4017,30 +4066,30 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>496</v>
+        <v>511</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>497</v>
+        <v>512</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>498</v>
+        <v>513</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>61</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>499</v>
+        <v>514</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>500</v>
+        <v>515</v>
       </c>
       <c r="B2" t="s">
-        <v>501</v>
+        <v>516</v>
       </c>
       <c r="C2" t="s">
-        <v>502</v>
+        <v>517</v>
       </c>
       <c r="D2" t="b">
         <v>0</v>
@@ -4051,13 +4100,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>503</v>
+        <v>518</v>
       </c>
       <c r="B3" t="s">
-        <v>504</v>
+        <v>519</v>
       </c>
       <c r="C3" t="s">
-        <v>475</v>
+        <v>490</v>
       </c>
       <c r="D3" t="b">
         <v>0</v>
@@ -4068,13 +4117,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>505</v>
+        <v>520</v>
       </c>
       <c r="B4" t="s">
-        <v>506</v>
+        <v>521</v>
       </c>
       <c r="C4" t="s">
-        <v>507</v>
+        <v>522</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
@@ -4085,13 +4134,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="B5" t="s">
-        <v>509</v>
+        <v>524</v>
       </c>
       <c r="C5" t="s">
-        <v>502</v>
+        <v>517</v>
       </c>
       <c r="D5" t="b">
         <v>0</v>
@@ -4099,13 +4148,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>510</v>
+        <v>525</v>
       </c>
       <c r="B6" t="s">
-        <v>511</v>
+        <v>526</v>
       </c>
       <c r="C6" t="s">
-        <v>512</v>
+        <v>527</v>
       </c>
       <c r="D6" t="b">
         <v>0</v>
@@ -4113,13 +4162,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>513</v>
+        <v>528</v>
       </c>
       <c r="B7" t="s">
-        <v>511</v>
+        <v>526</v>
       </c>
       <c r="C7" t="s">
-        <v>514</v>
+        <v>529</v>
       </c>
       <c r="D7" t="b">
         <v>0</v>
@@ -4145,16 +4194,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>515</v>
+        <v>530</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>516</v>
+        <v>531</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>517</v>
+        <v>532</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>518</v>
+        <v>533</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>61</v>
@@ -4162,16 +4211,16 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>519</v>
+        <v>534</v>
       </c>
       <c r="B2" t="s">
-        <v>520</v>
+        <v>535</v>
       </c>
       <c r="C2" t="s">
-        <v>521</v>
+        <v>536</v>
       </c>
       <c r="D2" t="s">
-        <v>522</v>
+        <v>537</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -4205,7 +4254,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>523</v>
+        <v>538</v>
       </c>
       <c r="B2" t="s">
         <v>146</v>
@@ -6010,7 +6059,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -6018,10 +6067,10 @@
     <col min="4" max="4" width="60" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="7" width="12" customWidth="1"/>
-    <col min="8" max="9" width="22" customWidth="1"/>
+    <col min="8" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>276</v>
       </c>
@@ -6049,19 +6098,25 @@
       <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B2" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="D2" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E2" t="s">
         <v>260</v>
@@ -6078,19 +6133,25 @@
       <c r="I2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J2" t="s">
+        <v>285</v>
+      </c>
+      <c r="K2" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="B3" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="C3" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="D3" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="E3" t="s">
         <v>264</v>
@@ -6102,24 +6163,30 @@
         <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="I3" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+        <v>291</v>
+      </c>
+      <c r="J3" t="s">
+        <v>292</v>
+      </c>
+      <c r="K3" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="B4" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="C4" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="D4" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="E4" t="s">
         <v>260</v>
@@ -6131,24 +6198,30 @@
         <v>42</v>
       </c>
       <c r="H4" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="I4" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>298</v>
+      </c>
+      <c r="J4" t="s">
+        <v>299</v>
+      </c>
+      <c r="K4" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="B5" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="C5" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="D5" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="E5" t="s">
         <v>260</v>
@@ -6160,24 +6233,30 @@
         <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="I5" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>305</v>
+      </c>
+      <c r="J5" t="s">
+        <v>306</v>
+      </c>
+      <c r="K5" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="B6" t="s">
-        <v>299</v>
+        <v>309</v>
       </c>
       <c r="C6" t="s">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="D6" t="s">
-        <v>301</v>
+        <v>311</v>
       </c>
       <c r="E6" t="s">
         <v>264</v>
@@ -6189,24 +6268,30 @@
         <v>42</v>
       </c>
       <c r="H6" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="I6" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>312</v>
+      </c>
+      <c r="J6" t="s">
+        <v>313</v>
+      </c>
+      <c r="K6" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="B7" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="C7" t="s">
-        <v>305</v>
+        <v>317</v>
       </c>
       <c r="D7" t="s">
-        <v>306</v>
+        <v>318</v>
       </c>
       <c r="E7" t="s">
         <v>264</v>
@@ -6218,10 +6303,16 @@
         <v>42</v>
       </c>
       <c r="H7" t="s">
-        <v>307</v>
+        <v>319</v>
       </c>
       <c r="I7" t="s">
-        <v>307</v>
+        <v>319</v>
+      </c>
+      <c r="J7" t="s">
+        <v>320</v>
+      </c>
+      <c r="K7" t="s">
+        <v>321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Admin: update posts POST0011 status and 14 more changes
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1672" uniqueCount="864">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1677" uniqueCount="867">
   <si>
     <t>setting_key</t>
   </si>
@@ -1224,10 +1224,7 @@
     <t>A hybrid pairs a petrol engine with an electric motor and a battery that charges itself while you drive. Here is what each part does, how braking recovers energy, and why it saves fuel.</t>
   </si>
   <si>
-    <t>draft</t>
-  </si>
-  <si>
-    <t>2026-10-31T06:27:34Z</t>
+    <t>2026-10-31T06:43:59Z</t>
   </si>
   <si>
     <t>POST0008</t>
@@ -1242,6 +1239,9 @@
     <t>Every flight comes down to four forces: lift, weight, thrust and drag. See what each one does, how pilots change the balance for takeoff, cruising and landing, and why engines do not lift the plane.</t>
   </si>
   <si>
+    <t>2026-10-31T06:43:48Z</t>
+  </si>
+  <si>
     <t>POST0009</t>
   </si>
   <si>
@@ -1254,6 +1254,9 @@
     <t>In 1913 Ford moved cars past workers instead of workers around cars. Build time for one Model T fell from 12 and a half hours to 93 minutes, and the price fell with it. Here is how it happened.</t>
   </si>
   <si>
+    <t>2026-10-31T06:43:28Z</t>
+  </si>
+  <si>
     <t>POST0010</t>
   </si>
   <si>
@@ -1266,6 +1269,9 @@
     <t>A context window is the amount of text an AI model can look at in one go. Learn what counts toward it, how tokens relate to words, and why long chats can lose track of earlier details.</t>
   </si>
   <si>
+    <t>2026-10-31T06:42:29Z</t>
+  </si>
+  <si>
     <t>POST0011</t>
   </si>
   <si>
@@ -1276,6 +1282,9 @@
   </si>
   <si>
     <t>USB Power Delivery lets a charger and a device agree on the power they need. See how the negotiation works, what the 100 W and 240 W limits mean, and why the cable matters.</t>
+  </si>
+  <si>
+    <t>2026-10-31T06:41:53Z</t>
   </si>
   <si>
     <t>block_id</t>
@@ -3377,7 +3386,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>304</v>
@@ -3386,21 +3395,21 @@
         <v>65</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="B2" t="s">
         <v>309</v>
@@ -3409,10 +3418,10 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E2" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="F2" t="s">
         <v>303</v>
@@ -3420,7 +3429,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="B3" t="s">
         <v>309</v>
@@ -3429,10 +3438,10 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E3" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="F3" t="s">
         <v>303</v>
@@ -3440,7 +3449,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="B4" t="s">
         <v>309</v>
@@ -3449,10 +3458,10 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E4" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="F4" t="s">
         <v>303</v>
@@ -3460,7 +3469,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="B5" t="s">
         <v>309</v>
@@ -3469,10 +3478,10 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E5" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="F5" t="s">
         <v>303</v>
@@ -3480,7 +3489,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="B6" t="s">
         <v>309</v>
@@ -3489,10 +3498,10 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E6" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="F6" t="s">
         <v>303</v>
@@ -3500,7 +3509,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="B7" t="s">
         <v>315</v>
@@ -3509,10 +3518,10 @@
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E7" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="F7" t="s">
         <v>303</v>
@@ -3520,7 +3529,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="B8" t="s">
         <v>315</v>
@@ -3529,10 +3538,10 @@
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E8" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="F8" t="s">
         <v>303</v>
@@ -3540,7 +3549,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="B9" t="s">
         <v>315</v>
@@ -3549,10 +3558,10 @@
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E9" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="F9" t="s">
         <v>303</v>
@@ -3560,7 +3569,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B10" t="s">
         <v>315</v>
@@ -3569,10 +3578,10 @@
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E10" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="F10" t="s">
         <v>303</v>
@@ -3580,7 +3589,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="B11" t="s">
         <v>315</v>
@@ -3589,10 +3598,10 @@
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E11" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="F11" t="s">
         <v>303</v>
@@ -3600,7 +3609,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B12" t="s">
         <v>315</v>
@@ -3609,10 +3618,10 @@
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E12" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="F12" t="s">
         <v>303</v>
@@ -3620,7 +3629,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="B13" t="s">
         <v>315</v>
@@ -3629,10 +3638,10 @@
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E13" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="F13" t="s">
         <v>303</v>
@@ -3640,7 +3649,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="B14" t="s">
         <v>315</v>
@@ -3649,10 +3658,10 @@
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E14" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="F14" t="s">
         <v>303</v>
@@ -3660,7 +3669,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B15" t="s">
         <v>315</v>
@@ -3669,10 +3678,10 @@
         <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E15" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="F15" t="s">
         <v>303</v>
@@ -3680,7 +3689,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="B16" t="s">
         <v>315</v>
@@ -3689,10 +3698,10 @@
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E16" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="F16" t="s">
         <v>303</v>
@@ -3700,7 +3709,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="B17" t="s">
         <v>322</v>
@@ -3709,10 +3718,10 @@
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E17" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="F17" t="s">
         <v>303</v>
@@ -3720,7 +3729,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="B18" t="s">
         <v>322</v>
@@ -3729,10 +3738,10 @@
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E18" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="F18" t="s">
         <v>303</v>
@@ -3740,7 +3749,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="B19" t="s">
         <v>322</v>
@@ -3749,10 +3758,10 @@
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E19" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="F19" t="s">
         <v>303</v>
@@ -3760,7 +3769,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="B20" t="s">
         <v>322</v>
@@ -3769,10 +3778,10 @@
         <v>4</v>
       </c>
       <c r="D20" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E20" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="F20" t="s">
         <v>303</v>
@@ -3780,7 +3789,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="B21" t="s">
         <v>322</v>
@@ -3789,10 +3798,10 @@
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E21" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="F21" t="s">
         <v>303</v>
@@ -3800,7 +3809,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="B22" t="s">
         <v>322</v>
@@ -3809,10 +3818,10 @@
         <v>6</v>
       </c>
       <c r="D22" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E22" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="F22" t="s">
         <v>303</v>
@@ -3820,7 +3829,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="B23" t="s">
         <v>322</v>
@@ -3829,10 +3838,10 @@
         <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E23" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="F23" t="s">
         <v>303</v>
@@ -3840,7 +3849,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="B24" t="s">
         <v>322</v>
@@ -3849,10 +3858,10 @@
         <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E24" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="F24" t="s">
         <v>303</v>
@@ -3860,7 +3869,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="B25" t="s">
         <v>322</v>
@@ -3869,10 +3878,10 @@
         <v>9</v>
       </c>
       <c r="D25" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E25" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="F25" t="s">
         <v>303</v>
@@ -3880,7 +3889,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="B26" t="s">
         <v>322</v>
@@ -3889,10 +3898,10 @@
         <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E26" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="F26" t="s">
         <v>303</v>
@@ -3900,7 +3909,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="B27" t="s">
         <v>322</v>
@@ -3909,10 +3918,10 @@
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E27" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="F27" t="s">
         <v>303</v>
@@ -3920,7 +3929,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B28" t="s">
         <v>322</v>
@@ -3929,10 +3938,10 @@
         <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E28" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="F28" t="s">
         <v>303</v>
@@ -3940,7 +3949,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="B29" t="s">
         <v>329</v>
@@ -3949,10 +3958,10 @@
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E29" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="F29" t="s">
         <v>303</v>
@@ -3960,7 +3969,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B30" t="s">
         <v>329</v>
@@ -3969,10 +3978,10 @@
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E30" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="F30" t="s">
         <v>303</v>
@@ -3980,7 +3989,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="B31" t="s">
         <v>329</v>
@@ -3989,10 +3998,10 @@
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E31" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="F31" t="s">
         <v>303</v>
@@ -4000,7 +4009,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="B32" t="s">
         <v>329</v>
@@ -4009,10 +4018,10 @@
         <v>4</v>
       </c>
       <c r="D32" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E32" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="F32" t="s">
         <v>303</v>
@@ -4020,7 +4029,7 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B33" t="s">
         <v>329</v>
@@ -4029,10 +4038,10 @@
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E33" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="F33" t="s">
         <v>303</v>
@@ -4040,7 +4049,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="B34" t="s">
         <v>329</v>
@@ -4049,10 +4058,10 @@
         <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E34" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="F34" t="s">
         <v>303</v>
@@ -4060,7 +4069,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="B35" t="s">
         <v>329</v>
@@ -4069,10 +4078,10 @@
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E35" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="F35" t="s">
         <v>303</v>
@@ -4080,7 +4089,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="B36" t="s">
         <v>329</v>
@@ -4089,10 +4098,10 @@
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E36" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="F36" t="s">
         <v>303</v>
@@ -4100,7 +4109,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="B37" t="s">
         <v>329</v>
@@ -4109,10 +4118,10 @@
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E37" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="F37" t="s">
         <v>303</v>
@@ -4120,7 +4129,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="B38" t="s">
         <v>329</v>
@@ -4129,10 +4138,10 @@
         <v>10</v>
       </c>
       <c r="D38" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E38" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="F38" t="s">
         <v>303</v>
@@ -4140,7 +4149,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="B39" t="s">
         <v>329</v>
@@ -4149,10 +4158,10 @@
         <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E39" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="F39" t="s">
         <v>303</v>
@@ -4160,7 +4169,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="B40" t="s">
         <v>329</v>
@@ -4169,10 +4178,10 @@
         <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E40" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="F40" t="s">
         <v>303</v>
@@ -4180,7 +4189,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="B41" t="s">
         <v>336</v>
@@ -4189,10 +4198,10 @@
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E41" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="F41" t="s">
         <v>303</v>
@@ -4200,7 +4209,7 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="B42" t="s">
         <v>336</v>
@@ -4209,10 +4218,10 @@
         <v>2</v>
       </c>
       <c r="D42" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E42" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="F42" t="s">
         <v>303</v>
@@ -4220,7 +4229,7 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="B43" t="s">
         <v>336</v>
@@ -4229,10 +4238,10 @@
         <v>3</v>
       </c>
       <c r="D43" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E43" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="F43" t="s">
         <v>303</v>
@@ -4240,7 +4249,7 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B44" t="s">
         <v>336</v>
@@ -4249,10 +4258,10 @@
         <v>4</v>
       </c>
       <c r="D44" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E44" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="F44" t="s">
         <v>303</v>
@@ -4260,7 +4269,7 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="B45" t="s">
         <v>336</v>
@@ -4269,10 +4278,10 @@
         <v>5</v>
       </c>
       <c r="D45" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E45" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="F45" t="s">
         <v>303</v>
@@ -4280,7 +4289,7 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="B46" t="s">
         <v>336</v>
@@ -4289,10 +4298,10 @@
         <v>6</v>
       </c>
       <c r="D46" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E46" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="F46" t="s">
         <v>303</v>
@@ -4300,7 +4309,7 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="B47" t="s">
         <v>336</v>
@@ -4309,10 +4318,10 @@
         <v>7</v>
       </c>
       <c r="D47" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E47" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="F47" t="s">
         <v>303</v>
@@ -4320,7 +4329,7 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="B48" t="s">
         <v>336</v>
@@ -4329,10 +4338,10 @@
         <v>8</v>
       </c>
       <c r="D48" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E48" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="F48" t="s">
         <v>303</v>
@@ -4340,7 +4349,7 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="B49" t="s">
         <v>336</v>
@@ -4349,10 +4358,10 @@
         <v>9</v>
       </c>
       <c r="D49" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E49" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="F49" t="s">
         <v>303</v>
@@ -4360,7 +4369,7 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B50" t="s">
         <v>336</v>
@@ -4369,10 +4378,10 @@
         <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E50" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="F50" t="s">
         <v>303</v>
@@ -4380,7 +4389,7 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="B51" t="s">
         <v>336</v>
@@ -4389,10 +4398,10 @@
         <v>11</v>
       </c>
       <c r="D51" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E51" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="F51" t="s">
         <v>303</v>
@@ -4400,7 +4409,7 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="B52" t="s">
         <v>336</v>
@@ -4409,10 +4418,10 @@
         <v>12</v>
       </c>
       <c r="D52" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E52" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="F52" t="s">
         <v>303</v>
@@ -4420,7 +4429,7 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="B53" t="s">
         <v>343</v>
@@ -4429,10 +4438,10 @@
         <v>1</v>
       </c>
       <c r="D53" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E53" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="F53" t="s">
         <v>303</v>
@@ -4440,7 +4449,7 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="B54" t="s">
         <v>343</v>
@@ -4449,10 +4458,10 @@
         <v>2</v>
       </c>
       <c r="D54" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E54" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="F54" t="s">
         <v>303</v>
@@ -4460,7 +4469,7 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="B55" t="s">
         <v>343</v>
@@ -4469,10 +4478,10 @@
         <v>3</v>
       </c>
       <c r="D55" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E55" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="F55" t="s">
         <v>303</v>
@@ -4480,7 +4489,7 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="B56" t="s">
         <v>343</v>
@@ -4489,10 +4498,10 @@
         <v>4</v>
       </c>
       <c r="D56" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E56" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="F56" t="s">
         <v>303</v>
@@ -4500,7 +4509,7 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="B57" t="s">
         <v>343</v>
@@ -4509,10 +4518,10 @@
         <v>5</v>
       </c>
       <c r="D57" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E57" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="F57" t="s">
         <v>303</v>
@@ -4520,7 +4529,7 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="B58" t="s">
         <v>343</v>
@@ -4529,10 +4538,10 @@
         <v>6</v>
       </c>
       <c r="D58" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E58" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="F58" t="s">
         <v>303</v>
@@ -4540,7 +4549,7 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="B59" t="s">
         <v>343</v>
@@ -4549,10 +4558,10 @@
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E59" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="F59" t="s">
         <v>303</v>
@@ -4560,7 +4569,7 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="B60" t="s">
         <v>343</v>
@@ -4569,10 +4578,10 @@
         <v>8</v>
       </c>
       <c r="D60" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E60" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="F60" t="s">
         <v>303</v>
@@ -4580,7 +4589,7 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="B61" t="s">
         <v>343</v>
@@ -4589,10 +4598,10 @@
         <v>9</v>
       </c>
       <c r="D61" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E61" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="F61" t="s">
         <v>303</v>
@@ -4600,7 +4609,7 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="B62" t="s">
         <v>343</v>
@@ -4609,10 +4618,10 @@
         <v>10</v>
       </c>
       <c r="D62" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E62" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="F62" t="s">
         <v>303</v>
@@ -4620,7 +4629,7 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="B63" t="s">
         <v>350</v>
@@ -4629,15 +4638,15 @@
         <v>1</v>
       </c>
       <c r="D63" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E63" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="B64" t="s">
         <v>350</v>
@@ -4646,15 +4655,15 @@
         <v>2</v>
       </c>
       <c r="D64" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E64" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="B65" t="s">
         <v>350</v>
@@ -4663,15 +4672,15 @@
         <v>3</v>
       </c>
       <c r="D65" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E65" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B66" t="s">
         <v>350</v>
@@ -4680,15 +4689,15 @@
         <v>4</v>
       </c>
       <c r="D66" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E66" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="B67" t="s">
         <v>350</v>
@@ -4697,15 +4706,15 @@
         <v>5</v>
       </c>
       <c r="D67" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E67" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B68" t="s">
         <v>350</v>
@@ -4714,15 +4723,15 @@
         <v>6</v>
       </c>
       <c r="D68" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E68" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="B69" t="s">
         <v>350</v>
@@ -4731,15 +4740,15 @@
         <v>7</v>
       </c>
       <c r="D69" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E69" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="B70" t="s">
         <v>350</v>
@@ -4748,15 +4757,15 @@
         <v>8</v>
       </c>
       <c r="D70" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E70" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B71" t="s">
         <v>350</v>
@@ -4765,15 +4774,15 @@
         <v>9</v>
       </c>
       <c r="D71" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E71" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="B72" t="s">
         <v>350</v>
@@ -4782,15 +4791,15 @@
         <v>10</v>
       </c>
       <c r="D72" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E72" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B73" t="s">
         <v>350</v>
@@ -4799,15 +4808,15 @@
         <v>11</v>
       </c>
       <c r="D73" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E73" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="B74" t="s">
         <v>350</v>
@@ -4816,15 +4825,15 @@
         <v>12</v>
       </c>
       <c r="D74" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E74" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="B75" t="s">
         <v>350</v>
@@ -4833,15 +4842,15 @@
         <v>13</v>
       </c>
       <c r="D75" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E75" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="B76" t="s">
         <v>350</v>
@@ -4850,15 +4859,15 @@
         <v>14</v>
       </c>
       <c r="D76" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E76" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="B77" t="s">
         <v>350</v>
@@ -4867,15 +4876,15 @@
         <v>15</v>
       </c>
       <c r="D77" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E77" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="B78" t="s">
         <v>350</v>
@@ -4884,15 +4893,15 @@
         <v>16</v>
       </c>
       <c r="D78" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E78" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="B79" t="s">
         <v>350</v>
@@ -4901,15 +4910,15 @@
         <v>17</v>
       </c>
       <c r="D79" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E79" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="B80" t="s">
         <v>350</v>
@@ -4918,15 +4927,15 @@
         <v>18</v>
       </c>
       <c r="D80" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E80" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="B81" t="s">
         <v>350</v>
@@ -4935,15 +4944,15 @@
         <v>19</v>
       </c>
       <c r="D81" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E81" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="B82" t="s">
         <v>350</v>
@@ -4952,15 +4961,15 @@
         <v>20</v>
       </c>
       <c r="D82" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E82" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="B83" t="s">
         <v>350</v>
@@ -4969,15 +4978,15 @@
         <v>21</v>
       </c>
       <c r="D83" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E83" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="B84" t="s">
         <v>350</v>
@@ -4986,406 +4995,406 @@
         <v>22</v>
       </c>
       <c r="D84" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E84" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="B85" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C85">
         <v>1</v>
       </c>
       <c r="D85" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E85" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="B86" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C86">
         <v>2</v>
       </c>
       <c r="D86" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E86" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="B87" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C87">
         <v>3</v>
       </c>
       <c r="D87" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E87" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="B88" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C88">
         <v>4</v>
       </c>
       <c r="D88" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E88" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="B89" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C89">
         <v>5</v>
       </c>
       <c r="D89" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E89" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="B90" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C90">
         <v>6</v>
       </c>
       <c r="D90" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E90" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="B91" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C91">
         <v>7</v>
       </c>
       <c r="D91" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E91" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B92" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C92">
         <v>8</v>
       </c>
       <c r="D92" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E92" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="B93" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C93">
         <v>9</v>
       </c>
       <c r="D93" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E93" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="B94" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C94">
         <v>10</v>
       </c>
       <c r="D94" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E94" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="B95" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C95">
         <v>11</v>
       </c>
       <c r="D95" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E95" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="B96" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C96">
         <v>12</v>
       </c>
       <c r="D96" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E96" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="B97" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C97">
         <v>13</v>
       </c>
       <c r="D97" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E97" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="B98" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C98">
         <v>14</v>
       </c>
       <c r="D98" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E98" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="B99" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C99">
         <v>15</v>
       </c>
       <c r="D99" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E99" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="B100" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C100">
         <v>16</v>
       </c>
       <c r="D100" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E100" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="B101" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C101">
         <v>17</v>
       </c>
       <c r="D101" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E101" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="B102" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C102">
         <v>18</v>
       </c>
       <c r="D102" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E102" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B103" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C103">
         <v>19</v>
       </c>
       <c r="D103" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E103" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="B104" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C104">
         <v>20</v>
       </c>
       <c r="D104" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E104" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="B105" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C105">
         <v>21</v>
       </c>
       <c r="D105" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E105" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="B106" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C106">
         <v>22</v>
       </c>
       <c r="D106" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E106" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="B107" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C107">
         <v>23</v>
       </c>
       <c r="D107" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E107" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="B108" t="s">
         <v>360</v>
@@ -5394,15 +5403,15 @@
         <v>1</v>
       </c>
       <c r="D108" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E108" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="B109" t="s">
         <v>360</v>
@@ -5411,15 +5420,15 @@
         <v>2</v>
       </c>
       <c r="D109" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E109" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="B110" t="s">
         <v>360</v>
@@ -5428,15 +5437,15 @@
         <v>3</v>
       </c>
       <c r="D110" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E110" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="B111" t="s">
         <v>360</v>
@@ -5445,15 +5454,15 @@
         <v>4</v>
       </c>
       <c r="D111" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E111" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="B112" t="s">
         <v>360</v>
@@ -5462,15 +5471,15 @@
         <v>5</v>
       </c>
       <c r="D112" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E112" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="B113" t="s">
         <v>360</v>
@@ -5479,15 +5488,15 @@
         <v>6</v>
       </c>
       <c r="D113" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E113" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="B114" t="s">
         <v>360</v>
@@ -5496,15 +5505,15 @@
         <v>7</v>
       </c>
       <c r="D114" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E114" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
       <c r="B115" t="s">
         <v>360</v>
@@ -5513,15 +5522,15 @@
         <v>8</v>
       </c>
       <c r="D115" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E115" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="B116" t="s">
         <v>360</v>
@@ -5530,15 +5539,15 @@
         <v>9</v>
       </c>
       <c r="D116" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E116" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B117" t="s">
         <v>360</v>
@@ -5547,15 +5556,15 @@
         <v>10</v>
       </c>
       <c r="D117" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E117" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="B118" t="s">
         <v>360</v>
@@ -5564,15 +5573,15 @@
         <v>11</v>
       </c>
       <c r="D118" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E118" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="B119" t="s">
         <v>360</v>
@@ -5581,15 +5590,15 @@
         <v>12</v>
       </c>
       <c r="D119" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E119" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="B120" t="s">
         <v>360</v>
@@ -5598,15 +5607,15 @@
         <v>13</v>
       </c>
       <c r="D120" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E120" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="B121" t="s">
         <v>360</v>
@@ -5615,15 +5624,15 @@
         <v>14</v>
       </c>
       <c r="D121" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E121" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="B122" t="s">
         <v>360</v>
@@ -5632,15 +5641,15 @@
         <v>15</v>
       </c>
       <c r="D122" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E122" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="B123" t="s">
         <v>360</v>
@@ -5649,15 +5658,15 @@
         <v>16</v>
       </c>
       <c r="D123" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E123" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="B124" t="s">
         <v>360</v>
@@ -5666,15 +5675,15 @@
         <v>17</v>
       </c>
       <c r="D124" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E124" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="B125" t="s">
         <v>360</v>
@@ -5683,15 +5692,15 @@
         <v>18</v>
       </c>
       <c r="D125" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E125" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="B126" t="s">
         <v>360</v>
@@ -5700,15 +5709,15 @@
         <v>19</v>
       </c>
       <c r="D126" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E126" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="B127" t="s">
         <v>360</v>
@@ -5717,15 +5726,15 @@
         <v>20</v>
       </c>
       <c r="D127" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E127" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="B128" t="s">
         <v>360</v>
@@ -5734,758 +5743,758 @@
         <v>21</v>
       </c>
       <c r="D128" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E128" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="B129" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C129">
         <v>1</v>
       </c>
       <c r="D129" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E129" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
       <c r="B130" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C130">
         <v>2</v>
       </c>
       <c r="D130" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E130" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="B131" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C131">
         <v>3</v>
       </c>
       <c r="D131" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E131" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="B132" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C132">
         <v>4</v>
       </c>
       <c r="D132" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E132" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="B133" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C133">
         <v>5</v>
       </c>
       <c r="D133" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E133" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
       <c r="B134" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C134">
         <v>6</v>
       </c>
       <c r="D134" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E134" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="B135" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C135">
         <v>7</v>
       </c>
       <c r="D135" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E135" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
       <c r="B136" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C136">
         <v>8</v>
       </c>
       <c r="D136" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E136" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="B137" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C137">
         <v>9</v>
       </c>
       <c r="D137" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E137" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="B138" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C138">
         <v>10</v>
       </c>
       <c r="D138" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E138" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="B139" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C139">
         <v>11</v>
       </c>
       <c r="D139" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E139" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="B140" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C140">
         <v>12</v>
       </c>
       <c r="D140" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E140" t="s">
-        <v>653</v>
+        <v>656</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="B141" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C141">
         <v>13</v>
       </c>
       <c r="D141" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E141" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="B142" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C142">
         <v>14</v>
       </c>
       <c r="D142" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E142" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="B143" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C143">
         <v>15</v>
       </c>
       <c r="D143" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E143" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="B144" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C144">
         <v>16</v>
       </c>
       <c r="D144" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E144" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
       <c r="B145" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C145">
         <v>17</v>
       </c>
       <c r="D145" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E145" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>664</v>
+        <v>667</v>
       </c>
       <c r="B146" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C146">
         <v>18</v>
       </c>
       <c r="D146" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E146" t="s">
-        <v>665</v>
+        <v>668</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>666</v>
+        <v>669</v>
       </c>
       <c r="B147" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C147">
         <v>19</v>
       </c>
       <c r="D147" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E147" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="B148" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C148">
         <v>20</v>
       </c>
       <c r="D148" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E148" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
       <c r="B149" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C149">
         <v>21</v>
       </c>
       <c r="D149" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E149" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="B150" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C150">
         <v>22</v>
       </c>
       <c r="D150" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E150" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="B151" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C151">
         <v>1</v>
       </c>
       <c r="D151" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E151" t="s">
-        <v>673</v>
+        <v>676</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>674</v>
+        <v>677</v>
       </c>
       <c r="B152" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C152">
         <v>2</v>
       </c>
       <c r="D152" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E152" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="B153" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C153">
         <v>3</v>
       </c>
       <c r="D153" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E153" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>678</v>
+        <v>681</v>
       </c>
       <c r="B154" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C154">
         <v>4</v>
       </c>
       <c r="D154" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E154" t="s">
-        <v>679</v>
+        <v>682</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="B155" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C155">
         <v>5</v>
       </c>
       <c r="D155" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E155" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>682</v>
+        <v>685</v>
       </c>
       <c r="B156" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C156">
         <v>6</v>
       </c>
       <c r="D156" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E156" t="s">
-        <v>683</v>
+        <v>686</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
       <c r="B157" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C157">
         <v>7</v>
       </c>
       <c r="D157" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E157" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>686</v>
+        <v>689</v>
       </c>
       <c r="B158" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C158">
         <v>8</v>
       </c>
       <c r="D158" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E158" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="B159" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C159">
         <v>9</v>
       </c>
       <c r="D159" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E159" t="s">
-        <v>689</v>
+        <v>692</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>690</v>
+        <v>693</v>
       </c>
       <c r="B160" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C160">
         <v>10</v>
       </c>
       <c r="D160" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E160" t="s">
-        <v>691</v>
+        <v>694</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>692</v>
+        <v>695</v>
       </c>
       <c r="B161" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C161">
         <v>11</v>
       </c>
       <c r="D161" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E161" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="B162" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C162">
         <v>12</v>
       </c>
       <c r="D162" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E162" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="B163" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C163">
         <v>13</v>
       </c>
       <c r="D163" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E163" t="s">
-        <v>697</v>
+        <v>700</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>698</v>
+        <v>701</v>
       </c>
       <c r="B164" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C164">
         <v>14</v>
       </c>
       <c r="D164" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E164" t="s">
-        <v>699</v>
+        <v>702</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
       <c r="B165" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C165">
         <v>15</v>
       </c>
       <c r="D165" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E165" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
       <c r="B166" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C166">
         <v>16</v>
       </c>
       <c r="D166" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E166" t="s">
-        <v>703</v>
+        <v>706</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="B167" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C167">
         <v>17</v>
       </c>
       <c r="D167" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E167" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B168" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C168">
         <v>18</v>
       </c>
       <c r="D168" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E168" t="s">
-        <v>707</v>
+        <v>710</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>708</v>
+        <v>711</v>
       </c>
       <c r="B169" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C169">
         <v>19</v>
       </c>
       <c r="D169" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E169" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="B170" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C170">
         <v>20</v>
       </c>
       <c r="D170" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E170" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>711</v>
+        <v>714</v>
       </c>
       <c r="B171" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C171">
         <v>21</v>
       </c>
       <c r="D171" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E171" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="B172" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C172">
         <v>22</v>
       </c>
       <c r="D172" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E172" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
     </row>
   </sheetData>
@@ -6505,7 +6514,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>90</v>
@@ -6516,205 +6525,205 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>715</v>
+        <v>718</v>
       </c>
       <c r="B2" t="s">
-        <v>716</v>
+        <v>719</v>
       </c>
       <c r="C2" t="s">
-        <v>717</v>
+        <v>720</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
       <c r="B3" t="s">
-        <v>719</v>
+        <v>722</v>
       </c>
       <c r="C3" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="B4" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="C4" t="s">
-        <v>723</v>
+        <v>726</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="B5" t="s">
-        <v>725</v>
+        <v>728</v>
       </c>
       <c r="C5" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>727</v>
+        <v>730</v>
       </c>
       <c r="B6" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
       <c r="C6" t="s">
-        <v>729</v>
+        <v>732</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="B7" t="s">
-        <v>731</v>
+        <v>734</v>
       </c>
       <c r="C7" t="s">
-        <v>732</v>
+        <v>735</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>733</v>
+        <v>736</v>
       </c>
       <c r="B8" t="s">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="C8" t="s">
-        <v>734</v>
+        <v>737</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="B9" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="C9" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>737</v>
+        <v>740</v>
       </c>
       <c r="B10" t="s">
-        <v>738</v>
+        <v>741</v>
       </c>
       <c r="C10" t="s">
-        <v>738</v>
+        <v>741</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>739</v>
+        <v>742</v>
       </c>
       <c r="B11" t="s">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="C11" t="s">
-        <v>741</v>
+        <v>744</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>742</v>
+        <v>745</v>
       </c>
       <c r="B12" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
       <c r="C12" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="B13" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
       <c r="C13" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>746</v>
+        <v>749</v>
       </c>
       <c r="B14" t="s">
-        <v>747</v>
+        <v>750</v>
       </c>
       <c r="C14" t="s">
-        <v>747</v>
+        <v>750</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
       <c r="B15" t="s">
-        <v>749</v>
+        <v>752</v>
       </c>
       <c r="C15" t="s">
-        <v>749</v>
+        <v>752</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>750</v>
+        <v>753</v>
       </c>
       <c r="B16" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
       <c r="C16" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>752</v>
+        <v>755</v>
       </c>
       <c r="B17" t="s">
-        <v>753</v>
+        <v>756</v>
       </c>
       <c r="C17" t="s">
-        <v>754</v>
+        <v>757</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>755</v>
+        <v>758</v>
       </c>
       <c r="B18" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="C18" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>757</v>
+        <v>760</v>
       </c>
       <c r="B19" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
       <c r="C19" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B20" t="s">
         <v>290</v>
@@ -6725,79 +6734,79 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
       <c r="B21" t="s">
-        <v>761</v>
+        <v>764</v>
       </c>
       <c r="C21" t="s">
-        <v>761</v>
+        <v>764</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
       <c r="B22" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="C22" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>764</v>
+        <v>767</v>
       </c>
       <c r="B23" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="C23" t="s">
-        <v>766</v>
+        <v>769</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="B24" t="s">
-        <v>768</v>
+        <v>771</v>
       </c>
       <c r="C24" t="s">
-        <v>768</v>
+        <v>771</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>769</v>
+        <v>772</v>
       </c>
       <c r="B25" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="C25" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="B26" t="s">
-        <v>772</v>
+        <v>775</v>
       </c>
       <c r="C26" t="s">
-        <v>773</v>
+        <v>776</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>774</v>
+        <v>777</v>
       </c>
       <c r="B27" t="s">
-        <v>775</v>
+        <v>778</v>
       </c>
       <c r="C27" t="s">
-        <v>775</v>
+        <v>778</v>
       </c>
     </row>
   </sheetData>
@@ -6817,343 +6826,343 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>776</v>
+        <v>779</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>304</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>777</v>
+        <v>780</v>
       </c>
       <c r="B2" t="s">
         <v>309</v>
       </c>
       <c r="C2" t="s">
-        <v>715</v>
+        <v>718</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>778</v>
+        <v>781</v>
       </c>
       <c r="B3" t="s">
         <v>309</v>
       </c>
       <c r="C3" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>779</v>
+        <v>782</v>
       </c>
       <c r="B4" t="s">
         <v>315</v>
       </c>
       <c r="C4" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>780</v>
+        <v>783</v>
       </c>
       <c r="B5" t="s">
         <v>315</v>
       </c>
       <c r="C5" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>781</v>
+        <v>784</v>
       </c>
       <c r="B6" t="s">
         <v>322</v>
       </c>
       <c r="C6" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>782</v>
+        <v>785</v>
       </c>
       <c r="B7" t="s">
         <v>322</v>
       </c>
       <c r="C7" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>783</v>
+        <v>786</v>
       </c>
       <c r="B8" t="s">
         <v>329</v>
       </c>
       <c r="C8" t="s">
-        <v>727</v>
+        <v>730</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>784</v>
+        <v>787</v>
       </c>
       <c r="B9" t="s">
         <v>329</v>
       </c>
       <c r="C9" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>785</v>
+        <v>788</v>
       </c>
       <c r="B10" t="s">
         <v>336</v>
       </c>
       <c r="C10" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>786</v>
+        <v>789</v>
       </c>
       <c r="B11" t="s">
         <v>343</v>
       </c>
       <c r="C11" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>787</v>
+        <v>790</v>
       </c>
       <c r="B12" t="s">
         <v>350</v>
       </c>
       <c r="C12" t="s">
-        <v>733</v>
+        <v>736</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="B13" t="s">
         <v>350</v>
       </c>
       <c r="C13" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="B14" t="s">
         <v>350</v>
       </c>
       <c r="C14" t="s">
-        <v>737</v>
+        <v>740</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>790</v>
+        <v>793</v>
       </c>
       <c r="B15" t="s">
         <v>350</v>
       </c>
       <c r="C15" t="s">
-        <v>739</v>
+        <v>742</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>791</v>
+        <v>794</v>
       </c>
       <c r="B16" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C16" t="s">
-        <v>742</v>
+        <v>745</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>792</v>
+        <v>795</v>
       </c>
       <c r="B17" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C17" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>793</v>
+        <v>796</v>
       </c>
       <c r="B18" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C18" t="s">
-        <v>746</v>
+        <v>749</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>794</v>
+        <v>797</v>
       </c>
       <c r="B19" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C19" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>795</v>
+        <v>798</v>
       </c>
       <c r="B20" t="s">
         <v>360</v>
       </c>
       <c r="C20" t="s">
-        <v>750</v>
+        <v>753</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>796</v>
+        <v>799</v>
       </c>
       <c r="B21" t="s">
         <v>360</v>
       </c>
       <c r="C21" t="s">
-        <v>752</v>
+        <v>755</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="B22" t="s">
         <v>360</v>
       </c>
       <c r="C22" t="s">
-        <v>755</v>
+        <v>758</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>798</v>
+        <v>801</v>
       </c>
       <c r="B23" t="s">
         <v>360</v>
       </c>
       <c r="C23" t="s">
-        <v>757</v>
+        <v>760</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>799</v>
+        <v>802</v>
       </c>
       <c r="B24" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C24" t="s">
-        <v>759</v>
+        <v>762</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>800</v>
+        <v>803</v>
       </c>
       <c r="B25" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C25" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>801</v>
+        <v>804</v>
       </c>
       <c r="B26" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C26" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>802</v>
+        <v>805</v>
       </c>
       <c r="B27" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C27" t="s">
-        <v>764</v>
+        <v>767</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>803</v>
+        <v>806</v>
       </c>
       <c r="B28" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C28" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>804</v>
+        <v>807</v>
       </c>
       <c r="B29" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C29" t="s">
-        <v>769</v>
+        <v>772</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>805</v>
+        <v>808</v>
       </c>
       <c r="B30" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C30" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>806</v>
+        <v>809</v>
       </c>
       <c r="B31" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C31" t="s">
-        <v>774</v>
+        <v>777</v>
       </c>
     </row>
   </sheetData>
@@ -7178,42 +7187,42 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>807</v>
+        <v>810</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>808</v>
+        <v>811</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>809</v>
+        <v>812</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>810</v>
+        <v>813</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>811</v>
+        <v>814</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>812</v>
+        <v>815</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>813</v>
+        <v>816</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>814</v>
+        <v>817</v>
       </c>
       <c r="B2" t="s">
-        <v>815</v>
+        <v>818</v>
       </c>
       <c r="C2" t="s">
         <v>123</v>
       </c>
       <c r="D2" t="s">
-        <v>816</v>
+        <v>819</v>
       </c>
       <c r="E2" t="s">
-        <v>817</v>
+        <v>820</v>
       </c>
       <c r="F2" t="s">
         <v>303</v>
@@ -7224,19 +7233,19 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>818</v>
+        <v>821</v>
       </c>
       <c r="B3" t="s">
-        <v>819</v>
+        <v>822</v>
       </c>
       <c r="C3" t="s">
         <v>309</v>
       </c>
       <c r="D3" t="s">
-        <v>820</v>
+        <v>823</v>
       </c>
       <c r="E3" t="s">
-        <v>821</v>
+        <v>824</v>
       </c>
       <c r="F3" t="s">
         <v>303</v>
@@ -7247,10 +7256,10 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>825</v>
+      </c>
+      <c r="B4" t="s">
         <v>822</v>
-      </c>
-      <c r="B4" t="s">
-        <v>819</v>
       </c>
       <c r="C4" t="s">
         <v>315</v>
@@ -7259,7 +7268,7 @@
         <v>316</v>
       </c>
       <c r="E4" t="s">
-        <v>823</v>
+        <v>826</v>
       </c>
       <c r="F4" t="s">
         <v>303</v>
@@ -7270,10 +7279,10 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>824</v>
+        <v>827</v>
       </c>
       <c r="B5" t="s">
-        <v>819</v>
+        <v>822</v>
       </c>
       <c r="C5" t="s">
         <v>322</v>
@@ -7282,7 +7291,7 @@
         <v>323</v>
       </c>
       <c r="E5" t="s">
-        <v>825</v>
+        <v>828</v>
       </c>
       <c r="F5" t="s">
         <v>303</v>
@@ -7293,19 +7302,19 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>826</v>
+        <v>829</v>
       </c>
       <c r="B6" t="s">
-        <v>819</v>
+        <v>822</v>
       </c>
       <c r="C6" t="s">
         <v>329</v>
       </c>
       <c r="D6" t="s">
-        <v>827</v>
+        <v>830</v>
       </c>
       <c r="E6" t="s">
-        <v>828</v>
+        <v>831</v>
       </c>
       <c r="F6" t="s">
         <v>303</v>
@@ -7316,10 +7325,10 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>829</v>
+        <v>832</v>
       </c>
       <c r="B7" t="s">
-        <v>819</v>
+        <v>822</v>
       </c>
       <c r="C7" t="s">
         <v>336</v>
@@ -7328,7 +7337,7 @@
         <v>337</v>
       </c>
       <c r="E7" t="s">
-        <v>830</v>
+        <v>833</v>
       </c>
       <c r="F7" t="s">
         <v>303</v>
@@ -7339,10 +7348,10 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>831</v>
+        <v>834</v>
       </c>
       <c r="B8" t="s">
-        <v>819</v>
+        <v>822</v>
       </c>
       <c r="C8" t="s">
         <v>343</v>
@@ -7351,7 +7360,7 @@
         <v>344</v>
       </c>
       <c r="E8" t="s">
-        <v>832</v>
+        <v>835</v>
       </c>
       <c r="F8" t="s">
         <v>303</v>
@@ -7362,10 +7371,10 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>833</v>
+        <v>836</v>
       </c>
       <c r="B9" t="s">
-        <v>834</v>
+        <v>837</v>
       </c>
       <c r="C9" t="s">
         <v>38</v>
@@ -7374,7 +7383,7 @@
         <v>40</v>
       </c>
       <c r="E9" t="s">
-        <v>835</v>
+        <v>838</v>
       </c>
       <c r="F9" t="s">
         <v>303</v>
@@ -7401,30 +7410,30 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>836</v>
+        <v>839</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>837</v>
+        <v>840</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>838</v>
+        <v>841</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>839</v>
+        <v>842</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>840</v>
+        <v>843</v>
       </c>
       <c r="B2" t="s">
-        <v>841</v>
+        <v>844</v>
       </c>
       <c r="C2" t="s">
-        <v>842</v>
+        <v>845</v>
       </c>
       <c r="D2" t="b">
         <v>0</v>
@@ -7435,13 +7444,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>843</v>
+        <v>846</v>
       </c>
       <c r="B3" t="s">
-        <v>844</v>
+        <v>847</v>
       </c>
       <c r="C3" t="s">
-        <v>815</v>
+        <v>818</v>
       </c>
       <c r="D3" t="b">
         <v>0</v>
@@ -7452,13 +7461,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>845</v>
+        <v>848</v>
       </c>
       <c r="B4" t="s">
-        <v>846</v>
+        <v>849</v>
       </c>
       <c r="C4" t="s">
-        <v>847</v>
+        <v>850</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
@@ -7469,13 +7478,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>848</v>
+        <v>851</v>
       </c>
       <c r="B5" t="s">
-        <v>849</v>
+        <v>852</v>
       </c>
       <c r="C5" t="s">
-        <v>842</v>
+        <v>845</v>
       </c>
       <c r="D5" t="b">
         <v>0</v>
@@ -7483,13 +7492,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>850</v>
+        <v>853</v>
       </c>
       <c r="B6" t="s">
-        <v>851</v>
+        <v>854</v>
       </c>
       <c r="C6" t="s">
-        <v>852</v>
+        <v>855</v>
       </c>
       <c r="D6" t="b">
         <v>0</v>
@@ -7497,13 +7506,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>853</v>
+        <v>856</v>
       </c>
       <c r="B7" t="s">
-        <v>851</v>
+        <v>854</v>
       </c>
       <c r="C7" t="s">
-        <v>854</v>
+        <v>857</v>
       </c>
       <c r="D7" t="b">
         <v>0</v>
@@ -7529,16 +7538,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>855</v>
+        <v>858</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>856</v>
+        <v>859</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>857</v>
+        <v>860</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>858</v>
+        <v>861</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>66</v>
@@ -7546,16 +7555,16 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>859</v>
+        <v>862</v>
       </c>
       <c r="B2" t="s">
-        <v>860</v>
+        <v>863</v>
       </c>
       <c r="C2" t="s">
-        <v>861</v>
+        <v>864</v>
       </c>
       <c r="D2" t="s">
-        <v>862</v>
+        <v>865</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -7589,7 +7598,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>863</v>
+        <v>866</v>
       </c>
       <c r="B2" t="s">
         <v>154</v>
@@ -9780,24 +9789,27 @@
         <v>300</v>
       </c>
       <c r="G8" t="s">
+        <v>42</v>
+      </c>
+      <c r="H8" t="s">
         <v>354</v>
       </c>
       <c r="I8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>355</v>
+      </c>
+      <c r="B9" t="s">
         <v>356</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>357</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>358</v>
-      </c>
-      <c r="D9" t="s">
-        <v>359</v>
       </c>
       <c r="E9" t="s">
         <v>280</v>
@@ -9806,10 +9818,13 @@
         <v>300</v>
       </c>
       <c r="G9" t="s">
-        <v>354</v>
+        <v>42</v>
+      </c>
+      <c r="H9" t="s">
+        <v>359</v>
       </c>
       <c r="I9" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -9832,24 +9847,27 @@
         <v>300</v>
       </c>
       <c r="G10" t="s">
-        <v>354</v>
+        <v>42</v>
+      </c>
+      <c r="H10" t="s">
+        <v>364</v>
       </c>
       <c r="I10" t="s">
-        <v>355</v>
+        <v>364</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E11" t="s">
         <v>288</v>
@@ -9858,24 +9876,27 @@
         <v>300</v>
       </c>
       <c r="G11" t="s">
-        <v>354</v>
+        <v>42</v>
+      </c>
+      <c r="H11" t="s">
+        <v>369</v>
       </c>
       <c r="I11" t="s">
-        <v>355</v>
+        <v>369</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B12" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C12" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="D12" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E12" t="s">
         <v>292</v>
@@ -9884,10 +9905,13 @@
         <v>300</v>
       </c>
       <c r="G12" t="s">
-        <v>354</v>
+        <v>42</v>
+      </c>
+      <c r="H12" t="s">
+        <v>374</v>
       </c>
       <c r="I12" t="s">
-        <v>355</v>
+        <v>374</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Wrap up Phase 8: link new and old tools, update home text, categories and docs (T8.7)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/oewer_database.xlsx
+++ b/data/oewer_database.xlsx
@@ -417,7 +417,7 @@
     <t>finance-calculators</t>
   </si>
   <si>
-    <t>Calculators for loans, deposits, tax and everyday percentages.</t>
+    <t>Calculators for loans, savings, investments, tax, discounts and everyday percentages.</t>
   </si>
   <si>
     <t>TCAT0003</t>
@@ -441,7 +441,7 @@
     <t>utilities</t>
   </si>
   <si>
-    <t>Small everyday tools such as QR codes and word counting.</t>
+    <t>Everyday tools: age and date calculators, unit converter, password generator, QR codes and word count.</t>
   </si>
   <si>
     <t>tool_id</t>
@@ -878,7 +878,7 @@
     <t>TSET0023</t>
   </si>
   <si>
-    <t>["TOOL0005","TOOL0007"]</t>
+    <t>["TOOL0005","TOOL0015","TOOL0007"]</t>
   </si>
   <si>
     <t>TSET0024</t>
@@ -913,7 +913,7 @@
     <t>TSET0028</t>
   </si>
   <si>
-    <t>["TOOL0004","TOOL0007"]</t>
+    <t>["TOOL0004","TOOL0015","TOOL0013"]</t>
   </si>
   <si>
     <t>TSET0029</t>
@@ -946,7 +946,7 @@
     <t>TSET0033</t>
   </si>
   <si>
-    <t>["TOOL0007","TOOL0004"]</t>
+    <t>["TOOL0007","TOOL0016","TOOL0004"]</t>
   </si>
   <si>
     <t>TSET0034</t>
@@ -980,7 +980,7 @@
     <t>TSET0038</t>
   </si>
   <si>
-    <t>["TOOL0006","TOOL0004"]</t>
+    <t>["TOOL0006","TOOL0016","TOOL0019"]</t>
   </si>
   <si>
     <t>TSET0039</t>
@@ -1012,7 +1012,7 @@
     <t>TSET0043</t>
   </si>
   <si>
-    <t>["TOOL0010","TOOL0009"]</t>
+    <t>["TOOL0010","TOOL0009","TOOL0020"]</t>
   </si>
   <si>
     <t>TSET0044</t>
@@ -1047,7 +1047,7 @@
     <t>TSET0048</t>
   </si>
   <si>
-    <t>["TOOL0010","TOOL0008"]</t>
+    <t>["TOOL0010","TOOL0020","TOOL0008"]</t>
   </si>
   <si>
     <t>TSET0049</t>
@@ -1080,7 +1080,7 @@
     <t>TSET0053</t>
   </si>
   <si>
-    <t>["TOOL0008","TOOL0009"]</t>
+    <t>["TOOL0008","TOOL0009","TOOL0020"]</t>
   </si>
   <si>
     <t>TSET0054</t>
@@ -1112,7 +1112,7 @@
     <t>TSET0058</t>
   </si>
   <si>
-    <t>["TOOL0012","TOOL0004","TOOL0005"]</t>
+    <t>["TOOL0012","TOOL0013","TOOL0015"]</t>
   </si>
   <si>
     <t>TSET0059</t>
@@ -1147,7 +1147,7 @@
     <t>TSET0063</t>
   </si>
   <si>
-    <t>["TOOL0011","TOOL0004","TOOL0005"]</t>
+    <t>["TOOL0011","TOOL0013","TOOL0005"]</t>
   </si>
   <si>
     <t>TSET0064</t>
@@ -1183,7 +1183,7 @@
     <t>TSET0068</t>
   </si>
   <si>
-    <t>["TOOL0012","TOOL0005","TOOL0014"]</t>
+    <t>["TOOL0012","TOOL0014","TOOL0011"]</t>
   </si>
   <si>
     <t>TSET0069</t>
@@ -1288,7 +1288,7 @@
     <t>TSET0083</t>
   </si>
   <si>
-    <t>["TOOL0007","TOOL0006"]</t>
+    <t>["TOOL0007","TOOL0006","TOOL0014"]</t>
   </si>
   <si>
     <t>TSET0084</t>
@@ -15719,7 +15719,7 @@
         <v>42</v>
       </c>
       <c r="H12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12">
         <v>5</v>

</xml_diff>